<commit_message>
Fill 4 blank costs from SSB invoices (D5, Gentamicin, Tramadol, PCM 100ml)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -977,19 +977,17 @@
       <c r="D10" s="47" t="n">
         <v>40.12</v>
       </c>
-      <c r="E10" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="E10" s="47" t="n">
+        <v>17.14</v>
       </c>
       <c r="F10" s="48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>57.3%</t>
         </is>
       </c>
       <c r="G10" s="46" t="inlineStr">
         <is>
-          <t>Stock file</t>
+          <t>SSB S000197</t>
         </is>
       </c>
     </row>
@@ -1412,19 +1410,17 @@
       <c r="D25" s="47" t="n">
         <v>11.4</v>
       </c>
-      <c r="E25" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="E25" s="47" t="n">
+        <v>7.89</v>
       </c>
       <c r="F25" s="48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>30.8%</t>
         </is>
       </c>
       <c r="G25" s="46" t="inlineStr">
         <is>
-          <t>Stock file</t>
+          <t>SSB S000135</t>
         </is>
       </c>
     </row>
@@ -1617,19 +1613,17 @@
       <c r="D32" s="47" t="n">
         <v>12.56</v>
       </c>
-      <c r="E32" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="E32" s="47" t="n">
+        <v>4.76</v>
       </c>
       <c r="F32" s="48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>62.1%</t>
         </is>
       </c>
       <c r="G32" s="46" t="inlineStr">
         <is>
-          <t>Stock file</t>
+          <t>SSB S000135</t>
         </is>
       </c>
     </row>
@@ -1681,19 +1675,17 @@
       <c r="D34" s="47" t="n">
         <v>591.3</v>
       </c>
-      <c r="E34" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="E34" s="47" t="n">
+        <v>33.33</v>
       </c>
       <c r="F34" s="48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>94.4%</t>
         </is>
       </c>
       <c r="G34" s="46" t="inlineStr">
         <is>
-          <t>Stock file</t>
+          <t>SSB S000399</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fill NS 100ml cost from Vivek F-748 invoice
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -882,19 +882,17 @@
       <c r="D7" s="47" t="n">
         <v>21</v>
       </c>
-      <c r="E7" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="E7" s="47" t="n">
+        <v>13</v>
       </c>
       <c r="F7" s="48" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>38.1%</t>
         </is>
       </c>
       <c r="G7" s="46" t="inlineStr">
         <is>
-          <t>Stock file</t>
+          <t>Vivek F-748</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update rate card: fill cost for Disposable Gloves (SL68) from Neelgagan F1737
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -3105,10 +3105,8 @@
           <t>⚠ FILL</t>
         </is>
       </c>
-      <c r="E86" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="E86" s="47" t="n">
+        <v>2.43</v>
       </c>
       <c r="F86" s="48" t="inlineStr">
         <is>
@@ -3117,7 +3115,7 @@
       </c>
       <c r="G86" s="46" t="inlineStr">
         <is>
-          <t>⚠ MRP NOT FOUND</t>
+          <t>Neelgagan F1737</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update rate card with Perfia consumables list; rebuild all 12 patient bills
Rate card updates:
- SL64 OT Mop cost updated to ₹29.17/pc (from ₹55 estimate)
- SL68 Exam Gloves: MRP ₹4.63/pc, cost ₹2.80/pc (Perfia 400pcs/₹1120)
- SL84 Soft Roll cost updated to ₹80/pc
- Added SL100–SL118: Hip U Drape, Ioban, Suction Tube, Bardia 3-Way/2-Way catheters,
  IV Cannula 24G, Gamji Roll, C Colin Tubes, Nasal Cannula, 7 VP/NW suture types

Bills rebuild:
- Fixed bed/OT charge formulas (were B2*C{row}, now B{row}*C{row})
- 12 patient sheets Pt28–Pt39 with correct cross-sheet rate links
- RATES & SUMMARY sheet with global editable bed/OT rates

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G149"/>
+  <dimension ref="A1:G168"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="36" min="1" max="1"/>
@@ -2980,7 +2980,7 @@
         <v>165</v>
       </c>
       <c r="E82" s="53" t="n">
-        <v>55</v>
+        <v>29.17</v>
       </c>
       <c r="F82" s="57" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="G82" s="52" t="inlineStr">
         <is>
-          <t>CLD 3x</t>
+          <t>Perfia Consumables List</t>
         </is>
       </c>
     </row>
@@ -3100,13 +3100,11 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D86" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D86" s="47" t="n">
+        <v>4.63</v>
       </c>
       <c r="E86" s="47" t="n">
-        <v>2.43</v>
+        <v>2.8</v>
       </c>
       <c r="F86" s="48" t="inlineStr">
         <is>
@@ -3115,7 +3113,7 @@
       </c>
       <c r="G86" s="46" t="inlineStr">
         <is>
-          <t>Neelgagan F1737</t>
+          <t>Perfia 400pcs/₹1120; MRP 1850/400pcs</t>
         </is>
       </c>
     </row>
@@ -3613,10 +3611,8 @@
       <c r="D102" s="47" t="n">
         <v>117</v>
       </c>
-      <c r="E102" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="E102" s="47" t="n">
+        <v>80</v>
       </c>
       <c r="F102" s="48" t="inlineStr">
         <is>
@@ -3625,7 +3621,7 @@
       </c>
       <c r="G102" s="46" t="inlineStr">
         <is>
-          <t>Stock file</t>
+          <t>Perfia Consumables List</t>
         </is>
       </c>
     </row>
@@ -4171,695 +4167,429 @@
     </row>
     <row r="121"/>
     <row r="122" ht="13.5" customHeight="1" s="37">
-      <c r="A122" s="72" t="inlineStr">
+      <c r="A122" t="n">
+        <v>100</v>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Hip U Drape</t>
+        </is>
+      </c>
+      <c r="D122" t="n">
+        <v>1983</v>
+      </c>
+      <c r="E122" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹6750</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="12.75" customHeight="1" s="37">
+      <c r="A123" t="n">
+        <v>101</v>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Ioban Surgical Drape</t>
+        </is>
+      </c>
+      <c r="D123" t="n">
+        <v>1590</v>
+      </c>
+      <c r="E123" t="n">
+        <v>625</v>
+      </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 1box/₹7500 (12pc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="12.75" customHeight="1" s="37">
+      <c r="A124" t="n">
+        <v>102</v>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Suction Tube (VACCU)</t>
+        </is>
+      </c>
+      <c r="D124" t="n">
+        <v>543</v>
+      </c>
+      <c r="E124" t="n">
+        <v>50</v>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="12.75" customHeight="1" s="37">
+      <c r="A125" t="n">
+        <v>103</v>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Bardia 3-Way Catheter 22Fr</t>
+        </is>
+      </c>
+      <c r="D125" t="n">
+        <v>408</v>
+      </c>
+      <c r="E125" t="n">
+        <v>320</v>
+      </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹1600</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="12.75" customHeight="1" s="37">
+      <c r="A126" t="n">
+        <v>104</v>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Bardia 2-Way Catheter 14Fr</t>
+        </is>
+      </c>
+      <c r="D126" t="n">
+        <v>179</v>
+      </c>
+      <c r="E126" t="n">
+        <v>130</v>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹650</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="12.75" customHeight="1" s="37">
+      <c r="A127" t="n">
+        <v>105</v>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Bardia 2-Way Catheter 16Fr</t>
+        </is>
+      </c>
+      <c r="D127" t="n">
+        <v>191</v>
+      </c>
+      <c r="E127" t="n">
+        <v>130</v>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹650</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="12.75" customHeight="1" s="37">
+      <c r="A128" t="n">
+        <v>106</v>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Bardia 2-Way Catheter 18Fr</t>
+        </is>
+      </c>
+      <c r="D128" t="n">
+        <v>174</v>
+      </c>
+      <c r="E128" t="n">
+        <v>130</v>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹650</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="12.75" customHeight="1" s="37">
+      <c r="A129" t="n">
+        <v>107</v>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>IV Cannula 24G</t>
+        </is>
+      </c>
+      <c r="D129" t="n">
+        <v>693</v>
+      </c>
+      <c r="E129" t="n">
+        <v>350</v>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="12.75" customHeight="1" s="37">
+      <c r="A130" t="n">
+        <v>108</v>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Gamji Roll</t>
+        </is>
+      </c>
+      <c r="D130" t="n">
+        <v>250</v>
+      </c>
+      <c r="E130" t="n">
+        <v>80</v>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹400</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="12.75" customHeight="1" s="37">
+      <c r="A131" t="n">
+        <v>109</v>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>C Colin Tube Size 14</t>
+        </is>
+      </c>
+      <c r="D131" t="n">
+        <v>842</v>
+      </c>
+      <c r="E131" t="n">
+        <v>20</v>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹100</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="12.75" customHeight="1" s="37">
+      <c r="A132" t="n">
+        <v>110</v>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>C Colin Tube Size 16</t>
+        </is>
+      </c>
+      <c r="D132" t="n">
+        <v>842</v>
+      </c>
+      <c r="E132" t="n">
+        <v>20</v>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹100</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="12.75" customHeight="1" s="37">
+      <c r="A133" t="n">
+        <v>111</v>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Nasal Cannula</t>
+        </is>
+      </c>
+      <c r="D133" t="n">
+        <v>255</v>
+      </c>
+      <c r="E133" t="n">
+        <v>50</v>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 3pcs/₹150</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="12.75" customHeight="1" s="37">
+      <c r="A134" t="n">
+        <v>112</v>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Suture VP 2478 (per piece)</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>1223</v>
+      </c>
+      <c r="E134" t="n">
+        <v>672.5</v>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Perfia box/₹8070, 12pc; MRP ₹14676/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="12.75" customHeight="1" s="37">
+      <c r="A135" t="n">
+        <v>113</v>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Suture NW 2477 (per piece)</t>
+        </is>
+      </c>
+      <c r="D135" t="n">
+        <v>636</v>
+      </c>
+      <c r="E135" t="n">
+        <v>350</v>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Perfia box/₹4200, 12pc; MRP ₹7632/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="12.75" customHeight="1" s="37">
+      <c r="A136" t="n">
+        <v>114</v>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Suture VP 2548 (per piece)</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>1059</v>
+      </c>
+      <c r="E136" t="n">
+        <v>558.33</v>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>Perfia box/₹6700, 12pc; MRP ₹12710/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="12.75" customHeight="1" s="37">
+      <c r="A137" t="n">
+        <v>115</v>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Suture VP 2421 (per piece)</t>
+        </is>
+      </c>
+      <c r="D137" t="n">
+        <v>1171</v>
+      </c>
+      <c r="E137" t="n">
+        <v>644.17</v>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Perfia box/₹7730, 12pc; MRP ₹14052/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="12.75" customHeight="1" s="37">
+      <c r="A138" t="n">
+        <v>116</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Suture VP 2304 (per piece)</t>
+        </is>
+      </c>
+      <c r="D138" t="n">
+        <v>672</v>
+      </c>
+      <c r="E138" t="n">
+        <v>369.17</v>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Perfia box/₹4430, 12pc; MRP ₹8064/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="12.75" customHeight="1" s="37">
+      <c r="A139" t="n">
+        <v>117</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Suture VP 2518 (per piece)</t>
+        </is>
+      </c>
+      <c r="D139" t="n">
+        <v>871</v>
+      </c>
+      <c r="E139" t="n">
+        <v>479.17</v>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>Perfia box/₹5750, 12pc; MRP ₹10452/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="12.75" customHeight="1" s="37">
+      <c r="A140" t="n">
+        <v>118</v>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Suture NW 2317 (per piece)</t>
+        </is>
+      </c>
+      <c r="D140" t="n">
+        <v>900</v>
+      </c>
+      <c r="E140" t="n">
+        <v>495</v>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Perfia box/₹5940, 12pc; MRP ₹10800/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="12.75" customHeight="1" s="37">
+      <c r="A141" s="72" t="inlineStr">
         <is>
           <t>🔴 ITEMS MISSING MRP — Collect from vendor and update above</t>
         </is>
       </c>
-      <c r="B122" s="42" t="n"/>
-      <c r="C122" s="42" t="n"/>
-      <c r="D122" s="42" t="n"/>
-      <c r="E122" s="42" t="n"/>
-      <c r="F122" s="42" t="n"/>
-      <c r="G122" s="42" t="n"/>
-    </row>
-    <row r="123" ht="12.75" customHeight="1" s="37">
-      <c r="A123" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="B123" s="73" t="inlineStr">
-        <is>
-          <t>NS 100ml — Normal Saline 100ml</t>
-        </is>
-      </c>
-      <c r="C123" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D123" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E123" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F123" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G123" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="124" ht="12.75" customHeight="1" s="37">
-      <c r="A124" s="48" t="n">
-        <v>2</v>
-      </c>
-      <c r="B124" s="73" t="inlineStr">
-        <is>
-          <t>D5 500ml — Dextrose 5%</t>
-        </is>
-      </c>
-      <c r="C124" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D124" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E124" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F124" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G124" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="125" ht="12.75" customHeight="1" s="37">
-      <c r="A125" s="48" t="n">
-        <v>3</v>
-      </c>
-      <c r="B125" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
-        </is>
-      </c>
-      <c r="C125" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Anaesthesia</t>
-        </is>
-      </c>
-      <c r="D125" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E125" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F125" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G125" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="126" ht="12.75" customHeight="1" s="37">
-      <c r="A126" s="48" t="n">
-        <v>4</v>
-      </c>
-      <c r="B126" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Gentamicin</t>
-        </is>
-      </c>
-      <c r="C126" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D126" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E126" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F126" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G126" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="127" ht="12.75" customHeight="1" s="37">
-      <c r="A127" s="48" t="n">
-        <v>5</v>
-      </c>
-      <c r="B127" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Tramadol 50mg</t>
-        </is>
-      </c>
-      <c r="C127" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Analgesic</t>
-        </is>
-      </c>
-      <c r="D127" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E127" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F127" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G127" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="128" ht="12.75" customHeight="1" s="37">
-      <c r="A128" s="48" t="n">
-        <v>6</v>
-      </c>
-      <c r="B128" s="73" t="inlineStr">
-        <is>
-          <t>Inj. PCM 100ml (Paracetamol IV)</t>
-        </is>
-      </c>
-      <c r="C128" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Analgesic</t>
-        </is>
-      </c>
-      <c r="D128" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E128" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F128" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G128" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="129" ht="12.75" customHeight="1" s="37">
-      <c r="A129" s="48" t="n">
-        <v>7</v>
-      </c>
-      <c r="B129" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Carboprost (Hemabate)</t>
-        </is>
-      </c>
-      <c r="C129" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Oxytocic</t>
-        </is>
-      </c>
-      <c r="D129" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E129" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F129" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G129" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="130" ht="12.75" customHeight="1" s="37">
-      <c r="A130" s="48" t="n">
-        <v>8</v>
-      </c>
-      <c r="B130" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Adrenaline</t>
-        </is>
-      </c>
-      <c r="C130" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Emergency</t>
-        </is>
-      </c>
-      <c r="D130" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E130" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F130" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G130" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="131" ht="12.75" customHeight="1" s="37">
-      <c r="A131" s="48" t="n">
-        <v>9</v>
-      </c>
-      <c r="B131" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Cetil (Cefuroxime Axetil)</t>
-        </is>
-      </c>
-      <c r="C131" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D131" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E131" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F131" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G131" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="132" ht="12.75" customHeight="1" s="37">
-      <c r="A132" s="48" t="n">
-        <v>10</v>
-      </c>
-      <c r="B132" s="73" t="inlineStr">
-        <is>
-          <t>Needles 26G (Injection)</t>
-        </is>
-      </c>
-      <c r="C132" s="46" t="inlineStr">
-        <is>
-          <t>Consumable</t>
-        </is>
-      </c>
-      <c r="D132" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E132" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F132" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G132" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="12.75" customHeight="1" s="37">
-      <c r="A133" s="48" t="n">
-        <v>11</v>
-      </c>
-      <c r="B133" s="73" t="inlineStr">
-        <is>
-          <t>Disposable Gloves (Exam)</t>
-        </is>
-      </c>
-      <c r="C133" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D133" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E133" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F133" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G133" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="134" ht="12.75" customHeight="1" s="37">
-      <c r="A134" s="48" t="n">
-        <v>12</v>
-      </c>
-      <c r="B134" s="73" t="inlineStr">
-        <is>
-          <t>Betadine Ointment 40g</t>
-        </is>
-      </c>
-      <c r="C134" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D134" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E134" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F134" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G134" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="135" ht="12.75" customHeight="1" s="37">
-      <c r="A135" s="48" t="n">
-        <v>13</v>
-      </c>
-      <c r="B135" s="73" t="inlineStr">
-        <is>
-          <t>Surgical Blade No. 10</t>
-        </is>
-      </c>
-      <c r="C135" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D135" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E135" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F135" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G135" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="136" ht="12.75" customHeight="1" s="37">
-      <c r="A136" s="48" t="n">
-        <v>14</v>
-      </c>
-      <c r="B136" s="73" t="inlineStr">
-        <is>
-          <t>Surgical Blade No. 20</t>
-        </is>
-      </c>
-      <c r="C136" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D136" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E136" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F136" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G136" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="137" ht="12.75" customHeight="1" s="37">
-      <c r="A137" s="48" t="n">
-        <v>15</v>
-      </c>
-      <c r="B137" s="73" t="inlineStr">
-        <is>
-          <t>Plain Sheet (OT Draping)</t>
-        </is>
-      </c>
-      <c r="C137" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D137" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E137" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F137" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G137" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="12.75" customHeight="1" s="37">
-      <c r="A138" s="48" t="n">
-        <v>16</v>
-      </c>
-      <c r="B138" s="73" t="inlineStr">
-        <is>
-          <t>Soft Roll (OT Padding)</t>
-        </is>
-      </c>
-      <c r="C138" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D138" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E138" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F138" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G138" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="139" ht="12.75" customHeight="1" s="37">
-      <c r="A139" s="48" t="n">
-        <v>17</v>
-      </c>
-      <c r="B139" s="73" t="inlineStr">
-        <is>
-          <t>Gypsona POP Bandage 40G</t>
-        </is>
-      </c>
-      <c r="C139" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D139" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E139" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F139" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G139" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="140" ht="12.75" customHeight="1" s="37">
-      <c r="A140" s="48" t="n">
-        <v>18</v>
-      </c>
-      <c r="B140" s="73" t="inlineStr">
-        <is>
-          <t>Cap + Mask (Disposable Set)</t>
-        </is>
-      </c>
-      <c r="C140" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D140" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E140" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F140" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G140" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="141" ht="12.75" customHeight="1" s="37">
-      <c r="A141" s="48" t="n">
-        <v>19</v>
-      </c>
-      <c r="B141" s="73" t="inlineStr">
-        <is>
-          <t>Glucostrip (Blood Glucose)</t>
-        </is>
-      </c>
-      <c r="C141" s="46" t="inlineStr">
-        <is>
-          <t>Investigation</t>
-        </is>
-      </c>
-      <c r="D141" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E141" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F141" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G141" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
+      <c r="B141" s="42" t="n"/>
+      <c r="C141" s="42" t="n"/>
+      <c r="D141" s="42" t="n"/>
+      <c r="E141" s="42" t="n"/>
+      <c r="F141" s="42" t="n"/>
+      <c r="G141" s="42" t="n"/>
     </row>
     <row r="142" ht="12.75" customHeight="1" s="37">
       <c r="A142" s="48" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B142" s="73" t="inlineStr">
         <is>
-          <t>Lancet Needle</t>
+          <t>NS 100ml — Normal Saline 100ml</t>
         </is>
       </c>
       <c r="C142" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>IV Fluid</t>
         </is>
       </c>
       <c r="D142" s="47" t="inlineStr">
@@ -4885,16 +4615,16 @@
     </row>
     <row r="143" ht="12.75" customHeight="1" s="37">
       <c r="A143" s="48" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="B143" s="73" t="inlineStr">
         <is>
-          <t>Red Top Tube (Blood Vial)</t>
+          <t>D5 500ml — Dextrose 5%</t>
         </is>
       </c>
       <c r="C143" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>IV Fluid</t>
         </is>
       </c>
       <c r="D143" s="47" t="inlineStr">
@@ -4920,16 +4650,16 @@
     </row>
     <row r="144" ht="12.75" customHeight="1" s="37">
       <c r="A144" s="48" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="B144" s="73" t="inlineStr">
         <is>
-          <t>CBC Vial Yellow + Red Top</t>
+          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
         </is>
       </c>
       <c r="C144" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>Injection — Anaesthesia</t>
         </is>
       </c>
       <c r="D144" s="47" t="inlineStr">
@@ -4955,16 +4685,16 @@
     </row>
     <row r="145" ht="12.75" customHeight="1" s="37">
       <c r="A145" s="48" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="B145" s="73" t="inlineStr">
         <is>
-          <t>O2 / Oxygen (per use)</t>
+          <t>Inj. Gentamicin</t>
         </is>
       </c>
       <c r="C145" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D145" s="47" t="inlineStr">
@@ -4990,16 +4720,16 @@
     </row>
     <row r="146" ht="12.75" customHeight="1" s="37">
       <c r="A146" s="48" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="B146" s="73" t="inlineStr">
         <is>
-          <t>Pulse Oximeter (per use)</t>
+          <t>Inj. Tramadol 50mg</t>
         </is>
       </c>
       <c r="C146" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Injection — Analgesic</t>
         </is>
       </c>
       <c r="D146" s="47" t="inlineStr">
@@ -5025,16 +4755,16 @@
     </row>
     <row r="147" ht="12.75" customHeight="1" s="37">
       <c r="A147" s="48" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="B147" s="73" t="inlineStr">
         <is>
-          <t>Cardiac Monitor (per use)</t>
+          <t>Inj. PCM 100ml (Paracetamol IV)</t>
         </is>
       </c>
       <c r="C147" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Injection — Analgesic</t>
         </is>
       </c>
       <c r="D147" s="47" t="inlineStr">
@@ -5060,16 +4790,16 @@
     </row>
     <row r="148" ht="12.75" customHeight="1" s="37">
       <c r="A148" s="48" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="B148" s="73" t="inlineStr">
         <is>
-          <t>C-arm (per use)</t>
+          <t>Inj. Carboprost (Hemabate)</t>
         </is>
       </c>
       <c r="C148" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Injection — Oxytocic</t>
         </is>
       </c>
       <c r="D148" s="47" t="inlineStr">
@@ -5095,34 +4825,699 @@
     </row>
     <row r="149" ht="12.75" customHeight="1" s="37">
       <c r="A149" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="B149" s="73" t="inlineStr">
+        <is>
+          <t>Inj. Adrenaline</t>
+        </is>
+      </c>
+      <c r="C149" s="46" t="inlineStr">
+        <is>
+          <t>Injection — Emergency</t>
+        </is>
+      </c>
+      <c r="D149" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E149" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F149" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G149" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="B150" s="73" t="inlineStr">
+        <is>
+          <t>Inj. Cetil (Cefuroxime Axetil)</t>
+        </is>
+      </c>
+      <c r="C150" s="46" t="inlineStr">
+        <is>
+          <t>Injection — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D150" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E150" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F150" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G150" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="B151" s="73" t="inlineStr">
+        <is>
+          <t>Needles 26G (Injection)</t>
+        </is>
+      </c>
+      <c r="C151" s="46" t="inlineStr">
+        <is>
+          <t>Consumable</t>
+        </is>
+      </c>
+      <c r="D151" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E151" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F151" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G151" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="48" t="n">
+        <v>11</v>
+      </c>
+      <c r="B152" s="73" t="inlineStr">
+        <is>
+          <t>Disposable Gloves (Exam)</t>
+        </is>
+      </c>
+      <c r="C152" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D152" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E152" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F152" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G152" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="B153" s="73" t="inlineStr">
+        <is>
+          <t>Betadine Ointment 40g</t>
+        </is>
+      </c>
+      <c r="C153" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D153" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E153" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F153" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G153" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="48" t="n">
+        <v>13</v>
+      </c>
+      <c r="B154" s="73" t="inlineStr">
+        <is>
+          <t>Surgical Blade No. 10</t>
+        </is>
+      </c>
+      <c r="C154" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D154" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E154" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F154" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G154" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="48" t="n">
+        <v>14</v>
+      </c>
+      <c r="B155" s="73" t="inlineStr">
+        <is>
+          <t>Surgical Blade No. 20</t>
+        </is>
+      </c>
+      <c r="C155" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D155" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E155" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F155" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G155" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="48" t="n">
+        <v>15</v>
+      </c>
+      <c r="B156" s="73" t="inlineStr">
+        <is>
+          <t>Plain Sheet (OT Draping)</t>
+        </is>
+      </c>
+      <c r="C156" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D156" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E156" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F156" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G156" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="48" t="n">
+        <v>16</v>
+      </c>
+      <c r="B157" s="73" t="inlineStr">
+        <is>
+          <t>Soft Roll (OT Padding)</t>
+        </is>
+      </c>
+      <c r="C157" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D157" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E157" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F157" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G157" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="48" t="n">
+        <v>17</v>
+      </c>
+      <c r="B158" s="73" t="inlineStr">
+        <is>
+          <t>Gypsona POP Bandage 40G</t>
+        </is>
+      </c>
+      <c r="C158" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D158" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E158" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F158" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G158" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="48" t="n">
+        <v>18</v>
+      </c>
+      <c r="B159" s="73" t="inlineStr">
+        <is>
+          <t>Cap + Mask (Disposable Set)</t>
+        </is>
+      </c>
+      <c r="C159" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D159" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E159" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F159" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G159" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="48" t="n">
+        <v>19</v>
+      </c>
+      <c r="B160" s="73" t="inlineStr">
+        <is>
+          <t>Glucostrip (Blood Glucose)</t>
+        </is>
+      </c>
+      <c r="C160" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D160" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E160" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F160" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G160" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="B161" s="73" t="inlineStr">
+        <is>
+          <t>Lancet Needle</t>
+        </is>
+      </c>
+      <c r="C161" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D161" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E161" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F161" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G161" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="48" t="n">
+        <v>21</v>
+      </c>
+      <c r="B162" s="73" t="inlineStr">
+        <is>
+          <t>Red Top Tube (Blood Vial)</t>
+        </is>
+      </c>
+      <c r="C162" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D162" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E162" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F162" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G162" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="48" t="n">
+        <v>22</v>
+      </c>
+      <c r="B163" s="73" t="inlineStr">
+        <is>
+          <t>CBC Vial Yellow + Red Top</t>
+        </is>
+      </c>
+      <c r="C163" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D163" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E163" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F163" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G163" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="48" t="n">
+        <v>23</v>
+      </c>
+      <c r="B164" s="73" t="inlineStr">
+        <is>
+          <t>O2 / Oxygen (per use)</t>
+        </is>
+      </c>
+      <c r="C164" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D164" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E164" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F164" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G164" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="48" t="n">
+        <v>24</v>
+      </c>
+      <c r="B165" s="73" t="inlineStr">
+        <is>
+          <t>Pulse Oximeter (per use)</t>
+        </is>
+      </c>
+      <c r="C165" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D165" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E165" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F165" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G165" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="48" t="n">
+        <v>25</v>
+      </c>
+      <c r="B166" s="73" t="inlineStr">
+        <is>
+          <t>Cardiac Monitor (per use)</t>
+        </is>
+      </c>
+      <c r="C166" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D166" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E166" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F166" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G166" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="48" t="n">
+        <v>26</v>
+      </c>
+      <c r="B167" s="73" t="inlineStr">
+        <is>
+          <t>C-arm (per use)</t>
+        </is>
+      </c>
+      <c r="C167" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D167" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E167" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F167" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G167" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="48" t="n">
         <v>27</v>
       </c>
-      <c r="B149" s="73" t="inlineStr">
+      <c r="B168" s="73" t="inlineStr">
         <is>
           <t>Volu-P / TiCUP</t>
         </is>
       </c>
-      <c r="C149" s="46" t="inlineStr">
+      <c r="C168" s="46" t="inlineStr">
         <is>
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D149" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E149" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F149" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G149" s="47" t="inlineStr">
+      <c r="D168" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E168" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F168" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G168" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL IN</t>
         </is>

</xml_diff>

<commit_message>
Update rate card: BP Pharma, CLD Surgical, MP Enterprise invoice costs; new SL119-127
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -729,7 +729,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G196"/>
+  <dimension ref="A1:G215"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="36" min="1" max="1"/>
@@ -4745,1094 +4745,828 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" t="n">
+      <c r="A150" s="36" t="n">
         <v>100</v>
       </c>
-      <c r="B150" t="inlineStr">
+      <c r="B150" s="36" t="inlineStr">
         <is>
           <t>Hip U Drape</t>
         </is>
       </c>
-      <c r="D150" t="n">
+      <c r="D150" s="36" t="n">
         <v>1983</v>
       </c>
-      <c r="E150" t="n">
+      <c r="E150" s="36" t="n">
         <v>1350</v>
       </c>
-      <c r="G150" t="inlineStr">
+      <c r="G150" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹6750</t>
         </is>
       </c>
     </row>
     <row r="151">
-      <c r="A151" t="n">
+      <c r="A151" s="36" t="n">
         <v>101</v>
       </c>
-      <c r="B151" t="inlineStr">
+      <c r="B151" s="36" t="inlineStr">
         <is>
           <t>Ioban Surgical Drape</t>
         </is>
       </c>
-      <c r="D151" t="n">
+      <c r="D151" s="36" t="n">
         <v>1590</v>
       </c>
-      <c r="E151" t="n">
+      <c r="E151" s="36" t="n">
         <v>625</v>
       </c>
-      <c r="G151" t="inlineStr">
+      <c r="G151" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 1box/₹7500 (12pc)</t>
         </is>
       </c>
     </row>
     <row r="152">
-      <c r="A152" t="n">
+      <c r="A152" s="36" t="n">
         <v>102</v>
       </c>
-      <c r="B152" t="inlineStr">
+      <c r="B152" s="36" t="inlineStr">
         <is>
           <t>Suction Tube (VACCU)</t>
         </is>
       </c>
-      <c r="D152" t="n">
+      <c r="D152" s="36" t="n">
         <v>543</v>
       </c>
-      <c r="E152" t="n">
+      <c r="E152" s="36" t="n">
         <v>50</v>
       </c>
-      <c r="G152" t="inlineStr">
+      <c r="G152" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List</t>
         </is>
       </c>
     </row>
     <row r="153">
-      <c r="A153" t="n">
+      <c r="A153" s="36" t="n">
         <v>103</v>
       </c>
-      <c r="B153" t="inlineStr">
+      <c r="B153" s="36" t="inlineStr">
         <is>
           <t>Bardia 3-Way Catheter 22Fr</t>
         </is>
       </c>
-      <c r="D153" t="n">
+      <c r="D153" s="36" t="n">
         <v>408</v>
       </c>
-      <c r="E153" t="n">
+      <c r="E153" s="36" t="n">
         <v>320</v>
       </c>
-      <c r="G153" t="inlineStr">
+      <c r="G153" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹1600</t>
         </is>
       </c>
     </row>
     <row r="154">
-      <c r="A154" t="n">
+      <c r="A154" s="36" t="n">
         <v>104</v>
       </c>
-      <c r="B154" t="inlineStr">
+      <c r="B154" s="36" t="inlineStr">
         <is>
           <t>Bardia 2-Way Catheter 14Fr</t>
         </is>
       </c>
-      <c r="D154" t="n">
+      <c r="D154" s="36" t="n">
         <v>179</v>
       </c>
-      <c r="E154" t="n">
+      <c r="E154" s="36" t="n">
         <v>130</v>
       </c>
-      <c r="G154" t="inlineStr">
+      <c r="G154" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹650</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" t="n">
+      <c r="A155" s="36" t="n">
         <v>105</v>
       </c>
-      <c r="B155" t="inlineStr">
+      <c r="B155" s="36" t="inlineStr">
         <is>
           <t>Bardia 2-Way Catheter 16Fr</t>
         </is>
       </c>
-      <c r="D155" t="n">
+      <c r="D155" s="36" t="n">
         <v>191</v>
       </c>
-      <c r="E155" t="n">
+      <c r="E155" s="36" t="n">
         <v>130</v>
       </c>
-      <c r="G155" t="inlineStr">
+      <c r="G155" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹650</t>
         </is>
       </c>
     </row>
     <row r="156">
-      <c r="A156" t="n">
+      <c r="A156" s="36" t="n">
         <v>106</v>
       </c>
-      <c r="B156" t="inlineStr">
+      <c r="B156" s="36" t="inlineStr">
         <is>
           <t>Bardia 2-Way Catheter 18Fr</t>
         </is>
       </c>
-      <c r="D156" t="n">
+      <c r="D156" s="36" t="n">
         <v>174</v>
       </c>
-      <c r="E156" t="n">
+      <c r="E156" s="36" t="n">
         <v>130</v>
       </c>
-      <c r="G156" t="inlineStr">
+      <c r="G156" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹650</t>
         </is>
       </c>
     </row>
     <row r="157">
-      <c r="A157" t="n">
+      <c r="A157" s="36" t="n">
         <v>107</v>
       </c>
-      <c r="B157" t="inlineStr">
+      <c r="B157" s="36" t="inlineStr">
         <is>
           <t>IV Cannula 24G</t>
         </is>
       </c>
-      <c r="D157" t="n">
+      <c r="D157" s="36" t="n">
         <v>693</v>
       </c>
-      <c r="E157" t="n">
+      <c r="E157" s="36" t="n">
         <v>350</v>
       </c>
-      <c r="G157" t="inlineStr">
+      <c r="G157" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List</t>
         </is>
       </c>
     </row>
     <row r="158">
-      <c r="A158" t="n">
+      <c r="A158" s="36" t="n">
         <v>108</v>
       </c>
-      <c r="B158" t="inlineStr">
+      <c r="B158" s="36" t="inlineStr">
         <is>
           <t>Gamji Roll</t>
         </is>
       </c>
-      <c r="D158" t="n">
+      <c r="D158" s="36" t="n">
         <v>250</v>
       </c>
-      <c r="E158" t="n">
+      <c r="E158" s="36" t="n">
         <v>80</v>
       </c>
-      <c r="G158" t="inlineStr">
+      <c r="G158" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹400</t>
         </is>
       </c>
     </row>
     <row r="159">
-      <c r="A159" t="n">
+      <c r="A159" s="36" t="n">
         <v>109</v>
       </c>
-      <c r="B159" t="inlineStr">
+      <c r="B159" s="36" t="inlineStr">
         <is>
           <t>C Colin Tube Size 14</t>
         </is>
       </c>
-      <c r="D159" t="n">
+      <c r="D159" s="36" t="n">
         <v>842</v>
       </c>
-      <c r="E159" t="n">
+      <c r="E159" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="G159" t="inlineStr">
+      <c r="G159" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹100</t>
         </is>
       </c>
     </row>
     <row r="160">
-      <c r="A160" t="n">
+      <c r="A160" s="36" t="n">
         <v>110</v>
       </c>
-      <c r="B160" t="inlineStr">
+      <c r="B160" s="36" t="inlineStr">
         <is>
           <t>C Colin Tube Size 16</t>
         </is>
       </c>
-      <c r="D160" t="n">
+      <c r="D160" s="36" t="n">
         <v>842</v>
       </c>
-      <c r="E160" t="n">
+      <c r="E160" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="G160" t="inlineStr">
+      <c r="G160" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹100</t>
         </is>
       </c>
     </row>
     <row r="161">
-      <c r="A161" t="n">
+      <c r="A161" s="36" t="n">
         <v>111</v>
       </c>
-      <c r="B161" t="inlineStr">
+      <c r="B161" s="36" t="inlineStr">
         <is>
           <t>Nasal Cannula</t>
         </is>
       </c>
-      <c r="D161" t="n">
+      <c r="D161" s="36" t="n">
         <v>255</v>
       </c>
-      <c r="E161" t="n">
+      <c r="E161" s="36" t="n">
         <v>50</v>
       </c>
-      <c r="G161" t="inlineStr">
+      <c r="G161" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 3pcs/₹150</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" t="n">
+      <c r="A162" s="36" t="n">
         <v>112</v>
       </c>
-      <c r="B162" t="inlineStr">
+      <c r="B162" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2478 (per piece)</t>
         </is>
       </c>
-      <c r="D162" t="n">
+      <c r="D162" s="36" t="n">
         <v>1223</v>
       </c>
-      <c r="E162" t="n">
+      <c r="E162" s="36" t="n">
         <v>672.5</v>
       </c>
-      <c r="G162" t="inlineStr">
+      <c r="G162" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹8070, 12pc; MRP ₹14676/box</t>
         </is>
       </c>
     </row>
     <row r="163">
-      <c r="A163" t="n">
+      <c r="A163" s="36" t="n">
         <v>113</v>
       </c>
-      <c r="B163" t="inlineStr">
+      <c r="B163" s="36" t="inlineStr">
         <is>
           <t>Suture NW 2477 (per piece)</t>
         </is>
       </c>
-      <c r="D163" t="n">
+      <c r="D163" s="36" t="n">
         <v>636</v>
       </c>
-      <c r="E163" t="n">
+      <c r="E163" s="36" t="n">
         <v>350</v>
       </c>
-      <c r="G163" t="inlineStr">
+      <c r="G163" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹4200, 12pc; MRP ₹7632/box</t>
         </is>
       </c>
     </row>
     <row r="164">
-      <c r="A164" t="n">
+      <c r="A164" s="36" t="n">
         <v>114</v>
       </c>
-      <c r="B164" t="inlineStr">
+      <c r="B164" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2548 (per piece)</t>
         </is>
       </c>
-      <c r="D164" t="n">
+      <c r="D164" s="36" t="n">
         <v>1059</v>
       </c>
-      <c r="E164" t="n">
+      <c r="E164" s="36" t="n">
         <v>558.33</v>
       </c>
-      <c r="G164" t="inlineStr">
+      <c r="G164" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹6700, 12pc; MRP ₹12710/box</t>
         </is>
       </c>
     </row>
     <row r="165">
-      <c r="A165" t="n">
+      <c r="A165" s="36" t="n">
         <v>115</v>
       </c>
-      <c r="B165" t="inlineStr">
+      <c r="B165" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2421 (per piece)</t>
         </is>
       </c>
-      <c r="D165" t="n">
+      <c r="D165" s="36" t="n">
         <v>1171</v>
       </c>
-      <c r="E165" t="n">
+      <c r="E165" s="36" t="n">
         <v>644.17</v>
       </c>
-      <c r="G165" t="inlineStr">
+      <c r="G165" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹7730, 12pc; MRP ₹14052/box</t>
         </is>
       </c>
     </row>
     <row r="166">
-      <c r="A166" t="n">
+      <c r="A166" s="36" t="n">
         <v>116</v>
       </c>
-      <c r="B166" t="inlineStr">
+      <c r="B166" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2304 (per piece)</t>
         </is>
       </c>
-      <c r="D166" t="n">
+      <c r="D166" s="36" t="n">
         <v>672</v>
       </c>
-      <c r="E166" t="n">
+      <c r="E166" s="36" t="n">
         <v>369.17</v>
       </c>
-      <c r="G166" t="inlineStr">
+      <c r="G166" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹4430, 12pc; MRP ₹8064/box</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" t="n">
+      <c r="A167" s="36" t="n">
         <v>117</v>
       </c>
-      <c r="B167" t="inlineStr">
+      <c r="B167" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2518 (per piece)</t>
         </is>
       </c>
-      <c r="D167" t="n">
+      <c r="D167" s="36" t="n">
         <v>871</v>
       </c>
-      <c r="E167" t="n">
+      <c r="E167" s="36" t="n">
         <v>479.17</v>
       </c>
-      <c r="G167" t="inlineStr">
+      <c r="G167" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹5750, 12pc; MRP ₹10452/box</t>
         </is>
       </c>
     </row>
     <row r="168">
-      <c r="A168" t="n">
+      <c r="A168" s="36" t="n">
         <v>118</v>
       </c>
-      <c r="B168" t="inlineStr">
+      <c r="B168" s="36" t="inlineStr">
         <is>
           <t>Suture NW 2317 (per piece)</t>
         </is>
       </c>
-      <c r="D168" t="n">
+      <c r="D168" s="36" t="n">
         <v>900</v>
       </c>
-      <c r="E168" t="n">
+      <c r="E168" s="36" t="n">
         <v>495</v>
       </c>
-      <c r="G168" t="inlineStr">
+      <c r="G168" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹5940, 12pc; MRP ₹10800/box</t>
         </is>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="72" t="inlineStr">
+      <c r="A169" t="n">
+        <v>100</v>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Hip U Drape</t>
+        </is>
+      </c>
+      <c r="D169" t="n">
+        <v>1983</v>
+      </c>
+      <c r="E169" t="n">
+        <v>1350</v>
+      </c>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹6750</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="n">
+        <v>101</v>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Ioban Surgical Drape</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>1590</v>
+      </c>
+      <c r="E170" t="n">
+        <v>625</v>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 1box/₹7500 (12pc)</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="n">
+        <v>102</v>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Suction Tube (VACCU)</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>543</v>
+      </c>
+      <c r="E171" t="n">
+        <v>50</v>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="n">
+        <v>103</v>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Bardia 3-Way Catheter 22Fr</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>408</v>
+      </c>
+      <c r="E172" t="n">
+        <v>320</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹1600</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="n">
+        <v>104</v>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Bardia 2-Way Catheter 14Fr</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>179</v>
+      </c>
+      <c r="E173" t="n">
+        <v>130</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹650</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="n">
+        <v>105</v>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Bardia 2-Way Catheter 16Fr</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>191</v>
+      </c>
+      <c r="E174" t="n">
+        <v>130</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹650</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="n">
+        <v>106</v>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Bardia 2-Way Catheter 18Fr</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>174</v>
+      </c>
+      <c r="E175" t="n">
+        <v>130</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹650</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="n">
+        <v>107</v>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>IV Cannula 24G</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>693</v>
+      </c>
+      <c r="E176" t="n">
+        <v>350</v>
+      </c>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="n">
+        <v>108</v>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Gamji Roll</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>250</v>
+      </c>
+      <c r="E177" t="n">
+        <v>80</v>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹400</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="n">
+        <v>109</v>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>C Colin Tube Size 14</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>842</v>
+      </c>
+      <c r="E178" t="n">
+        <v>20</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹100</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="n">
+        <v>110</v>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>C Colin Tube Size 16</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>842</v>
+      </c>
+      <c r="E179" t="n">
+        <v>20</v>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 5pcs/₹100</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="n">
+        <v>111</v>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Nasal Cannula</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>255</v>
+      </c>
+      <c r="E180" t="n">
+        <v>50</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>Perfia Consumables List 3pcs/₹150</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="n">
+        <v>112</v>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Suture VP 2478 (per piece)</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>1223</v>
+      </c>
+      <c r="E181" t="n">
+        <v>672.5</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>Perfia box/₹8070, 12pc; MRP ₹14676/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="n">
+        <v>113</v>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Suture NW 2477 (per piece)</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>636</v>
+      </c>
+      <c r="E182" t="n">
+        <v>350</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>Perfia box/₹4200, 12pc; MRP ₹7632/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="n">
+        <v>114</v>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Suture VP 2548 (per piece)</t>
+        </is>
+      </c>
+      <c r="D183" t="n">
+        <v>1059</v>
+      </c>
+      <c r="E183" t="n">
+        <v>558.33</v>
+      </c>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>Perfia box/₹6700, 12pc; MRP ₹12710/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="n">
+        <v>115</v>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Suture VP 2421 (per piece)</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>1171</v>
+      </c>
+      <c r="E184" t="n">
+        <v>644.17</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>Perfia box/₹7730, 12pc; MRP ₹14052/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="n">
+        <v>116</v>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Suture VP 2304 (per piece)</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>672</v>
+      </c>
+      <c r="E185" t="n">
+        <v>369.17</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>Perfia box/₹4430, 12pc; MRP ₹8064/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="n">
+        <v>117</v>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Suture VP 2518 (per piece)</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>871</v>
+      </c>
+      <c r="E186" t="n">
+        <v>479.17</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>Perfia box/₹5750, 12pc; MRP ₹10452/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="n">
+        <v>118</v>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Suture NW 2317 (per piece)</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>900</v>
+      </c>
+      <c r="E187" t="n">
+        <v>495</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>Perfia box/₹5940, 12pc; MRP ₹10800/box</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="72" t="inlineStr">
         <is>
           <t>🔴 ITEMS MISSING MRP — Collect from vendor and update above</t>
         </is>
       </c>
-      <c r="B169" s="42" t="n"/>
-      <c r="C169" s="42" t="n"/>
-      <c r="D169" s="42" t="n"/>
-      <c r="E169" s="42" t="n"/>
-      <c r="F169" s="42" t="n"/>
-      <c r="G169" s="42" t="n"/>
-    </row>
-    <row r="170">
-      <c r="A170" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="B170" s="73" t="inlineStr">
-        <is>
-          <t>NS 100ml — Normal Saline 100ml</t>
-        </is>
-      </c>
-      <c r="C170" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D170" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E170" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F170" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G170" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="48" t="n">
-        <v>2</v>
-      </c>
-      <c r="B171" s="73" t="inlineStr">
-        <is>
-          <t>D5 500ml — Dextrose 5%</t>
-        </is>
-      </c>
-      <c r="C171" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D171" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E171" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F171" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G171" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" s="48" t="n">
-        <v>3</v>
-      </c>
-      <c r="B172" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
-        </is>
-      </c>
-      <c r="C172" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Anaesthesia</t>
-        </is>
-      </c>
-      <c r="D172" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E172" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F172" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G172" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" s="48" t="n">
-        <v>4</v>
-      </c>
-      <c r="B173" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Gentamicin</t>
-        </is>
-      </c>
-      <c r="C173" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D173" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E173" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F173" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G173" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" s="48" t="n">
-        <v>5</v>
-      </c>
-      <c r="B174" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Tramadol 50mg</t>
-        </is>
-      </c>
-      <c r="C174" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Analgesic</t>
-        </is>
-      </c>
-      <c r="D174" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E174" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F174" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G174" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" s="48" t="n">
-        <v>6</v>
-      </c>
-      <c r="B175" s="73" t="inlineStr">
-        <is>
-          <t>Inj. PCM 100ml (Paracetamol IV)</t>
-        </is>
-      </c>
-      <c r="C175" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Analgesic</t>
-        </is>
-      </c>
-      <c r="D175" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E175" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F175" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G175" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" s="48" t="n">
-        <v>7</v>
-      </c>
-      <c r="B176" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Carboprost (Hemabate)</t>
-        </is>
-      </c>
-      <c r="C176" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Oxytocic</t>
-        </is>
-      </c>
-      <c r="D176" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E176" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F176" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G176" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" s="48" t="n">
-        <v>8</v>
-      </c>
-      <c r="B177" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Adrenaline</t>
-        </is>
-      </c>
-      <c r="C177" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Emergency</t>
-        </is>
-      </c>
-      <c r="D177" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E177" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F177" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G177" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" s="48" t="n">
-        <v>9</v>
-      </c>
-      <c r="B178" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Cetil (Cefuroxime Axetil)</t>
-        </is>
-      </c>
-      <c r="C178" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D178" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E178" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F178" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G178" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="48" t="n">
-        <v>10</v>
-      </c>
-      <c r="B179" s="73" t="inlineStr">
-        <is>
-          <t>Needles 26G (Injection)</t>
-        </is>
-      </c>
-      <c r="C179" s="46" t="inlineStr">
-        <is>
-          <t>Consumable</t>
-        </is>
-      </c>
-      <c r="D179" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E179" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F179" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G179" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" s="48" t="n">
-        <v>11</v>
-      </c>
-      <c r="B180" s="73" t="inlineStr">
-        <is>
-          <t>Disposable Gloves (Exam)</t>
-        </is>
-      </c>
-      <c r="C180" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D180" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E180" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F180" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G180" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" s="48" t="n">
-        <v>12</v>
-      </c>
-      <c r="B181" s="73" t="inlineStr">
-        <is>
-          <t>Betadine Ointment 40g</t>
-        </is>
-      </c>
-      <c r="C181" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D181" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E181" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F181" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G181" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="48" t="n">
-        <v>13</v>
-      </c>
-      <c r="B182" s="73" t="inlineStr">
-        <is>
-          <t>Surgical Blade No. 10</t>
-        </is>
-      </c>
-      <c r="C182" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D182" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E182" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F182" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G182" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="48" t="n">
-        <v>14</v>
-      </c>
-      <c r="B183" s="73" t="inlineStr">
-        <is>
-          <t>Surgical Blade No. 20</t>
-        </is>
-      </c>
-      <c r="C183" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D183" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E183" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F183" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G183" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="48" t="n">
-        <v>15</v>
-      </c>
-      <c r="B184" s="73" t="inlineStr">
-        <is>
-          <t>Plain Sheet (OT Draping)</t>
-        </is>
-      </c>
-      <c r="C184" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D184" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E184" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F184" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G184" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="48" t="n">
-        <v>16</v>
-      </c>
-      <c r="B185" s="73" t="inlineStr">
-        <is>
-          <t>Soft Roll (OT Padding)</t>
-        </is>
-      </c>
-      <c r="C185" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D185" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E185" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F185" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G185" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="48" t="n">
-        <v>17</v>
-      </c>
-      <c r="B186" s="73" t="inlineStr">
-        <is>
-          <t>Gypsona POP Bandage 40G</t>
-        </is>
-      </c>
-      <c r="C186" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D186" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E186" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F186" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G186" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="48" t="n">
-        <v>18</v>
-      </c>
-      <c r="B187" s="73" t="inlineStr">
-        <is>
-          <t>Cap + Mask (Disposable Set)</t>
-        </is>
-      </c>
-      <c r="C187" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D187" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E187" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F187" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G187" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" s="48" t="n">
-        <v>19</v>
-      </c>
-      <c r="B188" s="73" t="inlineStr">
-        <is>
-          <t>Glucostrip (Blood Glucose)</t>
-        </is>
-      </c>
-      <c r="C188" s="46" t="inlineStr">
-        <is>
-          <t>Investigation</t>
-        </is>
-      </c>
-      <c r="D188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
+      <c r="B188" s="42" t="n"/>
+      <c r="C188" s="42" t="n"/>
+      <c r="D188" s="42" t="n"/>
+      <c r="E188" s="42" t="n"/>
+      <c r="F188" s="42" t="n"/>
+      <c r="G188" s="42" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="48" t="n">
-        <v>20</v>
+        <v>1</v>
       </c>
       <c r="B189" s="73" t="inlineStr">
         <is>
-          <t>Lancet Needle</t>
+          <t>NS 100ml — Normal Saline 100ml</t>
         </is>
       </c>
       <c r="C189" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>IV Fluid</t>
         </is>
       </c>
       <c r="D189" s="47" t="inlineStr">
@@ -5858,16 +5592,16 @@
     </row>
     <row r="190">
       <c r="A190" s="48" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="B190" s="73" t="inlineStr">
         <is>
-          <t>Red Top Tube (Blood Vial)</t>
+          <t>D5 500ml — Dextrose 5%</t>
         </is>
       </c>
       <c r="C190" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>IV Fluid</t>
         </is>
       </c>
       <c r="D190" s="47" t="inlineStr">
@@ -5893,16 +5627,16 @@
     </row>
     <row r="191">
       <c r="A191" s="48" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="B191" s="73" t="inlineStr">
         <is>
-          <t>CBC Vial Yellow + Red Top</t>
+          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
         </is>
       </c>
       <c r="C191" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>Injection — Anaesthesia</t>
         </is>
       </c>
       <c r="D191" s="47" t="inlineStr">
@@ -5928,16 +5662,16 @@
     </row>
     <row r="192">
       <c r="A192" s="48" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="B192" s="73" t="inlineStr">
         <is>
-          <t>O2 / Oxygen (per use)</t>
+          <t>Inj. Gentamicin</t>
         </is>
       </c>
       <c r="C192" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D192" s="47" t="inlineStr">
@@ -5963,16 +5697,16 @@
     </row>
     <row r="193">
       <c r="A193" s="48" t="n">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="B193" s="73" t="inlineStr">
         <is>
-          <t>Pulse Oximeter (per use)</t>
+          <t>Inj. Tramadol 50mg</t>
         </is>
       </c>
       <c r="C193" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Injection — Analgesic</t>
         </is>
       </c>
       <c r="D193" s="47" t="inlineStr">
@@ -5998,16 +5732,16 @@
     </row>
     <row r="194">
       <c r="A194" s="48" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="B194" s="73" t="inlineStr">
         <is>
-          <t>Cardiac Monitor (per use)</t>
+          <t>Inj. PCM 100ml (Paracetamol IV)</t>
         </is>
       </c>
       <c r="C194" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Injection — Analgesic</t>
         </is>
       </c>
       <c r="D194" s="47" t="inlineStr">
@@ -6033,16 +5767,16 @@
     </row>
     <row r="195">
       <c r="A195" s="48" t="n">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="B195" s="73" t="inlineStr">
         <is>
-          <t>C-arm (per use)</t>
+          <t>Inj. Carboprost (Hemabate)</t>
         </is>
       </c>
       <c r="C195" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Injection — Oxytocic</t>
         </is>
       </c>
       <c r="D195" s="47" t="inlineStr">
@@ -6068,34 +5802,699 @@
     </row>
     <row r="196">
       <c r="A196" s="48" t="n">
+        <v>8</v>
+      </c>
+      <c r="B196" s="73" t="inlineStr">
+        <is>
+          <t>Inj. Adrenaline</t>
+        </is>
+      </c>
+      <c r="C196" s="46" t="inlineStr">
+        <is>
+          <t>Injection — Emergency</t>
+        </is>
+      </c>
+      <c r="D196" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E196" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F196" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G196" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="48" t="n">
+        <v>9</v>
+      </c>
+      <c r="B197" s="73" t="inlineStr">
+        <is>
+          <t>Inj. Cetil (Cefuroxime Axetil)</t>
+        </is>
+      </c>
+      <c r="C197" s="46" t="inlineStr">
+        <is>
+          <t>Injection — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D197" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E197" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F197" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G197" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="48" t="n">
+        <v>10</v>
+      </c>
+      <c r="B198" s="73" t="inlineStr">
+        <is>
+          <t>Needles 26G (Injection)</t>
+        </is>
+      </c>
+      <c r="C198" s="46" t="inlineStr">
+        <is>
+          <t>Consumable</t>
+        </is>
+      </c>
+      <c r="D198" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E198" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F198" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G198" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="48" t="n">
+        <v>11</v>
+      </c>
+      <c r="B199" s="73" t="inlineStr">
+        <is>
+          <t>Disposable Gloves (Exam)</t>
+        </is>
+      </c>
+      <c r="C199" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D199" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E199" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F199" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G199" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="48" t="n">
+        <v>12</v>
+      </c>
+      <c r="B200" s="73" t="inlineStr">
+        <is>
+          <t>Betadine Ointment 40g</t>
+        </is>
+      </c>
+      <c r="C200" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D200" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E200" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F200" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G200" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="48" t="n">
+        <v>13</v>
+      </c>
+      <c r="B201" s="73" t="inlineStr">
+        <is>
+          <t>Surgical Blade No. 10</t>
+        </is>
+      </c>
+      <c r="C201" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D201" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E201" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F201" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G201" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="48" t="n">
+        <v>14</v>
+      </c>
+      <c r="B202" s="73" t="inlineStr">
+        <is>
+          <t>Surgical Blade No. 20</t>
+        </is>
+      </c>
+      <c r="C202" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D202" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E202" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F202" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G202" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="48" t="n">
+        <v>15</v>
+      </c>
+      <c r="B203" s="73" t="inlineStr">
+        <is>
+          <t>Plain Sheet (OT Draping)</t>
+        </is>
+      </c>
+      <c r="C203" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D203" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E203" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F203" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G203" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="48" t="n">
+        <v>16</v>
+      </c>
+      <c r="B204" s="73" t="inlineStr">
+        <is>
+          <t>Soft Roll (OT Padding)</t>
+        </is>
+      </c>
+      <c r="C204" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D204" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E204" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F204" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G204" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="48" t="n">
+        <v>17</v>
+      </c>
+      <c r="B205" s="73" t="inlineStr">
+        <is>
+          <t>Gypsona POP Bandage 40G</t>
+        </is>
+      </c>
+      <c r="C205" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D205" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E205" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F205" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G205" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="48" t="n">
+        <v>18</v>
+      </c>
+      <c r="B206" s="73" t="inlineStr">
+        <is>
+          <t>Cap + Mask (Disposable Set)</t>
+        </is>
+      </c>
+      <c r="C206" s="46" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D206" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E206" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F206" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G206" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="48" t="n">
+        <v>19</v>
+      </c>
+      <c r="B207" s="73" t="inlineStr">
+        <is>
+          <t>Glucostrip (Blood Glucose)</t>
+        </is>
+      </c>
+      <c r="C207" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D207" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E207" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F207" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G207" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="B208" s="73" t="inlineStr">
+        <is>
+          <t>Lancet Needle</t>
+        </is>
+      </c>
+      <c r="C208" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D208" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E208" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F208" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G208" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="48" t="n">
+        <v>21</v>
+      </c>
+      <c r="B209" s="73" t="inlineStr">
+        <is>
+          <t>Red Top Tube (Blood Vial)</t>
+        </is>
+      </c>
+      <c r="C209" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D209" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E209" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F209" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G209" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="48" t="n">
+        <v>22</v>
+      </c>
+      <c r="B210" s="73" t="inlineStr">
+        <is>
+          <t>CBC Vial Yellow + Red Top</t>
+        </is>
+      </c>
+      <c r="C210" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D210" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E210" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F210" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G210" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="48" t="n">
+        <v>23</v>
+      </c>
+      <c r="B211" s="73" t="inlineStr">
+        <is>
+          <t>O2 / Oxygen (per use)</t>
+        </is>
+      </c>
+      <c r="C211" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D211" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E211" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F211" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G211" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="48" t="n">
+        <v>24</v>
+      </c>
+      <c r="B212" s="73" t="inlineStr">
+        <is>
+          <t>Pulse Oximeter (per use)</t>
+        </is>
+      </c>
+      <c r="C212" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D212" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E212" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F212" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G212" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="48" t="n">
+        <v>25</v>
+      </c>
+      <c r="B213" s="73" t="inlineStr">
+        <is>
+          <t>Cardiac Monitor (per use)</t>
+        </is>
+      </c>
+      <c r="C213" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D213" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E213" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F213" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G213" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="48" t="n">
+        <v>26</v>
+      </c>
+      <c r="B214" s="73" t="inlineStr">
+        <is>
+          <t>C-arm (per use)</t>
+        </is>
+      </c>
+      <c r="C214" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="48" t="n">
         <v>27</v>
       </c>
-      <c r="B196" s="73" t="inlineStr">
+      <c r="B215" s="73" t="inlineStr">
         <is>
           <t>Volu-P / TiCUP</t>
         </is>
       </c>
-      <c r="C196" s="46" t="inlineStr">
+      <c r="C215" s="46" t="inlineStr">
         <is>
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D196" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E196" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F196" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G196" s="47" t="inlineStr">
+      <c r="D215" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E215" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F215" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G215" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL IN</t>
         </is>

</xml_diff>

<commit_message>
Fix Easyfix rate ₹900 → ₹5 across all billing files; changed cells highlighted yellow
- Add BKAditya_PatientBilling_FINAL.xlsx (first 15 patients, Feb–May 2026)
  with 7 Easyfix rows corrected and all subtotals/grand totals/summary
  recomputed
- June 2026 workbook: 11 patient sheets corrected (formulas recalc)
- Master rate card SL48 & SL61 corrected; cost flagged for verification
- Raju Mondal mediclaim: section E, total and gap analysis recomputed

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YWgR3jd3MUcEXpU4s4WC54
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -110,7 +110,7 @@
       <sz val="8"/>
     </font>
   </fonts>
-  <fills count="14">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -189,6 +189,11 @@
         <bgColor rgb="FFEBF3FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -257,7 +262,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -474,6 +479,15 @@
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="10" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
@@ -2459,20 +2473,20 @@
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D65" s="53" t="n">
-        <v>900</v>
+      <c r="D65" s="74" t="n">
+        <v>5</v>
       </c>
       <c r="E65" s="53" t="n">
         <v>300</v>
       </c>
-      <c r="F65" s="65" t="inlineStr">
-        <is>
-          <t>66.7%</t>
-        </is>
-      </c>
-      <c r="G65" s="52" t="inlineStr">
-        <is>
-          <t>CLD 3x proxy</t>
+      <c r="F65" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G65" s="76" t="inlineStr">
+        <is>
+          <t>User-corrected rate ₹5 (was CLD 3x proxy ₹900); verify cost</t>
         </is>
       </c>
     </row>
@@ -2866,20 +2880,20 @@
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D78" s="53" t="n">
-        <v>900</v>
+      <c r="D78" s="74" t="n">
+        <v>5</v>
       </c>
       <c r="E78" s="53" t="n">
         <v>300</v>
       </c>
-      <c r="F78" s="65" t="inlineStr">
-        <is>
-          <t>66.7%</t>
-        </is>
-      </c>
-      <c r="G78" s="52" t="inlineStr">
-        <is>
-          <t>CLD 3x proxy</t>
+      <c r="F78" s="75" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G78" s="76" t="inlineStr">
+        <is>
+          <t>User-corrected rate ₹5 (was CLD 3x proxy ₹900); verify cost</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4171,6 @@
         </is>
       </c>
     </row>
-    <row r="121"/>
     <row r="122" ht="13.5" customHeight="1" s="37">
       <c r="A122" s="36" t="n">
         <v>100</v>
@@ -5144,399 +5157,399 @@
       </c>
     </row>
     <row r="169">
-      <c r="A169" t="n">
+      <c r="A169" s="36" t="n">
         <v>100</v>
       </c>
-      <c r="B169" t="inlineStr">
+      <c r="B169" s="36" t="inlineStr">
         <is>
           <t>Hip U Drape</t>
         </is>
       </c>
-      <c r="D169" t="n">
+      <c r="D169" s="36" t="n">
         <v>1983</v>
       </c>
-      <c r="E169" t="n">
+      <c r="E169" s="36" t="n">
         <v>1350</v>
       </c>
-      <c r="G169" t="inlineStr">
+      <c r="G169" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹6750</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" t="n">
+      <c r="A170" s="36" t="n">
         <v>101</v>
       </c>
-      <c r="B170" t="inlineStr">
+      <c r="B170" s="36" t="inlineStr">
         <is>
           <t>Ioban Surgical Drape</t>
         </is>
       </c>
-      <c r="D170" t="n">
+      <c r="D170" s="36" t="n">
         <v>1590</v>
       </c>
-      <c r="E170" t="n">
+      <c r="E170" s="36" t="n">
         <v>625</v>
       </c>
-      <c r="G170" t="inlineStr">
+      <c r="G170" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 1box/₹7500 (12pc)</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" t="n">
+      <c r="A171" s="36" t="n">
         <v>102</v>
       </c>
-      <c r="B171" t="inlineStr">
+      <c r="B171" s="36" t="inlineStr">
         <is>
           <t>Suction Tube (VACCU)</t>
         </is>
       </c>
-      <c r="D171" t="n">
+      <c r="D171" s="36" t="n">
         <v>543</v>
       </c>
-      <c r="E171" t="n">
+      <c r="E171" s="36" t="n">
         <v>50</v>
       </c>
-      <c r="G171" t="inlineStr">
+      <c r="G171" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List</t>
         </is>
       </c>
     </row>
     <row r="172">
-      <c r="A172" t="n">
+      <c r="A172" s="36" t="n">
         <v>103</v>
       </c>
-      <c r="B172" t="inlineStr">
+      <c r="B172" s="36" t="inlineStr">
         <is>
           <t>Bardia 3-Way Catheter 22Fr</t>
         </is>
       </c>
-      <c r="D172" t="n">
+      <c r="D172" s="36" t="n">
         <v>408</v>
       </c>
-      <c r="E172" t="n">
+      <c r="E172" s="36" t="n">
         <v>320</v>
       </c>
-      <c r="G172" t="inlineStr">
+      <c r="G172" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹1600</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" t="n">
+      <c r="A173" s="36" t="n">
         <v>104</v>
       </c>
-      <c r="B173" t="inlineStr">
+      <c r="B173" s="36" t="inlineStr">
         <is>
           <t>Bardia 2-Way Catheter 14Fr</t>
         </is>
       </c>
-      <c r="D173" t="n">
+      <c r="D173" s="36" t="n">
         <v>179</v>
       </c>
-      <c r="E173" t="n">
+      <c r="E173" s="36" t="n">
         <v>130</v>
       </c>
-      <c r="G173" t="inlineStr">
+      <c r="G173" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹650</t>
         </is>
       </c>
     </row>
     <row r="174">
-      <c r="A174" t="n">
+      <c r="A174" s="36" t="n">
         <v>105</v>
       </c>
-      <c r="B174" t="inlineStr">
+      <c r="B174" s="36" t="inlineStr">
         <is>
           <t>Bardia 2-Way Catheter 16Fr</t>
         </is>
       </c>
-      <c r="D174" t="n">
+      <c r="D174" s="36" t="n">
         <v>191</v>
       </c>
-      <c r="E174" t="n">
+      <c r="E174" s="36" t="n">
         <v>130</v>
       </c>
-      <c r="G174" t="inlineStr">
+      <c r="G174" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹650</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" t="n">
+      <c r="A175" s="36" t="n">
         <v>106</v>
       </c>
-      <c r="B175" t="inlineStr">
+      <c r="B175" s="36" t="inlineStr">
         <is>
           <t>Bardia 2-Way Catheter 18Fr</t>
         </is>
       </c>
-      <c r="D175" t="n">
+      <c r="D175" s="36" t="n">
         <v>174</v>
       </c>
-      <c r="E175" t="n">
+      <c r="E175" s="36" t="n">
         <v>130</v>
       </c>
-      <c r="G175" t="inlineStr">
+      <c r="G175" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹650</t>
         </is>
       </c>
     </row>
     <row r="176">
-      <c r="A176" t="n">
+      <c r="A176" s="36" t="n">
         <v>107</v>
       </c>
-      <c r="B176" t="inlineStr">
+      <c r="B176" s="36" t="inlineStr">
         <is>
           <t>IV Cannula 24G</t>
         </is>
       </c>
-      <c r="D176" t="n">
+      <c r="D176" s="36" t="n">
         <v>693</v>
       </c>
-      <c r="E176" t="n">
+      <c r="E176" s="36" t="n">
         <v>350</v>
       </c>
-      <c r="G176" t="inlineStr">
+      <c r="G176" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" t="n">
+      <c r="A177" s="36" t="n">
         <v>108</v>
       </c>
-      <c r="B177" t="inlineStr">
+      <c r="B177" s="36" t="inlineStr">
         <is>
           <t>Gamji Roll</t>
         </is>
       </c>
-      <c r="D177" t="n">
+      <c r="D177" s="36" t="n">
         <v>250</v>
       </c>
-      <c r="E177" t="n">
+      <c r="E177" s="36" t="n">
         <v>80</v>
       </c>
-      <c r="G177" t="inlineStr">
+      <c r="G177" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹400</t>
         </is>
       </c>
     </row>
     <row r="178">
-      <c r="A178" t="n">
+      <c r="A178" s="36" t="n">
         <v>109</v>
       </c>
-      <c r="B178" t="inlineStr">
+      <c r="B178" s="36" t="inlineStr">
         <is>
           <t>C Colin Tube Size 14</t>
         </is>
       </c>
-      <c r="D178" t="n">
+      <c r="D178" s="36" t="n">
         <v>842</v>
       </c>
-      <c r="E178" t="n">
+      <c r="E178" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="G178" t="inlineStr">
+      <c r="G178" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹100</t>
         </is>
       </c>
     </row>
     <row r="179">
-      <c r="A179" t="n">
+      <c r="A179" s="36" t="n">
         <v>110</v>
       </c>
-      <c r="B179" t="inlineStr">
+      <c r="B179" s="36" t="inlineStr">
         <is>
           <t>C Colin Tube Size 16</t>
         </is>
       </c>
-      <c r="D179" t="n">
+      <c r="D179" s="36" t="n">
         <v>842</v>
       </c>
-      <c r="E179" t="n">
+      <c r="E179" s="36" t="n">
         <v>20</v>
       </c>
-      <c r="G179" t="inlineStr">
+      <c r="G179" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 5pcs/₹100</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" t="n">
+      <c r="A180" s="36" t="n">
         <v>111</v>
       </c>
-      <c r="B180" t="inlineStr">
+      <c r="B180" s="36" t="inlineStr">
         <is>
           <t>Nasal Cannula</t>
         </is>
       </c>
-      <c r="D180" t="n">
+      <c r="D180" s="36" t="n">
         <v>255</v>
       </c>
-      <c r="E180" t="n">
+      <c r="E180" s="36" t="n">
         <v>50</v>
       </c>
-      <c r="G180" t="inlineStr">
+      <c r="G180" s="36" t="inlineStr">
         <is>
           <t>Perfia Consumables List 3pcs/₹150</t>
         </is>
       </c>
     </row>
     <row r="181">
-      <c r="A181" t="n">
+      <c r="A181" s="36" t="n">
         <v>112</v>
       </c>
-      <c r="B181" t="inlineStr">
+      <c r="B181" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2478 (per piece)</t>
         </is>
       </c>
-      <c r="D181" t="n">
+      <c r="D181" s="36" t="n">
         <v>1223</v>
       </c>
-      <c r="E181" t="n">
+      <c r="E181" s="36" t="n">
         <v>672.5</v>
       </c>
-      <c r="G181" t="inlineStr">
+      <c r="G181" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹8070, 12pc; MRP ₹14676/box</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" t="n">
+      <c r="A182" s="36" t="n">
         <v>113</v>
       </c>
-      <c r="B182" t="inlineStr">
+      <c r="B182" s="36" t="inlineStr">
         <is>
           <t>Suture NW 2477 (per piece)</t>
         </is>
       </c>
-      <c r="D182" t="n">
+      <c r="D182" s="36" t="n">
         <v>636</v>
       </c>
-      <c r="E182" t="n">
+      <c r="E182" s="36" t="n">
         <v>350</v>
       </c>
-      <c r="G182" t="inlineStr">
+      <c r="G182" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹4200, 12pc; MRP ₹7632/box</t>
         </is>
       </c>
     </row>
     <row r="183">
-      <c r="A183" t="n">
+      <c r="A183" s="36" t="n">
         <v>114</v>
       </c>
-      <c r="B183" t="inlineStr">
+      <c r="B183" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2548 (per piece)</t>
         </is>
       </c>
-      <c r="D183" t="n">
+      <c r="D183" s="36" t="n">
         <v>1059</v>
       </c>
-      <c r="E183" t="n">
+      <c r="E183" s="36" t="n">
         <v>558.33</v>
       </c>
-      <c r="G183" t="inlineStr">
+      <c r="G183" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹6700, 12pc; MRP ₹12710/box</t>
         </is>
       </c>
     </row>
     <row r="184">
-      <c r="A184" t="n">
+      <c r="A184" s="36" t="n">
         <v>115</v>
       </c>
-      <c r="B184" t="inlineStr">
+      <c r="B184" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2421 (per piece)</t>
         </is>
       </c>
-      <c r="D184" t="n">
+      <c r="D184" s="36" t="n">
         <v>1171</v>
       </c>
-      <c r="E184" t="n">
+      <c r="E184" s="36" t="n">
         <v>644.17</v>
       </c>
-      <c r="G184" t="inlineStr">
+      <c r="G184" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹7730, 12pc; MRP ₹14052/box</t>
         </is>
       </c>
     </row>
     <row r="185">
-      <c r="A185" t="n">
+      <c r="A185" s="36" t="n">
         <v>116</v>
       </c>
-      <c r="B185" t="inlineStr">
+      <c r="B185" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2304 (per piece)</t>
         </is>
       </c>
-      <c r="D185" t="n">
+      <c r="D185" s="36" t="n">
         <v>672</v>
       </c>
-      <c r="E185" t="n">
+      <c r="E185" s="36" t="n">
         <v>369.17</v>
       </c>
-      <c r="G185" t="inlineStr">
+      <c r="G185" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹4430, 12pc; MRP ₹8064/box</t>
         </is>
       </c>
     </row>
     <row r="186">
-      <c r="A186" t="n">
+      <c r="A186" s="36" t="n">
         <v>117</v>
       </c>
-      <c r="B186" t="inlineStr">
+      <c r="B186" s="36" t="inlineStr">
         <is>
           <t>Suture VP 2518 (per piece)</t>
         </is>
       </c>
-      <c r="D186" t="n">
+      <c r="D186" s="36" t="n">
         <v>871</v>
       </c>
-      <c r="E186" t="n">
+      <c r="E186" s="36" t="n">
         <v>479.17</v>
       </c>
-      <c r="G186" t="inlineStr">
+      <c r="G186" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹5750, 12pc; MRP ₹10452/box</t>
         </is>
       </c>
     </row>
     <row r="187">
-      <c r="A187" t="n">
+      <c r="A187" s="36" t="n">
         <v>118</v>
       </c>
-      <c r="B187" t="inlineStr">
+      <c r="B187" s="36" t="inlineStr">
         <is>
           <t>Suture NW 2317 (per piece)</t>
         </is>
       </c>
-      <c r="D187" t="n">
+      <c r="D187" s="36" t="n">
         <v>900</v>
       </c>
-      <c r="E187" t="n">
+      <c r="E187" s="36" t="n">
         <v>495</v>
       </c>
-      <c r="G187" t="inlineStr">
+      <c r="G187" s="36" t="inlineStr">
         <is>
           <t>Perfia box/₹5940, 12pc; MRP ₹10800/box</t>
         </is>

</xml_diff>

<commit_message>
Fill 20 rate card MRPs from stock file; fill 190 ⚠ items across 43 patient sheets
- Updated BKAditya_MasterRateCard_UPDATED.xlsx: filled MRPs for 20 items using
  stock file (Anawin, Carboprost, T-Tet, Adrenaline, TUR Set, C-Arm Cover,
  ET Tube, RAE Nasal, Romo Bougie, Romo-ADK, Suspensory, Glycine, Liquid
  Paraffin, Leukoplast, Betadine, Full Gown, Distilled Water, etc.)
- Updated BKAditya_AllPatients_FinalBill.xlsx: resolved 190 ⚠ items across
  43 patient sheets using rate card + stock file MRP lookups
- Updated ⚠ TO PRICE sheet: 79 rows now carry MRP/cost data
- 11 items still need manual MRP: Cardiac Monitor, O2, Pulse Oximeter,
  ECG Lead Wires, Lap Instruments, Tab PCM 650mg, and 5 others

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -1047,16 +1047,14 @@
           <t>Injection — Anaesthesia</t>
         </is>
       </c>
-      <c r="D13" s="47" t="inlineStr">
+      <c r="D13" s="47" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="E13" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL</t>
         </is>
       </c>
-      <c r="E13" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
-      </c>
       <c r="F13" s="48" t="inlineStr">
         <is>
           <t>—</t>
@@ -1064,7 +1062,7 @@
       </c>
       <c r="G13" s="46" t="inlineStr">
         <is>
-          <t>⚠ MRP NOT FOUND</t>
+          <t>Stock OT: ANAWIN 0.25% 20ML</t>
         </is>
       </c>
     </row>
@@ -1559,7 +1557,7 @@
       </c>
       <c r="G30" s="52" t="inlineStr">
         <is>
-          <t>⚠ Est. Market rate</t>
+          <t>Est. market — Diclofenac Sodium 100mg (Jonac)</t>
         </is>
       </c>
     </row>
@@ -2063,16 +2061,14 @@
           <t>Injection — Oxytocic</t>
         </is>
       </c>
-      <c r="D49" s="47" t="inlineStr">
+      <c r="D49" s="47" t="n">
+        <v>318.5</v>
+      </c>
+      <c r="E49" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL</t>
         </is>
       </c>
-      <c r="E49" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
-      </c>
       <c r="F49" s="48" t="inlineStr">
         <is>
           <t>—</t>
@@ -2080,7 +2076,7 @@
       </c>
       <c r="G49" s="46" t="inlineStr">
         <is>
-          <t>⚠ MRP NOT FOUND</t>
+          <t>Stock OT: CARBOPOST</t>
         </is>
       </c>
     </row>
@@ -2244,7 +2240,7 @@
         </is>
       </c>
       <c r="D57" s="53" t="n">
-        <v>20</v>
+        <v>27.27</v>
       </c>
       <c r="E57" s="58" t="inlineStr">
         <is>
@@ -2258,7 +2254,7 @@
       </c>
       <c r="G57" s="52" t="inlineStr">
         <is>
-          <t>⚠ Est. Market rate</t>
+          <t>Stock Fridge: TETANUS VACCINE ₹27.27</t>
         </is>
       </c>
     </row>
@@ -2304,7 +2300,7 @@
       </c>
       <c r="G59" s="46" t="inlineStr">
         <is>
-          <t>Stock file</t>
+          <t>Stock OT/Ward: ADRENALIN 1ML ₹13.40</t>
         </is>
       </c>
     </row>
@@ -2831,16 +2827,14 @@
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D77" s="47" t="inlineStr">
+      <c r="D77" s="47" t="n">
+        <v>260</v>
+      </c>
+      <c r="E77" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL</t>
         </is>
       </c>
-      <c r="E77" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
-      </c>
       <c r="F77" s="48" t="inlineStr">
         <is>
           <t>—</t>
@@ -2848,7 +2842,7 @@
       </c>
       <c r="G77" s="46" t="inlineStr">
         <is>
-          <t>⚠ MRP NOT FOUND</t>
+          <t>Stock Ward: DISPOVEIN NEEDLE 26 NO (per box ~100pcs)</t>
         </is>
       </c>
     </row>
@@ -3193,16 +3187,14 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D89" s="47" t="inlineStr">
+      <c r="D89" s="47" t="n">
+        <v>132</v>
+      </c>
+      <c r="E89" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL</t>
         </is>
       </c>
-      <c r="E89" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
-      </c>
       <c r="F89" s="48" t="inlineStr">
         <is>
           <t>—</t>
@@ -3210,7 +3202,7 @@
       </c>
       <c r="G89" s="46" t="inlineStr">
         <is>
-          <t>⚠ MRP NOT FOUND</t>
+          <t>Stock OT: POVIDINE OINTMENT 20gm ₹132 (proxy for 40g)</t>
         </is>
       </c>
     </row>
@@ -3666,16 +3658,14 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D104" s="47" t="inlineStr">
+      <c r="D104" s="47" t="n">
+        <v>25</v>
+      </c>
+      <c r="E104" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL</t>
         </is>
       </c>
-      <c r="E104" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
-      </c>
       <c r="F104" s="48" t="inlineStr">
         <is>
           <t>—</t>
@@ -3683,7 +3673,7 @@
       </c>
       <c r="G104" s="46" t="inlineStr">
         <is>
-          <t>⚠ MRP NOT FOUND</t>
+          <t>Est. market rate — cap+mask set per pair</t>
         </is>
       </c>
     </row>
@@ -4157,7 +4147,6 @@
         </is>
       </c>
     </row>
-    <row r="121"/>
     <row r="122" ht="13.5" customHeight="1" s="37">
       <c r="A122" s="36" t="n">
         <v>100</v>
@@ -4225,7 +4214,7 @@
       <c r="E125" s="36" t="n">
         <v>362.24</v>
       </c>
-      <c r="F125" t="inlineStr">
+      <c r="F125" s="36" t="inlineStr">
         <is>
           <t>11.2%</t>
         </is>
@@ -4612,17 +4601,20 @@
           <t>TUR Set (Transurethral Resection)</t>
         </is>
       </c>
-      <c r="D143" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D143" s="36" t="n">
+        <v>523</v>
       </c>
       <c r="E143" s="36" t="n">
         <v>107.95</v>
       </c>
+      <c r="F143" s="36" t="inlineStr">
+        <is>
+          <t>79.4%</t>
+        </is>
+      </c>
       <c r="G143" s="36" t="inlineStr">
         <is>
-          <t>CLD Surgical #270 — MRP not on invoice</t>
+          <t>Stock OT: TURP SET</t>
         </is>
       </c>
     </row>
@@ -4635,17 +4627,20 @@
           <t>C-Arm Cover (Disposable Drape)</t>
         </is>
       </c>
-      <c r="D144" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D144" s="36" t="n">
+        <v>234</v>
       </c>
       <c r="E144" s="36" t="n">
         <v>157.71</v>
       </c>
+      <c r="F144" s="36" t="inlineStr">
+        <is>
+          <t>32.6%</t>
+        </is>
+      </c>
       <c r="G144" s="36" t="inlineStr">
         <is>
-          <t>CLD Surgical #270 — MRP not on invoice</t>
+          <t>Stock OT: C-ARM COVER</t>
         </is>
       </c>
     </row>
@@ -4704,17 +4699,20 @@
           <t>ET Tube No.6 — Armead</t>
         </is>
       </c>
-      <c r="D147" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D147" s="36" t="n">
+        <v>399</v>
       </c>
       <c r="E147" s="36" t="n">
         <v>625.3200000000001</v>
       </c>
+      <c r="F147" s="36" t="inlineStr">
+        <is>
+          <t>-56.7%</t>
+        </is>
+      </c>
       <c r="G147" s="36" t="inlineStr">
         <is>
-          <t>MP Enterprise #236</t>
+          <t>Stock OT: ET TUBE 6 NO</t>
         </is>
       </c>
     </row>
@@ -4727,17 +4725,20 @@
           <t>RAE Nasal Tube</t>
         </is>
       </c>
-      <c r="D148" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D148" s="36" t="n">
+        <v>1595</v>
       </c>
       <c r="E148" s="36" t="n">
         <v>632</v>
       </c>
+      <c r="F148" s="36" t="inlineStr">
+        <is>
+          <t>60.4%</t>
+        </is>
+      </c>
       <c r="G148" s="36" t="inlineStr">
         <is>
-          <t>MP Enterprise #236</t>
+          <t>Stock OT: NASAL TUBE ADULT 6 NO</t>
         </is>
       </c>
     </row>
@@ -4750,17 +4751,20 @@
           <t>Romo Bougie (Surgical Dilator)</t>
         </is>
       </c>
-      <c r="D149" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D149" s="36" t="n">
+        <v>1952</v>
       </c>
       <c r="E149" s="36" t="n">
         <v>292.75</v>
       </c>
+      <c r="F149" s="36" t="inlineStr">
+        <is>
+          <t>85.0%</t>
+        </is>
+      </c>
       <c r="G149" s="36" t="inlineStr">
         <is>
-          <t>MP Enterprise #236</t>
+          <t>Stock OT: BOUGIE</t>
         </is>
       </c>
     </row>
@@ -4778,22 +4782,20 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D150" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D150" s="36" t="n">
+        <v>509</v>
       </c>
       <c r="E150" s="36" t="n">
         <v>124.87</v>
       </c>
       <c r="F150" s="36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>75.5%</t>
         </is>
       </c>
       <c r="G150" s="36" t="inlineStr">
         <is>
-          <t>MP Enterprise #236</t>
+          <t>Stock OT: ROMO-ADK (ABDOMINAL DRAINAGE) 28 NO</t>
         </is>
       </c>
     </row>
@@ -4811,22 +4813,20 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D151" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D151" s="36" t="n">
+        <v>70</v>
       </c>
       <c r="E151" s="36" t="n">
         <v>19.52</v>
       </c>
       <c r="F151" s="36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>72.1%</t>
         </is>
       </c>
       <c r="G151" s="36" t="inlineStr">
         <is>
-          <t>MP Enterprise #236</t>
+          <t>Stock OT: SUSPENSORY BANDAGE XL (per box)</t>
         </is>
       </c>
     </row>
@@ -4844,22 +4844,20 @@
           <t>IV Fluid</t>
         </is>
       </c>
-      <c r="D152" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D152" s="36" t="n">
+        <v>704</v>
       </c>
       <c r="E152" s="36" t="n">
         <v>128</v>
       </c>
       <c r="F152" s="36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>81.8%</t>
         </is>
       </c>
       <c r="G152" s="36" t="inlineStr">
         <is>
-          <t>MP Enterprise #234</t>
+          <t>Stock OT: GLYCIN (3000ml)</t>
         </is>
       </c>
     </row>
@@ -4877,22 +4875,20 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D153" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D153" s="36" t="n">
+        <v>262</v>
       </c>
       <c r="E153" s="36" t="n">
         <v>158.12</v>
       </c>
       <c r="F153" s="36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>39.6%</t>
         </is>
       </c>
       <c r="G153" s="36" t="inlineStr">
         <is>
-          <t>MP Enterprise #234</t>
+          <t>Stock OT: PARAPHI OIL</t>
         </is>
       </c>
     </row>
@@ -4941,22 +4937,20 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D155" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D155" s="36" t="n">
+        <v>364</v>
       </c>
       <c r="E155" s="36" t="n">
         <v>225</v>
       </c>
       <c r="F155" s="36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>38.2%</t>
         </is>
       </c>
       <c r="G155" s="36" t="inlineStr">
         <is>
-          <t>CLD Surgical #270</t>
+          <t>Stock Ward: LEUKOPLAST 7.5CM</t>
         </is>
       </c>
     </row>
@@ -5385,22 +5379,20 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D169" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D169" s="36" t="n">
+        <v>514</v>
       </c>
       <c r="E169" s="36" t="n">
         <v>200</v>
       </c>
       <c r="F169" s="36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>61.1%</t>
         </is>
       </c>
       <c r="G169" s="36" t="inlineStr">
         <is>
-          <t>CLD Surgical #328 BETADIN 500M</t>
+          <t>Stock Ward/OT: BETADINE 10% 500ML</t>
         </is>
       </c>
     </row>
@@ -5482,22 +5474,20 @@
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D172" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D172" s="36" t="n">
+        <v>470</v>
       </c>
       <c r="E172" s="36" t="n">
         <v>265</v>
       </c>
       <c r="F172" s="36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>43.6%</t>
         </is>
       </c>
       <c r="G172" s="36" t="inlineStr">
         <is>
-          <t>CLD Surgical #343 FULL GOWN SD SD10426</t>
+          <t>Stock OT: STERILE DISPOSABLE GOWN</t>
         </is>
       </c>
     </row>
@@ -5680,22 +5670,20 @@
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D178" s="36" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D178" s="36" t="n">
+        <v>3.12</v>
       </c>
       <c r="E178" s="36" t="n">
         <v>2.15</v>
       </c>
       <c r="F178" s="36" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>31.1%</t>
         </is>
       </c>
       <c r="G178" s="36" t="inlineStr">
         <is>
-          <t>CLD Surgical #355 DISTIL WATE</t>
+          <t>Stock OT: D. WATER per piece</t>
         </is>
       </c>
     </row>
@@ -6004,10 +5992,8 @@
           <t>Injection — Emergency</t>
         </is>
       </c>
-      <c r="D188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
+      <c r="D188" s="47" t="n">
+        <v>13.4</v>
       </c>
       <c r="E188" s="47" t="inlineStr">
         <is>
@@ -6016,12 +6002,12 @@
       </c>
       <c r="F188" s="47" t="inlineStr">
         <is>
-          <t>⚠ FILL IN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G188" s="47" t="inlineStr">
         <is>
-          <t>⚠ FILL IN</t>
+          <t>Stock OT/Ward: ADRENALIN 1ML</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add Aug 2026 invoices to rate card and purchase CSVs
Rate card: SL 158–164 added
  158: Doxyvac 100MG (Doxycycline) MRP 527 / Cost 120
  159: Alburel 20% IV (Albumin) Cost 4650 — MRP needs fill
  160: Neomol 400ML IV Bag MRP 591.50 / Cost 35
  161: Centro Trio (Drainage) MRP 3255 / Cost 782
  162: Urometer MRP 629 / Cost 97.50
  163: Molysheet NARASHA MRP 155 / Cost 13.50
  164: Jelonet Tin MRP 200.30 / Cost 145

Purchase Summary: 6 new invoices (MR000994, BP463, BP467, MR001009, BP485, MR001012)
Line Items: 18 new rows across all 6 invoices

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -109,8 +109,12 @@
       <color rgb="FF9C0006"/>
       <sz val="8"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="14">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -189,8 +193,20 @@
         <bgColor rgb="FFEBF3FB"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFDA"/>
+        <bgColor rgb="FFE2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -246,6 +262,20 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -257,7 +287,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="74">
+  <cellXfs count="76">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -475,6 +505,12 @@
     </xf>
     <xf numFmtId="0" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -729,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G207"/>
+  <dimension ref="A1:G214"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="36" min="1" max="1"/>
@@ -4147,6 +4183,7 @@
         </is>
       </c>
     </row>
+    <row r="121"/>
     <row r="122" ht="13.5" customHeight="1" s="37">
       <c r="A122" s="36" t="n">
         <v>100</v>
@@ -5721,279 +5758,249 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="72" t="inlineStr">
+      <c r="A180" s="74" t="n">
+        <v>158</v>
+      </c>
+      <c r="B180" s="74" t="inlineStr">
+        <is>
+          <t>Doxyvac 100MG (Doxycycline)</t>
+        </is>
+      </c>
+      <c r="C180" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D180" s="74" t="n">
+        <v>527</v>
+      </c>
+      <c r="E180" s="74" t="n">
+        <v>120</v>
+      </c>
+      <c r="F180" s="74">
+        <f>(D180-E180)/D180</f>
+        <v/>
+      </c>
+      <c r="G180" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001009 / 12-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="75" t="n">
+        <v>159</v>
+      </c>
+      <c r="B181" s="75" t="inlineStr">
+        <is>
+          <t>Alburel IV 20% 100ML (Human Albumin)</t>
+        </is>
+      </c>
+      <c r="C181" s="75" t="inlineStr">
+        <is>
+          <t>Injection — IV</t>
+        </is>
+      </c>
+      <c r="D181" s="75" t="inlineStr">
+        <is>
+          <t>⚠ FILL</t>
+        </is>
+      </c>
+      <c r="E181" s="75" t="n">
+        <v>4650</v>
+      </c>
+      <c r="F181" s="75" t="inlineStr">
+        <is>
+          <t>⚠ FILL</t>
+        </is>
+      </c>
+      <c r="G181" s="75" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001009 / 12-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="74" t="n">
+        <v>160</v>
+      </c>
+      <c r="B182" s="74" t="inlineStr">
+        <is>
+          <t>Neomol 400ML IV Bag (Paracetamol)</t>
+        </is>
+      </c>
+      <c r="C182" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Analgesic</t>
+        </is>
+      </c>
+      <c r="D182" s="74" t="n">
+        <v>591.5</v>
+      </c>
+      <c r="E182" s="74" t="n">
+        <v>35</v>
+      </c>
+      <c r="F182" s="74">
+        <f>(D182-E182)/D182</f>
+        <v/>
+      </c>
+      <c r="G182" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR000994 / 10-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="74" t="n">
+        <v>161</v>
+      </c>
+      <c r="B183" s="74" t="inlineStr">
+        <is>
+          <t>Centro Trio (Drainage Device)</t>
+        </is>
+      </c>
+      <c r="C183" s="74" t="inlineStr">
+        <is>
+          <t>Surgical Device</t>
+        </is>
+      </c>
+      <c r="D183" s="74" t="n">
+        <v>3255</v>
+      </c>
+      <c r="E183" s="74" t="n">
+        <v>782</v>
+      </c>
+      <c r="F183" s="74">
+        <f>(D183-E183)/D183</f>
+        <v/>
+      </c>
+      <c r="G183" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #485 / 12-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="74" t="n">
+        <v>162</v>
+      </c>
+      <c r="B184" s="74" t="inlineStr">
+        <is>
+          <t>Urometer (Urine Output Measuring)</t>
+        </is>
+      </c>
+      <c r="C184" s="74" t="inlineStr">
+        <is>
+          <t>Surgical Device</t>
+        </is>
+      </c>
+      <c r="D184" s="74" t="n">
+        <v>629</v>
+      </c>
+      <c r="E184" s="74" t="n">
+        <v>97.5</v>
+      </c>
+      <c r="F184" s="74">
+        <f>(D184-E184)/D184</f>
+        <v/>
+      </c>
+      <c r="G184" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #485 / 12-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="74" t="n">
+        <v>163</v>
+      </c>
+      <c r="B185" s="74" t="inlineStr">
+        <is>
+          <t>Molysheet (NARASHA OT Sheet)</t>
+        </is>
+      </c>
+      <c r="C185" s="74" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D185" s="74" t="n">
+        <v>155</v>
+      </c>
+      <c r="E185" s="74" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F185" s="74">
+        <f>(D185-E185)/D185</f>
+        <v/>
+      </c>
+      <c r="G185" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #467 / 08-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="74" t="n">
+        <v>164</v>
+      </c>
+      <c r="B186" s="74" t="inlineStr">
+        <is>
+          <t>Jelonet Tin (Paraffin Gauze — Tin)</t>
+        </is>
+      </c>
+      <c r="C186" s="74" t="inlineStr">
+        <is>
+          <t>Surgical Consumable</t>
+        </is>
+      </c>
+      <c r="D186" s="74" t="n">
+        <v>200.3</v>
+      </c>
+      <c r="E186" s="74" t="n">
+        <v>145</v>
+      </c>
+      <c r="F186" s="74">
+        <f>(D186-E186)/D186</f>
+        <v/>
+      </c>
+      <c r="G186" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #467 / 08-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="72" t="inlineStr">
         <is>
           <t>🔴 ITEMS MISSING MRP — Collect from vendor and update above</t>
         </is>
       </c>
-      <c r="B180" s="42" t="n"/>
-      <c r="C180" s="42" t="n"/>
-      <c r="D180" s="42" t="n"/>
-      <c r="E180" s="42" t="n"/>
-      <c r="F180" s="42" t="n"/>
-      <c r="G180" s="42" t="n"/>
-    </row>
-    <row r="181">
-      <c r="A181" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="B181" s="73" t="inlineStr">
-        <is>
-          <t>NS 100ml — Normal Saline 100ml</t>
-        </is>
-      </c>
-      <c r="C181" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D181" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E181" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F181" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G181" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" s="48" t="n">
-        <v>2</v>
-      </c>
-      <c r="B182" s="73" t="inlineStr">
-        <is>
-          <t>D5 500ml — Dextrose 5%</t>
-        </is>
-      </c>
-      <c r="C182" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D182" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E182" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F182" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G182" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" s="48" t="n">
-        <v>3</v>
-      </c>
-      <c r="B183" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
-        </is>
-      </c>
-      <c r="C183" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Anaesthesia</t>
-        </is>
-      </c>
-      <c r="D183" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E183" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F183" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G183" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="48" t="n">
-        <v>4</v>
-      </c>
-      <c r="B184" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Gentamicin</t>
-        </is>
-      </c>
-      <c r="C184" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D184" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E184" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F184" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G184" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" s="48" t="n">
-        <v>5</v>
-      </c>
-      <c r="B185" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Tramadol 50mg</t>
-        </is>
-      </c>
-      <c r="C185" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Analgesic</t>
-        </is>
-      </c>
-      <c r="D185" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E185" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F185" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G185" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="48" t="n">
-        <v>6</v>
-      </c>
-      <c r="B186" s="73" t="inlineStr">
-        <is>
-          <t>Inj. PCM 100ml (Paracetamol IV)</t>
-        </is>
-      </c>
-      <c r="C186" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Analgesic</t>
-        </is>
-      </c>
-      <c r="D186" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E186" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F186" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G186" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="48" t="n">
-        <v>7</v>
-      </c>
-      <c r="B187" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Carboprost (Hemabate)</t>
-        </is>
-      </c>
-      <c r="C187" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Oxytocic</t>
-        </is>
-      </c>
-      <c r="D187" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E187" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F187" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G187" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
+      <c r="B187" s="42" t="n"/>
+      <c r="C187" s="42" t="n"/>
+      <c r="D187" s="42" t="n"/>
+      <c r="E187" s="42" t="n"/>
+      <c r="F187" s="42" t="n"/>
+      <c r="G187" s="42" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="48" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="B188" s="73" t="inlineStr">
         <is>
-          <t>Inj. Adrenaline</t>
+          <t>NS 100ml — Normal Saline 100ml</t>
         </is>
       </c>
       <c r="C188" s="46" t="inlineStr">
         <is>
-          <t>Injection — Emergency</t>
-        </is>
-      </c>
-      <c r="D188" s="47" t="n">
-        <v>13.4</v>
+          <t>IV Fluid</t>
+        </is>
+      </c>
+      <c r="D188" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
       </c>
       <c r="E188" s="47" t="inlineStr">
         <is>
@@ -6002,27 +6009,27 @@
       </c>
       <c r="F188" s="47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⚠ FILL IN</t>
         </is>
       </c>
       <c r="G188" s="47" t="inlineStr">
         <is>
-          <t>Stock OT/Ward: ADRENALIN 1ML</t>
+          <t>⚠ FILL IN</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="48" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="B189" s="73" t="inlineStr">
         <is>
-          <t>Inj. Cetil (Cefuroxime Axetil)</t>
+          <t>D5 500ml — Dextrose 5%</t>
         </is>
       </c>
       <c r="C189" s="46" t="inlineStr">
         <is>
-          <t>Injection — Antibiotic</t>
+          <t>IV Fluid</t>
         </is>
       </c>
       <c r="D189" s="47" t="inlineStr">
@@ -6048,16 +6055,16 @@
     </row>
     <row r="190">
       <c r="A190" s="48" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="B190" s="73" t="inlineStr">
         <is>
-          <t>Needles 26G (Injection)</t>
+          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
         </is>
       </c>
       <c r="C190" s="46" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Injection — Anaesthesia</t>
         </is>
       </c>
       <c r="D190" s="47" t="inlineStr">
@@ -6083,16 +6090,16 @@
     </row>
     <row r="191">
       <c r="A191" s="48" t="n">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="B191" s="73" t="inlineStr">
         <is>
-          <t>Disposable Gloves (Exam)</t>
+          <t>Inj. Gentamicin</t>
         </is>
       </c>
       <c r="C191" s="46" t="inlineStr">
         <is>
-          <t>Surgical Consumable</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D191" s="47" t="inlineStr">
@@ -6118,16 +6125,16 @@
     </row>
     <row r="192">
       <c r="A192" s="48" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="B192" s="73" t="inlineStr">
         <is>
-          <t>Betadine Ointment 40g</t>
+          <t>Inj. Tramadol 50mg</t>
         </is>
       </c>
       <c r="C192" s="46" t="inlineStr">
         <is>
-          <t>Surgical Consumable</t>
+          <t>Injection — Analgesic</t>
         </is>
       </c>
       <c r="D192" s="47" t="inlineStr">
@@ -6153,16 +6160,16 @@
     </row>
     <row r="193">
       <c r="A193" s="48" t="n">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="B193" s="73" t="inlineStr">
         <is>
-          <t>Surgical Blade No. 10</t>
+          <t>Inj. PCM 100ml (Paracetamol IV)</t>
         </is>
       </c>
       <c r="C193" s="46" t="inlineStr">
         <is>
-          <t>Surgical Consumable</t>
+          <t>Injection — Analgesic</t>
         </is>
       </c>
       <c r="D193" s="47" t="inlineStr">
@@ -6188,16 +6195,16 @@
     </row>
     <row r="194">
       <c r="A194" s="48" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B194" s="73" t="inlineStr">
         <is>
-          <t>Surgical Blade No. 20</t>
+          <t>Inj. Carboprost (Hemabate)</t>
         </is>
       </c>
       <c r="C194" s="46" t="inlineStr">
         <is>
-          <t>Surgical Consumable</t>
+          <t>Injection — Oxytocic</t>
         </is>
       </c>
       <c r="D194" s="47" t="inlineStr">
@@ -6223,22 +6230,20 @@
     </row>
     <row r="195">
       <c r="A195" s="48" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="B195" s="73" t="inlineStr">
         <is>
-          <t>Plain Sheet (OT Draping)</t>
+          <t>Inj. Adrenaline</t>
         </is>
       </c>
       <c r="C195" s="46" t="inlineStr">
         <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D195" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
+          <t>Injection — Emergency</t>
+        </is>
+      </c>
+      <c r="D195" s="47" t="n">
+        <v>13.4</v>
       </c>
       <c r="E195" s="47" t="inlineStr">
         <is>
@@ -6247,27 +6252,27 @@
       </c>
       <c r="F195" s="47" t="inlineStr">
         <is>
-          <t>⚠ FILL IN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G195" s="47" t="inlineStr">
         <is>
-          <t>⚠ FILL IN</t>
+          <t>Stock OT/Ward: ADRENALIN 1ML</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="48" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="B196" s="73" t="inlineStr">
         <is>
-          <t>Soft Roll (OT Padding)</t>
+          <t>Inj. Cetil (Cefuroxime Axetil)</t>
         </is>
       </c>
       <c r="C196" s="46" t="inlineStr">
         <is>
-          <t>Surgical Consumable</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D196" s="47" t="inlineStr">
@@ -6293,16 +6298,16 @@
     </row>
     <row r="197">
       <c r="A197" s="48" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="B197" s="73" t="inlineStr">
         <is>
-          <t>Gypsona POP Bandage 40G</t>
+          <t>Needles 26G (Injection)</t>
         </is>
       </c>
       <c r="C197" s="46" t="inlineStr">
         <is>
-          <t>Surgical Consumable</t>
+          <t>Consumable</t>
         </is>
       </c>
       <c r="D197" s="47" t="inlineStr">
@@ -6328,11 +6333,11 @@
     </row>
     <row r="198">
       <c r="A198" s="48" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="B198" s="73" t="inlineStr">
         <is>
-          <t>Cap + Mask (Disposable Set)</t>
+          <t>Disposable Gloves (Exam)</t>
         </is>
       </c>
       <c r="C198" s="46" t="inlineStr">
@@ -6363,16 +6368,16 @@
     </row>
     <row r="199">
       <c r="A199" s="48" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="B199" s="73" t="inlineStr">
         <is>
-          <t>Glucostrip (Blood Glucose)</t>
+          <t>Betadine Ointment 40g</t>
         </is>
       </c>
       <c r="C199" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>Surgical Consumable</t>
         </is>
       </c>
       <c r="D199" s="47" t="inlineStr">
@@ -6398,16 +6403,16 @@
     </row>
     <row r="200">
       <c r="A200" s="48" t="n">
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="B200" s="73" t="inlineStr">
         <is>
-          <t>Lancet Needle</t>
+          <t>Surgical Blade No. 10</t>
         </is>
       </c>
       <c r="C200" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>Surgical Consumable</t>
         </is>
       </c>
       <c r="D200" s="47" t="inlineStr">
@@ -6433,16 +6438,16 @@
     </row>
     <row r="201">
       <c r="A201" s="48" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B201" s="73" t="inlineStr">
         <is>
-          <t>Red Top Tube (Blood Vial)</t>
+          <t>Surgical Blade No. 20</t>
         </is>
       </c>
       <c r="C201" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>Surgical Consumable</t>
         </is>
       </c>
       <c r="D201" s="47" t="inlineStr">
@@ -6468,16 +6473,16 @@
     </row>
     <row r="202">
       <c r="A202" s="48" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="B202" s="73" t="inlineStr">
         <is>
-          <t>CBC Vial Yellow + Red Top</t>
+          <t>Plain Sheet (OT Draping)</t>
         </is>
       </c>
       <c r="C202" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>Surgical Consumable</t>
         </is>
       </c>
       <c r="D202" s="47" t="inlineStr">
@@ -6503,16 +6508,16 @@
     </row>
     <row r="203">
       <c r="A203" s="48" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B203" s="73" t="inlineStr">
         <is>
-          <t>O2 / Oxygen (per use)</t>
+          <t>Soft Roll (OT Padding)</t>
         </is>
       </c>
       <c r="C203" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Surgical Consumable</t>
         </is>
       </c>
       <c r="D203" s="47" t="inlineStr">
@@ -6538,16 +6543,16 @@
     </row>
     <row r="204">
       <c r="A204" s="48" t="n">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B204" s="73" t="inlineStr">
         <is>
-          <t>Pulse Oximeter (per use)</t>
+          <t>Gypsona POP Bandage 40G</t>
         </is>
       </c>
       <c r="C204" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Surgical Consumable</t>
         </is>
       </c>
       <c r="D204" s="47" t="inlineStr">
@@ -6573,16 +6578,16 @@
     </row>
     <row r="205">
       <c r="A205" s="48" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="B205" s="73" t="inlineStr">
         <is>
-          <t>Cardiac Monitor (per use)</t>
+          <t>Cap + Mask (Disposable Set)</t>
         </is>
       </c>
       <c r="C205" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Surgical Consumable</t>
         </is>
       </c>
       <c r="D205" s="47" t="inlineStr">
@@ -6608,16 +6613,16 @@
     </row>
     <row r="206">
       <c r="A206" s="48" t="n">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="B206" s="73" t="inlineStr">
         <is>
-          <t>C-arm (per use)</t>
+          <t>Glucostrip (Blood Glucose)</t>
         </is>
       </c>
       <c r="C206" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Investigation</t>
         </is>
       </c>
       <c r="D206" s="47" t="inlineStr">
@@ -6643,34 +6648,279 @@
     </row>
     <row r="207">
       <c r="A207" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="B207" s="73" t="inlineStr">
+        <is>
+          <t>Lancet Needle</t>
+        </is>
+      </c>
+      <c r="C207" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D207" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E207" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F207" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G207" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="48" t="n">
+        <v>21</v>
+      </c>
+      <c r="B208" s="73" t="inlineStr">
+        <is>
+          <t>Red Top Tube (Blood Vial)</t>
+        </is>
+      </c>
+      <c r="C208" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D208" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E208" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F208" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G208" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="48" t="n">
+        <v>22</v>
+      </c>
+      <c r="B209" s="73" t="inlineStr">
+        <is>
+          <t>CBC Vial Yellow + Red Top</t>
+        </is>
+      </c>
+      <c r="C209" s="46" t="inlineStr">
+        <is>
+          <t>Investigation</t>
+        </is>
+      </c>
+      <c r="D209" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E209" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F209" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G209" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="48" t="n">
+        <v>23</v>
+      </c>
+      <c r="B210" s="73" t="inlineStr">
+        <is>
+          <t>O2 / Oxygen (per use)</t>
+        </is>
+      </c>
+      <c r="C210" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D210" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E210" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F210" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G210" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="48" t="n">
+        <v>24</v>
+      </c>
+      <c r="B211" s="73" t="inlineStr">
+        <is>
+          <t>Pulse Oximeter (per use)</t>
+        </is>
+      </c>
+      <c r="C211" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D211" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E211" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F211" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G211" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="48" t="n">
+        <v>25</v>
+      </c>
+      <c r="B212" s="73" t="inlineStr">
+        <is>
+          <t>Cardiac Monitor (per use)</t>
+        </is>
+      </c>
+      <c r="C212" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D212" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E212" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F212" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G212" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="48" t="n">
+        <v>26</v>
+      </c>
+      <c r="B213" s="73" t="inlineStr">
+        <is>
+          <t>C-arm (per use)</t>
+        </is>
+      </c>
+      <c r="C213" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D213" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E213" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F213" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G213" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="48" t="n">
         <v>27</v>
       </c>
-      <c r="B207" s="73" t="inlineStr">
+      <c r="B214" s="73" t="inlineStr">
         <is>
           <t>Volu-P / TiCUP</t>
         </is>
       </c>
-      <c r="C207" s="46" t="inlineStr">
+      <c r="C214" s="46" t="inlineStr">
         <is>
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D207" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E207" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F207" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G207" s="47" t="inlineStr">
+      <c r="D214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G214" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL IN</t>
         </is>

</xml_diff>

<commit_message>
Fix Alburel MRP; add Klotin 5ML (SL165); add MR000969
- SL159 Alburel 20% IV: MRP corrected to ₹10724 (Cost ₹4650)
- SL165 Klotin 5ML INJ (Clonazepam): MRP ₹73.10, Cost ₹30 — new item
- MR000969 (07-Aug-26): Rantac 2ML + Klotin 5ML → ₹376 added to summary & line items

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -765,7 +765,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G214"/>
+  <dimension ref="A1:G215"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="36" min="1" max="1"/>
@@ -5801,18 +5801,15 @@
           <t>Injection — IV</t>
         </is>
       </c>
-      <c r="D181" s="75" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="D181" s="75" t="n">
+        <v>10724</v>
       </c>
       <c r="E181" s="75" t="n">
         <v>4650</v>
       </c>
-      <c r="F181" s="75" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
+      <c r="F181" s="75">
+        <f>(D181-E181)/D181</f>
+        <v/>
       </c>
       <c r="G181" s="75" t="inlineStr">
         <is>
@@ -5971,60 +5968,55 @@
       </c>
     </row>
     <row r="187">
-      <c r="A187" s="72" t="inlineStr">
+      <c r="A187" s="74" t="n">
+        <v>165</v>
+      </c>
+      <c r="B187" s="74" t="inlineStr">
+        <is>
+          <t>Klotin 5ML INJ (Clonazepam)</t>
+        </is>
+      </c>
+      <c r="C187" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Neuro/Sedative</t>
+        </is>
+      </c>
+      <c r="D187" s="74" t="n">
+        <v>73.09999999999999</v>
+      </c>
+      <c r="E187" s="74" t="n">
+        <v>30</v>
+      </c>
+      <c r="F187" s="74">
+        <f>(D187-E187)/D187</f>
+        <v/>
+      </c>
+      <c r="G187" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR000969 / 07-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="72" t="inlineStr">
         <is>
           <t>🔴 ITEMS MISSING MRP — Collect from vendor and update above</t>
         </is>
       </c>
-      <c r="B187" s="42" t="n"/>
-      <c r="C187" s="42" t="n"/>
-      <c r="D187" s="42" t="n"/>
-      <c r="E187" s="42" t="n"/>
-      <c r="F187" s="42" t="n"/>
-      <c r="G187" s="42" t="n"/>
-    </row>
-    <row r="188">
-      <c r="A188" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="B188" s="73" t="inlineStr">
-        <is>
-          <t>NS 100ml — Normal Saline 100ml</t>
-        </is>
-      </c>
-      <c r="C188" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G188" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
+      <c r="B188" s="42" t="n"/>
+      <c r="C188" s="42" t="n"/>
+      <c r="D188" s="42" t="n"/>
+      <c r="E188" s="42" t="n"/>
+      <c r="F188" s="42" t="n"/>
+      <c r="G188" s="42" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="48" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="B189" s="73" t="inlineStr">
         <is>
-          <t>D5 500ml — Dextrose 5%</t>
+          <t>NS 100ml — Normal Saline 100ml</t>
         </is>
       </c>
       <c r="C189" s="46" t="inlineStr">
@@ -6055,16 +6047,16 @@
     </row>
     <row r="190">
       <c r="A190" s="48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B190" s="73" t="inlineStr">
         <is>
-          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
+          <t>D5 500ml — Dextrose 5%</t>
         </is>
       </c>
       <c r="C190" s="46" t="inlineStr">
         <is>
-          <t>Injection — Anaesthesia</t>
+          <t>IV Fluid</t>
         </is>
       </c>
       <c r="D190" s="47" t="inlineStr">
@@ -6090,16 +6082,16 @@
     </row>
     <row r="191">
       <c r="A191" s="48" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B191" s="73" t="inlineStr">
         <is>
-          <t>Inj. Gentamicin</t>
+          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
         </is>
       </c>
       <c r="C191" s="46" t="inlineStr">
         <is>
-          <t>Injection — Antibiotic</t>
+          <t>Injection — Anaesthesia</t>
         </is>
       </c>
       <c r="D191" s="47" t="inlineStr">
@@ -6125,16 +6117,16 @@
     </row>
     <row r="192">
       <c r="A192" s="48" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B192" s="73" t="inlineStr">
         <is>
-          <t>Inj. Tramadol 50mg</t>
+          <t>Inj. Gentamicin</t>
         </is>
       </c>
       <c r="C192" s="46" t="inlineStr">
         <is>
-          <t>Injection — Analgesic</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D192" s="47" t="inlineStr">
@@ -6160,11 +6152,11 @@
     </row>
     <row r="193">
       <c r="A193" s="48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B193" s="73" t="inlineStr">
         <is>
-          <t>Inj. PCM 100ml (Paracetamol IV)</t>
+          <t>Inj. Tramadol 50mg</t>
         </is>
       </c>
       <c r="C193" s="46" t="inlineStr">
@@ -6195,16 +6187,16 @@
     </row>
     <row r="194">
       <c r="A194" s="48" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B194" s="73" t="inlineStr">
         <is>
-          <t>Inj. Carboprost (Hemabate)</t>
+          <t>Inj. PCM 100ml (Paracetamol IV)</t>
         </is>
       </c>
       <c r="C194" s="46" t="inlineStr">
         <is>
-          <t>Injection — Oxytocic</t>
+          <t>Injection — Analgesic</t>
         </is>
       </c>
       <c r="D194" s="47" t="inlineStr">
@@ -6230,20 +6222,22 @@
     </row>
     <row r="195">
       <c r="A195" s="48" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B195" s="73" t="inlineStr">
         <is>
-          <t>Inj. Adrenaline</t>
+          <t>Inj. Carboprost (Hemabate)</t>
         </is>
       </c>
       <c r="C195" s="46" t="inlineStr">
         <is>
-          <t>Injection — Emergency</t>
-        </is>
-      </c>
-      <c r="D195" s="47" t="n">
-        <v>13.4</v>
+          <t>Injection — Oxytocic</t>
+        </is>
+      </c>
+      <c r="D195" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
       </c>
       <c r="E195" s="47" t="inlineStr">
         <is>
@@ -6252,33 +6246,31 @@
       </c>
       <c r="F195" s="47" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>⚠ FILL IN</t>
         </is>
       </c>
       <c r="G195" s="47" t="inlineStr">
         <is>
-          <t>Stock OT/Ward: ADRENALIN 1ML</t>
+          <t>⚠ FILL IN</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" s="48" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B196" s="73" t="inlineStr">
         <is>
-          <t>Inj. Cetil (Cefuroxime Axetil)</t>
+          <t>Inj. Adrenaline</t>
         </is>
       </c>
       <c r="C196" s="46" t="inlineStr">
         <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D196" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
+          <t>Injection — Emergency</t>
+        </is>
+      </c>
+      <c r="D196" s="47" t="n">
+        <v>13.4</v>
       </c>
       <c r="E196" s="47" t="inlineStr">
         <is>
@@ -6287,27 +6279,27 @@
       </c>
       <c r="F196" s="47" t="inlineStr">
         <is>
-          <t>⚠ FILL IN</t>
+          <t>—</t>
         </is>
       </c>
       <c r="G196" s="47" t="inlineStr">
         <is>
-          <t>⚠ FILL IN</t>
+          <t>Stock OT/Ward: ADRENALIN 1ML</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" s="48" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B197" s="73" t="inlineStr">
         <is>
-          <t>Needles 26G (Injection)</t>
+          <t>Inj. Cetil (Cefuroxime Axetil)</t>
         </is>
       </c>
       <c r="C197" s="46" t="inlineStr">
         <is>
-          <t>Consumable</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D197" s="47" t="inlineStr">
@@ -6333,16 +6325,16 @@
     </row>
     <row r="198">
       <c r="A198" s="48" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B198" s="73" t="inlineStr">
         <is>
-          <t>Disposable Gloves (Exam)</t>
+          <t>Needles 26G (Injection)</t>
         </is>
       </c>
       <c r="C198" s="46" t="inlineStr">
         <is>
-          <t>Surgical Consumable</t>
+          <t>Consumable</t>
         </is>
       </c>
       <c r="D198" s="47" t="inlineStr">
@@ -6368,11 +6360,11 @@
     </row>
     <row r="199">
       <c r="A199" s="48" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B199" s="73" t="inlineStr">
         <is>
-          <t>Betadine Ointment 40g</t>
+          <t>Disposable Gloves (Exam)</t>
         </is>
       </c>
       <c r="C199" s="46" t="inlineStr">
@@ -6403,11 +6395,11 @@
     </row>
     <row r="200">
       <c r="A200" s="48" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B200" s="73" t="inlineStr">
         <is>
-          <t>Surgical Blade No. 10</t>
+          <t>Betadine Ointment 40g</t>
         </is>
       </c>
       <c r="C200" s="46" t="inlineStr">
@@ -6438,11 +6430,11 @@
     </row>
     <row r="201">
       <c r="A201" s="48" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B201" s="73" t="inlineStr">
         <is>
-          <t>Surgical Blade No. 20</t>
+          <t>Surgical Blade No. 10</t>
         </is>
       </c>
       <c r="C201" s="46" t="inlineStr">
@@ -6473,11 +6465,11 @@
     </row>
     <row r="202">
       <c r="A202" s="48" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B202" s="73" t="inlineStr">
         <is>
-          <t>Plain Sheet (OT Draping)</t>
+          <t>Surgical Blade No. 20</t>
         </is>
       </c>
       <c r="C202" s="46" t="inlineStr">
@@ -6508,11 +6500,11 @@
     </row>
     <row r="203">
       <c r="A203" s="48" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B203" s="73" t="inlineStr">
         <is>
-          <t>Soft Roll (OT Padding)</t>
+          <t>Plain Sheet (OT Draping)</t>
         </is>
       </c>
       <c r="C203" s="46" t="inlineStr">
@@ -6543,11 +6535,11 @@
     </row>
     <row r="204">
       <c r="A204" s="48" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B204" s="73" t="inlineStr">
         <is>
-          <t>Gypsona POP Bandage 40G</t>
+          <t>Soft Roll (OT Padding)</t>
         </is>
       </c>
       <c r="C204" s="46" t="inlineStr">
@@ -6578,11 +6570,11 @@
     </row>
     <row r="205">
       <c r="A205" s="48" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B205" s="73" t="inlineStr">
         <is>
-          <t>Cap + Mask (Disposable Set)</t>
+          <t>Gypsona POP Bandage 40G</t>
         </is>
       </c>
       <c r="C205" s="46" t="inlineStr">
@@ -6613,16 +6605,16 @@
     </row>
     <row r="206">
       <c r="A206" s="48" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B206" s="73" t="inlineStr">
         <is>
-          <t>Glucostrip (Blood Glucose)</t>
+          <t>Cap + Mask (Disposable Set)</t>
         </is>
       </c>
       <c r="C206" s="46" t="inlineStr">
         <is>
-          <t>Investigation</t>
+          <t>Surgical Consumable</t>
         </is>
       </c>
       <c r="D206" s="47" t="inlineStr">
@@ -6648,11 +6640,11 @@
     </row>
     <row r="207">
       <c r="A207" s="48" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B207" s="73" t="inlineStr">
         <is>
-          <t>Lancet Needle</t>
+          <t>Glucostrip (Blood Glucose)</t>
         </is>
       </c>
       <c r="C207" s="46" t="inlineStr">
@@ -6683,11 +6675,11 @@
     </row>
     <row r="208">
       <c r="A208" s="48" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B208" s="73" t="inlineStr">
         <is>
-          <t>Red Top Tube (Blood Vial)</t>
+          <t>Lancet Needle</t>
         </is>
       </c>
       <c r="C208" s="46" t="inlineStr">
@@ -6718,11 +6710,11 @@
     </row>
     <row r="209">
       <c r="A209" s="48" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B209" s="73" t="inlineStr">
         <is>
-          <t>CBC Vial Yellow + Red Top</t>
+          <t>Red Top Tube (Blood Vial)</t>
         </is>
       </c>
       <c r="C209" s="46" t="inlineStr">
@@ -6753,16 +6745,16 @@
     </row>
     <row r="210">
       <c r="A210" s="48" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B210" s="73" t="inlineStr">
         <is>
-          <t>O2 / Oxygen (per use)</t>
+          <t>CBC Vial Yellow + Red Top</t>
         </is>
       </c>
       <c r="C210" s="46" t="inlineStr">
         <is>
-          <t>Equipment</t>
+          <t>Investigation</t>
         </is>
       </c>
       <c r="D210" s="47" t="inlineStr">
@@ -6788,11 +6780,11 @@
     </row>
     <row r="211">
       <c r="A211" s="48" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B211" s="73" t="inlineStr">
         <is>
-          <t>Pulse Oximeter (per use)</t>
+          <t>O2 / Oxygen (per use)</t>
         </is>
       </c>
       <c r="C211" s="46" t="inlineStr">
@@ -6823,11 +6815,11 @@
     </row>
     <row r="212">
       <c r="A212" s="48" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B212" s="73" t="inlineStr">
         <is>
-          <t>Cardiac Monitor (per use)</t>
+          <t>Pulse Oximeter (per use)</t>
         </is>
       </c>
       <c r="C212" s="46" t="inlineStr">
@@ -6858,11 +6850,11 @@
     </row>
     <row r="213">
       <c r="A213" s="48" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B213" s="73" t="inlineStr">
         <is>
-          <t>C-arm (per use)</t>
+          <t>Cardiac Monitor (per use)</t>
         </is>
       </c>
       <c r="C213" s="46" t="inlineStr">
@@ -6893,34 +6885,69 @@
     </row>
     <row r="214">
       <c r="A214" s="48" t="n">
+        <v>26</v>
+      </c>
+      <c r="B214" s="73" t="inlineStr">
+        <is>
+          <t>C-arm (per use)</t>
+        </is>
+      </c>
+      <c r="C214" s="46" t="inlineStr">
+        <is>
+          <t>Equipment</t>
+        </is>
+      </c>
+      <c r="D214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G214" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="48" t="n">
         <v>27</v>
       </c>
-      <c r="B214" s="73" t="inlineStr">
+      <c r="B215" s="73" t="inlineStr">
         <is>
           <t>Volu-P / TiCUP</t>
         </is>
       </c>
-      <c r="C214" s="46" t="inlineStr">
+      <c r="C215" s="46" t="inlineStr">
         <is>
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D214" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E214" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F214" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G214" s="47" t="inlineStr">
+      <c r="D215" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E215" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F215" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G215" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL IN</t>
         </is>

</xml_diff>

<commit_message>
Add final invoices BP526/531/533/545/548 MR001168 Chirag MP-38; update rate card SL166-SL217
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0%"/>
+  </numFmts>
   <fonts count="14">
     <font>
       <name val="Calibri"/>
@@ -287,7 +289,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="77">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -510,6 +512,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -765,7 +770,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G215"/>
+  <dimension ref="A1:G267"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="36" min="1" max="1"/>
@@ -4183,7 +4188,6 @@
         </is>
       </c>
     </row>
-    <row r="121"/>
     <row r="122" ht="13.5" customHeight="1" s="37">
       <c r="A122" s="36" t="n">
         <v>100</v>
@@ -5998,956 +6002,2516 @@
       </c>
     </row>
     <row r="188">
-      <c r="A188" s="72" t="inlineStr">
+      <c r="A188" s="74" t="n">
+        <v>166</v>
+      </c>
+      <c r="B188" s="74" t="inlineStr">
+        <is>
+          <t>NS 3000ML IV Bag (KRPL)</t>
+        </is>
+      </c>
+      <c r="C188" s="74" t="inlineStr">
+        <is>
+          <t>IV Fluid</t>
+        </is>
+      </c>
+      <c r="D188" s="74" t="n">
+        <v>698</v>
+      </c>
+      <c r="E188" s="74" t="n">
+        <v>123</v>
+      </c>
+      <c r="F188" s="76">
+        <f>(D188-E188)/D188</f>
+        <v/>
+      </c>
+      <c r="G188" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #493 / 17-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="74" t="n">
+        <v>167</v>
+      </c>
+      <c r="B189" s="74" t="inlineStr">
+        <is>
+          <t>Hydrogen Peroxide Solution 45</t>
+        </is>
+      </c>
+      <c r="C189" s="74" t="inlineStr">
+        <is>
+          <t>Antiseptic/Disinfectant</t>
+        </is>
+      </c>
+      <c r="D189" s="74" t="n">
+        <v>83</v>
+      </c>
+      <c r="E189" s="74" t="n">
+        <v>38.5</v>
+      </c>
+      <c r="F189" s="76">
+        <f>(D189-E189)/D189</f>
+        <v/>
+      </c>
+      <c r="G189" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #493 / 17-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="74" t="n">
+        <v>168</v>
+      </c>
+      <c r="B190" s="74" t="inlineStr">
+        <is>
+          <t>Spinocan-25 Spinal Needle</t>
+        </is>
+      </c>
+      <c r="C190" s="74" t="inlineStr">
+        <is>
+          <t>Anaesthesia Consumable</t>
+        </is>
+      </c>
+      <c r="D190" s="74" t="n">
+        <v>143.44</v>
+      </c>
+      <c r="E190" s="74" t="n">
+        <v>80.75</v>
+      </c>
+      <c r="F190" s="76">
+        <f>(D190-E190)/D190</f>
+        <v/>
+      </c>
+      <c r="G190" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #493 / 17-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="74" t="n">
+        <v>169</v>
+      </c>
+      <c r="B191" s="74" t="inlineStr">
+        <is>
+          <t>Full Body OT Gown (NAERLZM)</t>
+        </is>
+      </c>
+      <c r="C191" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Protective</t>
+        </is>
+      </c>
+      <c r="D191" s="74" t="n">
+        <v>426</v>
+      </c>
+      <c r="E191" s="74" t="n">
+        <v>261.25</v>
+      </c>
+      <c r="F191" s="76">
+        <f>(D191-E191)/D191</f>
+        <v/>
+      </c>
+      <c r="G191" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #493 / 17-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="74" t="n">
+        <v>170</v>
+      </c>
+      <c r="B192" s="74" t="inlineStr">
+        <is>
+          <t>Cloth Drape CD01</t>
+        </is>
+      </c>
+      <c r="C192" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Drape</t>
+        </is>
+      </c>
+      <c r="D192" s="74" t="n">
+        <v>62</v>
+      </c>
+      <c r="E192" s="74" t="n">
+        <v>43.33</v>
+      </c>
+      <c r="F192" s="76">
+        <f>(D192-E192)/D192</f>
+        <v/>
+      </c>
+      <c r="G192" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #493 / 17-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="74" t="n">
+        <v>171</v>
+      </c>
+      <c r="B193" s="74" t="inlineStr">
+        <is>
+          <t>OT X-Ray Gauze</t>
+        </is>
+      </c>
+      <c r="C193" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Gauze</t>
+        </is>
+      </c>
+      <c r="D193" s="74" t="n">
+        <v>51.56</v>
+      </c>
+      <c r="E193" s="74" t="n">
+        <v>24.55</v>
+      </c>
+      <c r="F193" s="76">
+        <f>(D193-E193)/D193</f>
+        <v/>
+      </c>
+      <c r="G193" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #493 / 17-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="74" t="n">
+        <v>172</v>
+      </c>
+      <c r="B194" s="74" t="inlineStr">
+        <is>
+          <t>Ondem 4ML INJ (Ondansetron)</t>
+        </is>
+      </c>
+      <c r="C194" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antiemetic</t>
+        </is>
+      </c>
+      <c r="D194" s="74" t="n">
+        <v>25.45</v>
+      </c>
+      <c r="E194" s="74" t="n">
+        <v>10</v>
+      </c>
+      <c r="F194" s="76">
+        <f>(D194-E194)/D194</f>
+        <v/>
+      </c>
+      <c r="G194" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001046 / 18-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="74" t="n">
+        <v>173</v>
+      </c>
+      <c r="B195" s="74" t="inlineStr">
+        <is>
+          <t>PAN IV 40MG (Pantoprazole IV)</t>
+        </is>
+      </c>
+      <c r="C195" s="74" t="inlineStr">
+        <is>
+          <t>Injection — PPI</t>
+        </is>
+      </c>
+      <c r="D195" s="74" t="n">
+        <v>54.24</v>
+      </c>
+      <c r="E195" s="74" t="n">
+        <v>18</v>
+      </c>
+      <c r="F195" s="76">
+        <f>(D195-E195)/D195</f>
+        <v/>
+      </c>
+      <c r="G195" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001046 / 18-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="74" t="n">
+        <v>174</v>
+      </c>
+      <c r="B196" s="74" t="inlineStr">
+        <is>
+          <t>Nllg-Mycin INJ (Gentamicin)</t>
+        </is>
+      </c>
+      <c r="C196" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D196" s="74" t="n">
+        <v>9.84</v>
+      </c>
+      <c r="E196" s="74" t="n">
+        <v>5.87</v>
+      </c>
+      <c r="F196" s="76">
+        <f>(D196-E196)/D196</f>
+        <v/>
+      </c>
+      <c r="G196" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001046 / 18-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="74" t="n">
+        <v>175</v>
+      </c>
+      <c r="B197" s="74" t="inlineStr">
+        <is>
+          <t>Diathermy Pencil (RM)</t>
+        </is>
+      </c>
+      <c r="C197" s="74" t="inlineStr">
+        <is>
+          <t>OT Equipment — Diathermy</t>
+        </is>
+      </c>
+      <c r="D197" s="74" t="n">
+        <v>917</v>
+      </c>
+      <c r="E197" s="74" t="n">
+        <v>121.12</v>
+      </c>
+      <c r="F197" s="76">
+        <f>(D197-E197)/D197</f>
+        <v/>
+      </c>
+      <c r="G197" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="74" t="n">
+        <v>176</v>
+      </c>
+      <c r="B198" s="74" t="inlineStr">
+        <is>
+          <t>Vaccu Suction Set (A)</t>
+        </is>
+      </c>
+      <c r="C198" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Suction</t>
+        </is>
+      </c>
+      <c r="D198" s="74" t="n">
+        <v>609</v>
+      </c>
+      <c r="E198" s="74" t="n">
+        <v>64</v>
+      </c>
+      <c r="F198" s="76">
+        <f>(D198-E198)/D198</f>
+        <v/>
+      </c>
+      <c r="G198" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="74" t="n">
+        <v>177</v>
+      </c>
+      <c r="B199" s="74" t="inlineStr">
+        <is>
+          <t>Roll Bandage 4" (LC)</t>
+        </is>
+      </c>
+      <c r="C199" s="74" t="inlineStr">
+        <is>
+          <t>Dressing &amp; Bandage</t>
+        </is>
+      </c>
+      <c r="D199" s="74" t="n">
+        <v>120</v>
+      </c>
+      <c r="E199" s="74" t="n">
+        <v>58</v>
+      </c>
+      <c r="F199" s="76">
+        <f>(D199-E199)/D199</f>
+        <v/>
+      </c>
+      <c r="G199" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="74" t="n">
+        <v>178</v>
+      </c>
+      <c r="B200" s="74" t="inlineStr">
+        <is>
+          <t>Roll Bandage 6" (LC)</t>
+        </is>
+      </c>
+      <c r="C200" s="74" t="inlineStr">
+        <is>
+          <t>Dressing &amp; Bandage</t>
+        </is>
+      </c>
+      <c r="D200" s="74" t="n">
+        <v>124</v>
+      </c>
+      <c r="E200" s="74" t="n">
+        <v>78</v>
+      </c>
+      <c r="F200" s="76">
+        <f>(D200-E200)/D200</f>
+        <v/>
+      </c>
+      <c r="G200" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="74" t="n">
+        <v>179</v>
+      </c>
+      <c r="B201" s="74" t="inlineStr">
+        <is>
+          <t>Urobag (ROND-10)</t>
+        </is>
+      </c>
+      <c r="C201" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D201" s="74" t="n">
+        <v>361</v>
+      </c>
+      <c r="E201" s="74" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="F201" s="76">
+        <f>(D201-E201)/D201</f>
+        <v/>
+      </c>
+      <c r="G201" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="74" t="n">
+        <v>180</v>
+      </c>
+      <c r="B202" s="74" t="inlineStr">
+        <is>
+          <t>Camera Cover (D904)</t>
+        </is>
+      </c>
+      <c r="C202" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Laparoscopy</t>
+        </is>
+      </c>
+      <c r="D202" s="74" t="n">
+        <v>237</v>
+      </c>
+      <c r="E202" s="74" t="n">
+        <v>169</v>
+      </c>
+      <c r="F202" s="76">
+        <f>(D202-E202)/D202</f>
+        <v/>
+      </c>
+      <c r="G202" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="74" t="n">
+        <v>181</v>
+      </c>
+      <c r="B203" s="74" t="inlineStr">
+        <is>
+          <t>Nasal Cannula (AIRWA)</t>
+        </is>
+      </c>
+      <c r="C203" s="74" t="inlineStr">
+        <is>
+          <t>Respiratory Consumable</t>
+        </is>
+      </c>
+      <c r="D203" s="74" t="n">
+        <v>363</v>
+      </c>
+      <c r="E203" s="74" t="n">
+        <v>18.62</v>
+      </c>
+      <c r="F203" s="76">
+        <f>(D203-E203)/D203</f>
+        <v/>
+      </c>
+      <c r="G203" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="74" t="n">
+        <v>182</v>
+      </c>
+      <c r="B204" s="74" t="inlineStr">
+        <is>
+          <t>Genellium Pro (Pink 5)</t>
+        </is>
+      </c>
+      <c r="C204" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Haemostat</t>
+        </is>
+      </c>
+      <c r="D204" s="74" t="n">
+        <v>2750</v>
+      </c>
+      <c r="E204" s="74" t="n">
+        <v>810</v>
+      </c>
+      <c r="F204" s="76">
+        <f>(D204-E204)/D204</f>
+        <v/>
+      </c>
+      <c r="G204" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="74" t="n">
+        <v>183</v>
+      </c>
+      <c r="B205" s="74" t="inlineStr">
+        <is>
+          <t>Foley's Catheter 3-Way 22Fr</t>
+        </is>
+      </c>
+      <c r="C205" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D205" s="74" t="n">
+        <v>491</v>
+      </c>
+      <c r="E205" s="74" t="n">
+        <v>353.75</v>
+      </c>
+      <c r="F205" s="76">
+        <f>(D205-E205)/D205</f>
+        <v/>
+      </c>
+      <c r="G205" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="74" t="n">
+        <v>184</v>
+      </c>
+      <c r="B206" s="74" t="inlineStr">
+        <is>
+          <t>Foley's Catheter 3-Way 18Fr</t>
+        </is>
+      </c>
+      <c r="C206" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D206" s="74" t="n">
+        <v>460</v>
+      </c>
+      <c r="E206" s="74" t="n">
+        <v>353.75</v>
+      </c>
+      <c r="F206" s="76">
+        <f>(D206-E206)/D206</f>
+        <v/>
+      </c>
+      <c r="G206" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="74" t="n">
+        <v>185</v>
+      </c>
+      <c r="B207" s="74" t="inlineStr">
+        <is>
+          <t>Foley's Catheter 3-Way 24Fr</t>
+        </is>
+      </c>
+      <c r="C207" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D207" s="74" t="n">
+        <v>448</v>
+      </c>
+      <c r="E207" s="74" t="n">
+        <v>353.75</v>
+      </c>
+      <c r="F207" s="76">
+        <f>(D207-E207)/D207</f>
+        <v/>
+      </c>
+      <c r="G207" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="74" t="n">
+        <v>186</v>
+      </c>
+      <c r="B208" s="74" t="inlineStr">
+        <is>
+          <t>Foley's Catheter 2-Way 16Fr</t>
+        </is>
+      </c>
+      <c r="C208" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D208" s="74" t="n">
+        <v>191</v>
+      </c>
+      <c r="E208" s="74" t="n">
+        <v>131.45</v>
+      </c>
+      <c r="F208" s="76">
+        <f>(D208-E208)/D208</f>
+        <v/>
+      </c>
+      <c r="G208" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="74" t="n">
+        <v>187</v>
+      </c>
+      <c r="B209" s="74" t="inlineStr">
+        <is>
+          <t>Foley's Catheter 2-Way 20Fr</t>
+        </is>
+      </c>
+      <c r="C209" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D209" s="74" t="n">
+        <v>174</v>
+      </c>
+      <c r="E209" s="74" t="n">
+        <v>131.45</v>
+      </c>
+      <c r="F209" s="76">
+        <f>(D209-E209)/D209</f>
+        <v/>
+      </c>
+      <c r="G209" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="74" t="n">
+        <v>188</v>
+      </c>
+      <c r="B210" s="74" t="inlineStr">
+        <is>
+          <t>Foley's Catheter 2-Way 22Fr</t>
+        </is>
+      </c>
+      <c r="C210" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D210" s="74" t="n">
+        <v>163.13</v>
+      </c>
+      <c r="E210" s="74" t="n">
+        <v>131.45</v>
+      </c>
+      <c r="F210" s="76">
+        <f>(D210-E210)/D210</f>
+        <v/>
+      </c>
+      <c r="G210" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="74" t="n">
+        <v>189</v>
+      </c>
+      <c r="B211" s="74" t="inlineStr">
+        <is>
+          <t>RL 500ML Flat Cap</t>
+        </is>
+      </c>
+      <c r="C211" s="74" t="inlineStr">
+        <is>
+          <t>IV Fluid</t>
+        </is>
+      </c>
+      <c r="D211" s="74" t="n">
+        <v>60.74</v>
+      </c>
+      <c r="E211" s="74" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="F211" s="76">
+        <f>(D211-E211)/D211</f>
+        <v/>
+      </c>
+      <c r="G211" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #513 / 20-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="74" t="n">
+        <v>190</v>
+      </c>
+      <c r="B212" s="74" t="inlineStr">
+        <is>
+          <t>Weardn Disposable Apron</t>
+        </is>
+      </c>
+      <c r="C212" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Protective</t>
+        </is>
+      </c>
+      <c r="D212" s="74" t="n">
+        <v>672</v>
+      </c>
+      <c r="E212" s="74" t="n">
+        <v>186.5</v>
+      </c>
+      <c r="F212" s="76">
+        <f>(D212-E212)/D212</f>
+        <v/>
+      </c>
+      <c r="G212" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #513 / 20-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="74" t="n">
+        <v>191</v>
+      </c>
+      <c r="B213" s="74" t="inlineStr">
+        <is>
+          <t>Adult Diaper (Large) RAM</t>
+        </is>
+      </c>
+      <c r="C213" s="74" t="inlineStr">
+        <is>
+          <t>Ward Consumable</t>
+        </is>
+      </c>
+      <c r="D213" s="74" t="n">
+        <v>120</v>
+      </c>
+      <c r="E213" s="74" t="n">
+        <v>25</v>
+      </c>
+      <c r="F213" s="76">
+        <f>(D213-E213)/D213</f>
+        <v/>
+      </c>
+      <c r="G213" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #513 / 20-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="74" t="n">
+        <v>192</v>
+      </c>
+      <c r="B214" s="74" t="inlineStr">
+        <is>
+          <t>Betadine Scrub 500ML</t>
+        </is>
+      </c>
+      <c r="C214" s="74" t="inlineStr">
+        <is>
+          <t>Antiseptic/Disinfectant</t>
+        </is>
+      </c>
+      <c r="D214" s="74" t="n">
+        <v>1071</v>
+      </c>
+      <c r="E214" s="74" t="n">
+        <v>928</v>
+      </c>
+      <c r="F214" s="76">
+        <f>(D214-E214)/D214</f>
+        <v/>
+      </c>
+      <c r="G214" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #526 / 24-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="74" t="n">
+        <v>193</v>
+      </c>
+      <c r="B215" s="74" t="inlineStr">
+        <is>
+          <t>Dispovan 10ML Syringe (ROMOJE)</t>
+        </is>
+      </c>
+      <c r="C215" s="74" t="inlineStr">
+        <is>
+          <t>Syringe &amp; Needle</t>
+        </is>
+      </c>
+      <c r="D215" s="74" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="E215" s="74" t="n">
+        <v>4.55</v>
+      </c>
+      <c r="F215" s="76">
+        <f>(D215-E215)/D215</f>
+        <v/>
+      </c>
+      <c r="G215" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #531 / 25-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" s="74" t="n">
+        <v>194</v>
+      </c>
+      <c r="B216" s="74" t="inlineStr">
+        <is>
+          <t>E Coli Cath L4</t>
+        </is>
+      </c>
+      <c r="C216" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D216" s="74" t="n">
+        <v>120</v>
+      </c>
+      <c r="E216" s="74" t="n">
+        <v>16.6</v>
+      </c>
+      <c r="F216" s="76">
+        <f>(D216-E216)/D216</f>
+        <v/>
+      </c>
+      <c r="G216" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #531 / 25-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="74" t="n">
+        <v>195</v>
+      </c>
+      <c r="B217" s="74" t="inlineStr">
+        <is>
+          <t>Vein O Line-10 CM</t>
+        </is>
+      </c>
+      <c r="C217" s="74" t="inlineStr">
+        <is>
+          <t>IV Consumable</t>
+        </is>
+      </c>
+      <c r="D217" s="74" t="n">
+        <v>386</v>
+      </c>
+      <c r="E217" s="74" t="n">
+        <v>31.15</v>
+      </c>
+      <c r="F217" s="76">
+        <f>(D217-E217)/D217</f>
+        <v/>
+      </c>
+      <c r="G217" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #531 / 25-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="74" t="n">
+        <v>196</v>
+      </c>
+      <c r="B218" s="74" t="inlineStr">
+        <is>
+          <t>I.V. Set (RON)</t>
+        </is>
+      </c>
+      <c r="C218" s="74" t="inlineStr">
+        <is>
+          <t>IV Consumable</t>
+        </is>
+      </c>
+      <c r="D218" s="74" t="n">
+        <v>201</v>
+      </c>
+      <c r="E218" s="74" t="n">
+        <v>14.06</v>
+      </c>
+      <c r="F218" s="76">
+        <f>(D218-E218)/D218</f>
+        <v/>
+      </c>
+      <c r="G218" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #531 / 25-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="74" t="n">
+        <v>197</v>
+      </c>
+      <c r="B219" s="74" t="inlineStr">
+        <is>
+          <t>Micro Drip Set (RN)</t>
+        </is>
+      </c>
+      <c r="C219" s="74" t="inlineStr">
+        <is>
+          <t>IV Consumable</t>
+        </is>
+      </c>
+      <c r="D219" s="74" t="n">
+        <v>180</v>
+      </c>
+      <c r="E219" s="74" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="F219" s="76">
+        <f>(D219-E219)/D219</f>
+        <v/>
+      </c>
+      <c r="G219" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #531 / 25-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="74" t="n">
+        <v>198</v>
+      </c>
+      <c r="B220" s="74" t="inlineStr">
+        <is>
+          <t>Kaltex Examination Gloves (100s)</t>
+        </is>
+      </c>
+      <c r="C220" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Gloves</t>
+        </is>
+      </c>
+      <c r="D220" s="74" t="n">
+        <v>2344</v>
+      </c>
+      <c r="E220" s="74" t="n">
+        <v>305.5</v>
+      </c>
+      <c r="F220" s="76">
+        <f>(D220-E220)/D220</f>
+        <v/>
+      </c>
+      <c r="G220" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #533 / 26-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="74" t="n">
+        <v>199</v>
+      </c>
+      <c r="B221" s="74" t="inlineStr">
+        <is>
+          <t>Face Mask 3PLY (ASPAI)</t>
+        </is>
+      </c>
+      <c r="C221" s="74" t="inlineStr">
+        <is>
+          <t>PPE / Protective</t>
+        </is>
+      </c>
+      <c r="D221" s="74" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E221" s="74" t="n">
+        <v>140</v>
+      </c>
+      <c r="F221" s="76">
+        <f>(D221-E221)/D221</f>
+        <v/>
+      </c>
+      <c r="G221" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #545 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="74" t="n">
+        <v>200</v>
+      </c>
+      <c r="B222" s="74" t="inlineStr">
+        <is>
+          <t>Surgical Blade #10 (G) 100s</t>
+        </is>
+      </c>
+      <c r="C222" s="74" t="inlineStr">
+        <is>
+          <t>Surgical Instrument</t>
+        </is>
+      </c>
+      <c r="D222" s="74" t="n">
+        <v>650</v>
+      </c>
+      <c r="E222" s="74" t="n">
+        <v>350</v>
+      </c>
+      <c r="F222" s="76">
+        <f>(D222-E222)/D222</f>
+        <v/>
+      </c>
+      <c r="G222" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #545 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="74" t="n">
+        <v>201</v>
+      </c>
+      <c r="B223" s="74" t="inlineStr">
+        <is>
+          <t>Dispovan 5ML Syringe (ROMOJE)</t>
+        </is>
+      </c>
+      <c r="C223" s="74" t="inlineStr">
+        <is>
+          <t>Syringe &amp; Needle</t>
+        </is>
+      </c>
+      <c r="D223" s="74" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="E223" s="74" t="n">
+        <v>2.98</v>
+      </c>
+      <c r="F223" s="76">
+        <f>(D223-E223)/D223</f>
+        <v/>
+      </c>
+      <c r="G223" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #545 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="74" t="n">
+        <v>202</v>
+      </c>
+      <c r="B224" s="74" t="inlineStr">
+        <is>
+          <t>All Silicon Foley 14Fr (RM)</t>
+        </is>
+      </c>
+      <c r="C224" s="74" t="inlineStr">
+        <is>
+          <t>Urological Consumable</t>
+        </is>
+      </c>
+      <c r="D224" s="74" t="n">
+        <v>824</v>
+      </c>
+      <c r="E224" s="74" t="n">
+        <v>165</v>
+      </c>
+      <c r="F224" s="76">
+        <f>(D224-E224)/D224</f>
+        <v/>
+      </c>
+      <c r="G224" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #545 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="74" t="n">
+        <v>203</v>
+      </c>
+      <c r="B225" s="74" t="inlineStr">
+        <is>
+          <t>Lox 2% Jelly (Lignocaine)</t>
+        </is>
+      </c>
+      <c r="C225" s="74" t="inlineStr">
+        <is>
+          <t>Anaesthesia Consumable</t>
+        </is>
+      </c>
+      <c r="D225" s="74" t="n">
+        <v>34.58</v>
+      </c>
+      <c r="E225" s="74" t="n">
+        <v>27</v>
+      </c>
+      <c r="F225" s="76">
+        <f>(D225-E225)/D225</f>
+        <v/>
+      </c>
+      <c r="G225" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #545 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="74" t="n">
+        <v>204</v>
+      </c>
+      <c r="B226" s="74" t="inlineStr">
+        <is>
+          <t>NS 1000ML FFS (CARTE)</t>
+        </is>
+      </c>
+      <c r="C226" s="74" t="inlineStr">
+        <is>
+          <t>IV Fluid</t>
+        </is>
+      </c>
+      <c r="D226" s="74" t="n">
+        <v>62.65</v>
+      </c>
+      <c r="E226" s="74" t="n">
+        <v>36.53</v>
+      </c>
+      <c r="F226" s="76">
+        <f>(D226-E226)/D226</f>
+        <v/>
+      </c>
+      <c r="G226" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #545 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="74" t="n">
+        <v>205</v>
+      </c>
+      <c r="B227" s="74" t="inlineStr">
+        <is>
+          <t>Moncef 1GM INJ (Cefoperazone)</t>
+        </is>
+      </c>
+      <c r="C227" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D227" s="74" t="n">
+        <v>67.05</v>
+      </c>
+      <c r="E227" s="74" t="n">
+        <v>27.71</v>
+      </c>
+      <c r="F227" s="76">
+        <f>(D227-E227)/D227</f>
+        <v/>
+      </c>
+      <c r="G227" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="74" t="n">
+        <v>206</v>
+      </c>
+      <c r="B228" s="74" t="inlineStr">
+        <is>
+          <t>Vanking 500MG INJ (Vancomycin)</t>
+        </is>
+      </c>
+      <c r="C228" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D228" s="74" t="n">
+        <v>539</v>
+      </c>
+      <c r="E228" s="74" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="F228" s="76">
+        <f>(D228-E228)/D228</f>
+        <v/>
+      </c>
+      <c r="G228" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="74" t="n">
+        <v>207</v>
+      </c>
+      <c r="B229" s="74" t="inlineStr">
+        <is>
+          <t>Artacil 50MG INJ</t>
+        </is>
+      </c>
+      <c r="C229" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D229" s="74" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="E229" s="74" t="n">
+        <v>55</v>
+      </c>
+      <c r="F229" s="76">
+        <f>(D229-E229)/D229</f>
+        <v/>
+      </c>
+      <c r="G229" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="74" t="n">
+        <v>208</v>
+      </c>
+      <c r="B230" s="74" t="inlineStr">
+        <is>
+          <t>Neovec 10MG Vial</t>
+        </is>
+      </c>
+      <c r="C230" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antiemetic</t>
+        </is>
+      </c>
+      <c r="D230" s="74" t="n">
+        <v>125.65</v>
+      </c>
+      <c r="E230" s="74" t="n">
+        <v>87</v>
+      </c>
+      <c r="F230" s="76">
+        <f>(D230-E230)/D230</f>
+        <v/>
+      </c>
+      <c r="G230" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="74" t="n">
+        <v>209</v>
+      </c>
+      <c r="B231" s="74" t="inlineStr">
+        <is>
+          <t>Neovec 4MG INJ</t>
+        </is>
+      </c>
+      <c r="C231" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antiemetic</t>
+        </is>
+      </c>
+      <c r="D231" s="74" t="n">
+        <v>78</v>
+      </c>
+      <c r="E231" s="74" t="n">
+        <v>44</v>
+      </c>
+      <c r="F231" s="76">
+        <f>(D231-E231)/D231</f>
+        <v/>
+      </c>
+      <c r="G231" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="74" t="n">
+        <v>210</v>
+      </c>
+      <c r="B232" s="74" t="inlineStr">
+        <is>
+          <t>Teicobiotic-400 INJ (Teicoplanin)</t>
+        </is>
+      </c>
+      <c r="C232" s="74" t="inlineStr">
+        <is>
+          <t>Injection — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D232" s="74" t="n">
+        <v>3341</v>
+      </c>
+      <c r="E232" s="74" t="n">
+        <v>488</v>
+      </c>
+      <c r="F232" s="76">
+        <f>(D232-E232)/D232</f>
+        <v/>
+      </c>
+      <c r="G232" s="74" t="inlineStr">
+        <is>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="74" t="n">
+        <v>211</v>
+      </c>
+      <c r="B233" s="74" t="inlineStr">
+        <is>
+          <t>Ugaxis-F Tab 1x10</t>
+        </is>
+      </c>
+      <c r="C233" s="74" t="inlineStr">
+        <is>
+          <t>Tablet — Urology</t>
+        </is>
+      </c>
+      <c r="D233" s="74" t="n">
+        <v>450</v>
+      </c>
+      <c r="E233" s="74" t="n">
+        <v>308.57</v>
+      </c>
+      <c r="F233" s="76">
+        <f>(D233-E233)/D233</f>
+        <v/>
+      </c>
+      <c r="G233" s="74" t="inlineStr">
+        <is>
+          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="74" t="n">
+        <v>212</v>
+      </c>
+      <c r="B234" s="74" t="inlineStr">
+        <is>
+          <t>Nefsafe Tab 1x10</t>
+        </is>
+      </c>
+      <c r="C234" s="74" t="inlineStr">
+        <is>
+          <t>Tablet — Antibiotic</t>
+        </is>
+      </c>
+      <c r="D234" s="74" t="n">
+        <v>180</v>
+      </c>
+      <c r="E234" s="74" t="n">
+        <v>123.43</v>
+      </c>
+      <c r="F234" s="76">
+        <f>(D234-E234)/D234</f>
+        <v/>
+      </c>
+      <c r="G234" s="74" t="inlineStr">
+        <is>
+          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="74" t="n">
+        <v>213</v>
+      </c>
+      <c r="B235" s="74" t="inlineStr">
+        <is>
+          <t>KB5 Syrup 200ML</t>
+        </is>
+      </c>
+      <c r="C235" s="74" t="inlineStr">
+        <is>
+          <t>Syrup</t>
+        </is>
+      </c>
+      <c r="D235" s="74" t="n">
+        <v>242</v>
+      </c>
+      <c r="E235" s="74" t="n">
+        <v>165.94</v>
+      </c>
+      <c r="F235" s="76">
+        <f>(D235-E235)/D235</f>
+        <v/>
+      </c>
+      <c r="G235" s="74" t="inlineStr">
+        <is>
+          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="74" t="n">
+        <v>214</v>
+      </c>
+      <c r="B236" s="74" t="inlineStr">
+        <is>
+          <t>Siluts 8ME Tab 1x10</t>
+        </is>
+      </c>
+      <c r="C236" s="74" t="inlineStr">
+        <is>
+          <t>Tablet</t>
+        </is>
+      </c>
+      <c r="D236" s="74" t="n">
+        <v>315</v>
+      </c>
+      <c r="E236" s="74" t="n">
+        <v>216</v>
+      </c>
+      <c r="F236" s="76">
+        <f>(D236-E236)/D236</f>
+        <v/>
+      </c>
+      <c r="G236" s="74" t="inlineStr">
+        <is>
+          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="74" t="n">
+        <v>215</v>
+      </c>
+      <c r="B237" s="74" t="inlineStr">
+        <is>
+          <t>SS Tube-16 (Suction Tube)</t>
+        </is>
+      </c>
+      <c r="C237" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Suction</t>
+        </is>
+      </c>
+      <c r="D237" s="74" t="n">
+        <v>79.58</v>
+      </c>
+      <c r="E237" s="74" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="F237" s="76">
+        <f>(D237-E237)/D237</f>
+        <v/>
+      </c>
+      <c r="G237" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #548 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="74" t="n">
+        <v>216</v>
+      </c>
+      <c r="B238" s="74" t="inlineStr">
+        <is>
+          <t>Surgicare-6.0 Suture</t>
+        </is>
+      </c>
+      <c r="C238" s="74" t="inlineStr">
+        <is>
+          <t>Suture</t>
+        </is>
+      </c>
+      <c r="D238" s="74" t="n">
+        <v>91</v>
+      </c>
+      <c r="E238" s="74" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="F238" s="76">
+        <f>(D238-E238)/D238</f>
+        <v/>
+      </c>
+      <c r="G238" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #548 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="74" t="n">
+        <v>217</v>
+      </c>
+      <c r="B239" s="74" t="inlineStr">
+        <is>
+          <t>Genellium Pro (Large)</t>
+        </is>
+      </c>
+      <c r="C239" s="74" t="inlineStr">
+        <is>
+          <t>OT Consumable — Haemostat</t>
+        </is>
+      </c>
+      <c r="D239" s="74" t="n">
+        <v>3200</v>
+      </c>
+      <c r="E239" s="74" t="n">
+        <v>2250</v>
+      </c>
+      <c r="F239" s="76">
+        <f>(D239-E239)/D239</f>
+        <v/>
+      </c>
+      <c r="G239" s="74" t="inlineStr">
+        <is>
+          <t>B.P. Pharma #548 / 31-Aug-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="72" t="inlineStr">
         <is>
           <t>🔴 ITEMS MISSING MRP — Collect from vendor and update above</t>
         </is>
       </c>
-      <c r="B188" s="42" t="n"/>
-      <c r="C188" s="42" t="n"/>
-      <c r="D188" s="42" t="n"/>
-      <c r="E188" s="42" t="n"/>
-      <c r="F188" s="42" t="n"/>
-      <c r="G188" s="42" t="n"/>
-    </row>
-    <row r="189">
-      <c r="A189" s="48" t="n">
+      <c r="B240" s="42" t="n"/>
+      <c r="C240" s="42" t="n"/>
+      <c r="D240" s="42" t="n"/>
+      <c r="E240" s="42" t="n"/>
+      <c r="F240" s="42" t="n"/>
+      <c r="G240" s="42" t="n"/>
+    </row>
+    <row r="241">
+      <c r="A241" s="48" t="n">
         <v>1</v>
       </c>
-      <c r="B189" s="73" t="inlineStr">
+      <c r="B241" s="73" t="inlineStr">
         <is>
           <t>NS 100ml — Normal Saline 100ml</t>
         </is>
       </c>
-      <c r="C189" s="46" t="inlineStr">
+      <c r="C241" s="46" t="inlineStr">
         <is>
           <t>IV Fluid</t>
         </is>
       </c>
-      <c r="D189" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E189" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F189" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G189" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" s="48" t="n">
+      <c r="D241" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E241" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F241" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G241" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="48" t="n">
         <v>2</v>
       </c>
-      <c r="B190" s="73" t="inlineStr">
+      <c r="B242" s="73" t="inlineStr">
         <is>
           <t>D5 500ml — Dextrose 5%</t>
         </is>
       </c>
-      <c r="C190" s="46" t="inlineStr">
+      <c r="C242" s="46" t="inlineStr">
         <is>
           <t>IV Fluid</t>
         </is>
       </c>
-      <c r="D190" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E190" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F190" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G190" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" s="48" t="n">
+      <c r="D242" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E242" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F242" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G242" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="48" t="n">
         <v>3</v>
       </c>
-      <c r="B191" s="73" t="inlineStr">
+      <c r="B243" s="73" t="inlineStr">
         <is>
           <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
         </is>
       </c>
-      <c r="C191" s="46" t="inlineStr">
+      <c r="C243" s="46" t="inlineStr">
         <is>
           <t>Injection — Anaesthesia</t>
         </is>
       </c>
-      <c r="D191" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E191" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F191" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G191" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" s="48" t="n">
+      <c r="D243" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E243" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F243" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G243" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="48" t="n">
         <v>4</v>
       </c>
-      <c r="B192" s="73" t="inlineStr">
+      <c r="B244" s="73" t="inlineStr">
         <is>
           <t>Inj. Gentamicin</t>
         </is>
       </c>
-      <c r="C192" s="46" t="inlineStr">
+      <c r="C244" s="46" t="inlineStr">
         <is>
           <t>Injection — Antibiotic</t>
         </is>
       </c>
-      <c r="D192" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E192" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F192" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G192" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" s="48" t="n">
+      <c r="D244" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E244" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F244" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G244" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="48" t="n">
         <v>5</v>
       </c>
-      <c r="B193" s="73" t="inlineStr">
+      <c r="B245" s="73" t="inlineStr">
         <is>
           <t>Inj. Tramadol 50mg</t>
         </is>
       </c>
-      <c r="C193" s="46" t="inlineStr">
+      <c r="C245" s="46" t="inlineStr">
         <is>
           <t>Injection — Analgesic</t>
         </is>
       </c>
-      <c r="D193" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E193" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F193" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G193" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" s="48" t="n">
+      <c r="D245" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E245" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F245" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G245" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="48" t="n">
         <v>6</v>
       </c>
-      <c r="B194" s="73" t="inlineStr">
+      <c r="B246" s="73" t="inlineStr">
         <is>
           <t>Inj. PCM 100ml (Paracetamol IV)</t>
         </is>
       </c>
-      <c r="C194" s="46" t="inlineStr">
+      <c r="C246" s="46" t="inlineStr">
         <is>
           <t>Injection — Analgesic</t>
         </is>
       </c>
-      <c r="D194" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E194" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F194" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G194" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" s="48" t="n">
+      <c r="D246" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E246" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F246" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G246" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="48" t="n">
         <v>7</v>
       </c>
-      <c r="B195" s="73" t="inlineStr">
+      <c r="B247" s="73" t="inlineStr">
         <is>
           <t>Inj. Carboprost (Hemabate)</t>
         </is>
       </c>
-      <c r="C195" s="46" t="inlineStr">
+      <c r="C247" s="46" t="inlineStr">
         <is>
           <t>Injection — Oxytocic</t>
         </is>
       </c>
-      <c r="D195" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E195" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F195" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G195" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" s="48" t="n">
+      <c r="D247" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E247" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F247" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G247" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="48" t="n">
         <v>8</v>
       </c>
-      <c r="B196" s="73" t="inlineStr">
+      <c r="B248" s="73" t="inlineStr">
         <is>
           <t>Inj. Adrenaline</t>
         </is>
       </c>
-      <c r="C196" s="46" t="inlineStr">
+      <c r="C248" s="46" t="inlineStr">
         <is>
           <t>Injection — Emergency</t>
         </is>
       </c>
-      <c r="D196" s="47" t="n">
+      <c r="D248" s="47" t="n">
         <v>13.4</v>
       </c>
-      <c r="E196" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F196" s="47" t="inlineStr">
+      <c r="E248" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F248" s="47" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G196" s="47" t="inlineStr">
+      <c r="G248" s="47" t="inlineStr">
         <is>
           <t>Stock OT/Ward: ADRENALIN 1ML</t>
         </is>
       </c>
     </row>
-    <row r="197">
-      <c r="A197" s="48" t="n">
+    <row r="249">
+      <c r="A249" s="48" t="n">
         <v>9</v>
       </c>
-      <c r="B197" s="73" t="inlineStr">
+      <c r="B249" s="73" t="inlineStr">
         <is>
           <t>Inj. Cetil (Cefuroxime Axetil)</t>
         </is>
       </c>
-      <c r="C197" s="46" t="inlineStr">
+      <c r="C249" s="46" t="inlineStr">
         <is>
           <t>Injection — Antibiotic</t>
         </is>
       </c>
-      <c r="D197" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E197" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F197" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G197" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" s="48" t="n">
+      <c r="D249" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E249" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F249" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G249" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="48" t="n">
         <v>10</v>
       </c>
-      <c r="B198" s="73" t="inlineStr">
+      <c r="B250" s="73" t="inlineStr">
         <is>
           <t>Needles 26G (Injection)</t>
         </is>
       </c>
-      <c r="C198" s="46" t="inlineStr">
+      <c r="C250" s="46" t="inlineStr">
         <is>
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D198" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E198" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F198" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G198" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" s="48" t="n">
+      <c r="D250" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E250" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F250" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G250" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="48" t="n">
         <v>11</v>
       </c>
-      <c r="B199" s="73" t="inlineStr">
+      <c r="B251" s="73" t="inlineStr">
         <is>
           <t>Disposable Gloves (Exam)</t>
         </is>
       </c>
-      <c r="C199" s="46" t="inlineStr">
+      <c r="C251" s="46" t="inlineStr">
         <is>
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D199" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E199" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F199" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G199" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" s="48" t="n">
+      <c r="D251" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E251" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F251" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G251" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="48" t="n">
         <v>12</v>
       </c>
-      <c r="B200" s="73" t="inlineStr">
+      <c r="B252" s="73" t="inlineStr">
         <is>
           <t>Betadine Ointment 40g</t>
         </is>
       </c>
-      <c r="C200" s="46" t="inlineStr">
+      <c r="C252" s="46" t="inlineStr">
         <is>
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D200" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E200" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F200" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G200" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" s="48" t="n">
+      <c r="D252" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E252" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F252" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G252" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" s="48" t="n">
         <v>13</v>
       </c>
-      <c r="B201" s="73" t="inlineStr">
+      <c r="B253" s="73" t="inlineStr">
         <is>
           <t>Surgical Blade No. 10</t>
         </is>
       </c>
-      <c r="C201" s="46" t="inlineStr">
+      <c r="C253" s="46" t="inlineStr">
         <is>
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D201" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E201" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F201" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G201" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" s="48" t="n">
+      <c r="D253" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E253" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F253" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G253" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="48" t="n">
         <v>14</v>
       </c>
-      <c r="B202" s="73" t="inlineStr">
+      <c r="B254" s="73" t="inlineStr">
         <is>
           <t>Surgical Blade No. 20</t>
         </is>
       </c>
-      <c r="C202" s="46" t="inlineStr">
+      <c r="C254" s="46" t="inlineStr">
         <is>
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D202" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E202" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F202" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G202" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" s="48" t="n">
+      <c r="D254" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E254" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F254" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G254" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="48" t="n">
         <v>15</v>
       </c>
-      <c r="B203" s="73" t="inlineStr">
+      <c r="B255" s="73" t="inlineStr">
         <is>
           <t>Plain Sheet (OT Draping)</t>
         </is>
       </c>
-      <c r="C203" s="46" t="inlineStr">
+      <c r="C255" s="46" t="inlineStr">
         <is>
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D203" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E203" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F203" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G203" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" s="48" t="n">
+      <c r="D255" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E255" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F255" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G255" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="48" t="n">
         <v>16</v>
       </c>
-      <c r="B204" s="73" t="inlineStr">
+      <c r="B256" s="73" t="inlineStr">
         <is>
           <t>Soft Roll (OT Padding)</t>
         </is>
       </c>
-      <c r="C204" s="46" t="inlineStr">
+      <c r="C256" s="46" t="inlineStr">
         <is>
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D204" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E204" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F204" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G204" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" s="48" t="n">
+      <c r="D256" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E256" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F256" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G256" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="48" t="n">
         <v>17</v>
       </c>
-      <c r="B205" s="73" t="inlineStr">
+      <c r="B257" s="73" t="inlineStr">
         <is>
           <t>Gypsona POP Bandage 40G</t>
         </is>
       </c>
-      <c r="C205" s="46" t="inlineStr">
+      <c r="C257" s="46" t="inlineStr">
         <is>
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D205" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E205" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F205" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G205" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" s="48" t="n">
+      <c r="D257" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E257" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F257" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G257" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="48" t="n">
         <v>18</v>
       </c>
-      <c r="B206" s="73" t="inlineStr">
+      <c r="B258" s="73" t="inlineStr">
         <is>
           <t>Cap + Mask (Disposable Set)</t>
         </is>
       </c>
-      <c r="C206" s="46" t="inlineStr">
+      <c r="C258" s="46" t="inlineStr">
         <is>
           <t>Surgical Consumable</t>
         </is>
       </c>
-      <c r="D206" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E206" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F206" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G206" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" s="48" t="n">
+      <c r="D258" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E258" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F258" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G258" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="48" t="n">
         <v>19</v>
       </c>
-      <c r="B207" s="73" t="inlineStr">
+      <c r="B259" s="73" t="inlineStr">
         <is>
           <t>Glucostrip (Blood Glucose)</t>
         </is>
       </c>
-      <c r="C207" s="46" t="inlineStr">
+      <c r="C259" s="46" t="inlineStr">
         <is>
           <t>Investigation</t>
         </is>
       </c>
-      <c r="D207" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E207" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F207" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G207" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" s="48" t="n">
+      <c r="D259" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E259" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F259" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G259" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="48" t="n">
         <v>20</v>
       </c>
-      <c r="B208" s="73" t="inlineStr">
+      <c r="B260" s="73" t="inlineStr">
         <is>
           <t>Lancet Needle</t>
         </is>
       </c>
-      <c r="C208" s="46" t="inlineStr">
+      <c r="C260" s="46" t="inlineStr">
         <is>
           <t>Investigation</t>
         </is>
       </c>
-      <c r="D208" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E208" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F208" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G208" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" s="48" t="n">
+      <c r="D260" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E260" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F260" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G260" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="48" t="n">
         <v>21</v>
       </c>
-      <c r="B209" s="73" t="inlineStr">
+      <c r="B261" s="73" t="inlineStr">
         <is>
           <t>Red Top Tube (Blood Vial)</t>
         </is>
       </c>
-      <c r="C209" s="46" t="inlineStr">
+      <c r="C261" s="46" t="inlineStr">
         <is>
           <t>Investigation</t>
         </is>
       </c>
-      <c r="D209" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E209" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F209" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G209" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" s="48" t="n">
+      <c r="D261" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E261" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F261" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G261" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="48" t="n">
         <v>22</v>
       </c>
-      <c r="B210" s="73" t="inlineStr">
+      <c r="B262" s="73" t="inlineStr">
         <is>
           <t>CBC Vial Yellow + Red Top</t>
         </is>
       </c>
-      <c r="C210" s="46" t="inlineStr">
+      <c r="C262" s="46" t="inlineStr">
         <is>
           <t>Investigation</t>
         </is>
       </c>
-      <c r="D210" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E210" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F210" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G210" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" s="48" t="n">
+      <c r="D262" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E262" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F262" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G262" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="48" t="n">
         <v>23</v>
       </c>
-      <c r="B211" s="73" t="inlineStr">
+      <c r="B263" s="73" t="inlineStr">
         <is>
           <t>O2 / Oxygen (per use)</t>
         </is>
       </c>
-      <c r="C211" s="46" t="inlineStr">
+      <c r="C263" s="46" t="inlineStr">
         <is>
           <t>Equipment</t>
         </is>
       </c>
-      <c r="D211" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E211" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F211" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G211" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" s="48" t="n">
+      <c r="D263" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E263" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F263" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G263" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="48" t="n">
         <v>24</v>
       </c>
-      <c r="B212" s="73" t="inlineStr">
+      <c r="B264" s="73" t="inlineStr">
         <is>
           <t>Pulse Oximeter (per use)</t>
         </is>
       </c>
-      <c r="C212" s="46" t="inlineStr">
+      <c r="C264" s="46" t="inlineStr">
         <is>
           <t>Equipment</t>
         </is>
       </c>
-      <c r="D212" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E212" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F212" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G212" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" s="48" t="n">
+      <c r="D264" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E264" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F264" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G264" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="48" t="n">
         <v>25</v>
       </c>
-      <c r="B213" s="73" t="inlineStr">
+      <c r="B265" s="73" t="inlineStr">
         <is>
           <t>Cardiac Monitor (per use)</t>
         </is>
       </c>
-      <c r="C213" s="46" t="inlineStr">
+      <c r="C265" s="46" t="inlineStr">
         <is>
           <t>Equipment</t>
         </is>
       </c>
-      <c r="D213" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E213" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F213" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G213" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="48" t="n">
+      <c r="D265" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E265" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F265" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G265" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="48" t="n">
         <v>26</v>
       </c>
-      <c r="B214" s="73" t="inlineStr">
+      <c r="B266" s="73" t="inlineStr">
         <is>
           <t>C-arm (per use)</t>
         </is>
       </c>
-      <c r="C214" s="46" t="inlineStr">
+      <c r="C266" s="46" t="inlineStr">
         <is>
           <t>Equipment</t>
         </is>
       </c>
-      <c r="D214" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E214" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F214" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G214" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" s="48" t="n">
+      <c r="D266" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E266" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F266" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G266" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="48" t="n">
         <v>27</v>
       </c>
-      <c r="B215" s="73" t="inlineStr">
+      <c r="B267" s="73" t="inlineStr">
         <is>
           <t>Volu-P / TiCUP</t>
         </is>
       </c>
-      <c r="C215" s="46" t="inlineStr">
+      <c r="C267" s="46" t="inlineStr">
         <is>
           <t>Consumable</t>
         </is>
       </c>
-      <c r="D215" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E215" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F215" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G215" s="47" t="inlineStr">
+      <c r="D267" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="E267" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="F267" s="47" t="inlineStr">
+        <is>
+          <t>⚠ FILL IN</t>
+        </is>
+      </c>
+      <c r="G267" s="47" t="inlineStr">
         <is>
           <t>⚠ FILL IN</t>
         </is>

</xml_diff>

<commit_message>
Clean rate card: remove duplicates, update costs SL1-165, add SL166-193
- Removed 26 duplicate new items already present in SL1-165
- Removed MISSING MRP section (items now priced in main list)
- Updated costs on 29 existing items from invoice data
- New items SL166-193: new consumables, catheters, antibiotics, tabs
- Final count: 193 unique items

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BaDBrFfWRB3QZkCwovhVaH
</commit_message>
<xml_diff>
--- a/BKAditya_MasterRateCard_UPDATED.xlsx
+++ b/BKAditya_MasterRateCard_UPDATED.xlsx
@@ -289,7 +289,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -517,6 +517,28 @@
     <xf numFmtId="164" fontId="13" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="general" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -770,7 +792,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G267"/>
+  <dimension ref="A1:G216"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="36" min="1" max="1"/>
@@ -893,12 +915,11 @@
         <v>62.24</v>
       </c>
       <c r="E6" s="45" t="n">
-        <v>36.33</v>
-      </c>
-      <c r="F6" s="43" t="inlineStr">
-        <is>
-          <t>41.6%</t>
-        </is>
+        <v>36.53</v>
+      </c>
+      <c r="F6" s="77">
+        <f>(D6-E6)/D6</f>
+        <v/>
       </c>
       <c r="G6" s="44" t="inlineStr">
         <is>
@@ -926,10 +947,9 @@
       <c r="E7" s="47" t="n">
         <v>11.1</v>
       </c>
-      <c r="F7" s="48" t="inlineStr">
-        <is>
-          <t>47.2%</t>
-        </is>
+      <c r="F7" s="78">
+        <f>(D7-E7)/D7</f>
+        <v/>
       </c>
       <c r="G7" s="46" t="inlineStr">
         <is>
@@ -957,10 +977,9 @@
       <c r="E8" s="45" t="n">
         <v>23.8</v>
       </c>
-      <c r="F8" s="43" t="inlineStr">
-        <is>
-          <t>60.6%</t>
-        </is>
+      <c r="F8" s="77">
+        <f>(D8-E8)/D8</f>
+        <v/>
       </c>
       <c r="G8" s="44" t="inlineStr">
         <is>
@@ -1282,10 +1301,9 @@
       <c r="E19" s="51" t="n">
         <v>27</v>
       </c>
-      <c r="F19" s="49" t="inlineStr">
-        <is>
-          <t>21.9%</t>
-        </is>
+      <c r="F19" s="79">
+        <f>(D19-E19)/D19</f>
+        <v/>
       </c>
       <c r="G19" s="50" t="inlineStr">
         <is>
@@ -1448,12 +1466,11 @@
         <v>11.4</v>
       </c>
       <c r="E25" s="47" t="n">
-        <v>7.89</v>
-      </c>
-      <c r="F25" s="48" t="inlineStr">
-        <is>
-          <t>30.8%</t>
-        </is>
+        <v>5.87</v>
+      </c>
+      <c r="F25" s="78">
+        <f>(D25-E25)/D25</f>
+        <v/>
       </c>
       <c r="G25" s="46" t="inlineStr">
         <is>
@@ -1509,15 +1526,12 @@
       <c r="D27" s="47" t="n">
         <v>346.9</v>
       </c>
-      <c r="E27" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL</t>
-        </is>
-      </c>
-      <c r="F27" s="48" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="E27" s="47" t="n">
+        <v>90</v>
+      </c>
+      <c r="F27" s="78">
+        <f>(D27-E27)/D27</f>
+        <v/>
       </c>
       <c r="G27" s="46" t="inlineStr">
         <is>
@@ -1788,12 +1802,11 @@
         <v>12.72</v>
       </c>
       <c r="E37" s="56" t="n">
-        <v>4.85</v>
-      </c>
-      <c r="F37" s="54" t="inlineStr">
-        <is>
-          <t>61.9%</t>
-        </is>
+        <v>10</v>
+      </c>
+      <c r="F37" s="80">
+        <f>(D37-E37)/D37</f>
+        <v/>
       </c>
       <c r="G37" s="55" t="inlineStr">
         <is>
@@ -1925,12 +1938,11 @@
         <v>53.9</v>
       </c>
       <c r="E42" s="56" t="n">
-        <v>41.07</v>
-      </c>
-      <c r="F42" s="54" t="inlineStr">
-        <is>
-          <t>23.8%</t>
-        </is>
+        <v>18</v>
+      </c>
+      <c r="F42" s="80">
+        <f>(D42-E42)/D42</f>
+        <v/>
       </c>
       <c r="G42" s="55" t="inlineStr">
         <is>
@@ -2376,12 +2388,11 @@
         <v>221</v>
       </c>
       <c r="E61" s="67" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="F61" s="65" t="inlineStr">
-        <is>
-          <t>93.4%</t>
-        </is>
+        <v>14.06</v>
+      </c>
+      <c r="F61" s="81">
+        <f>(D61-E61)/D61</f>
+        <v/>
       </c>
       <c r="G61" s="66" t="inlineStr">
         <is>
@@ -2533,10 +2544,9 @@
       <c r="E66" s="67" t="n">
         <v>40.5</v>
       </c>
-      <c r="F66" s="65" t="inlineStr">
-        <is>
-          <t>92.0%</t>
-        </is>
+      <c r="F66" s="81">
+        <f>(D66-E66)/D66</f>
+        <v/>
       </c>
       <c r="G66" s="66" t="inlineStr">
         <is>
@@ -2717,12 +2727,11 @@
         <v>153</v>
       </c>
       <c r="E72" s="67" t="n">
-        <v>74.29000000000001</v>
-      </c>
-      <c r="F72" s="65" t="inlineStr">
-        <is>
-          <t>51.4%</t>
-        </is>
+        <v>80.75</v>
+      </c>
+      <c r="F72" s="81">
+        <f>(D72-E72)/D72</f>
+        <v/>
       </c>
       <c r="G72" s="66" t="inlineStr">
         <is>
@@ -2748,12 +2757,11 @@
         <v>20</v>
       </c>
       <c r="E73" s="67" t="n">
-        <v>3.76</v>
-      </c>
-      <c r="F73" s="65" t="inlineStr">
-        <is>
-          <t>81.2%</t>
-        </is>
+        <v>4.55</v>
+      </c>
+      <c r="F73" s="81">
+        <f>(D73-E73)/D73</f>
+        <v/>
       </c>
       <c r="G73" s="66" t="inlineStr">
         <is>
@@ -2779,12 +2787,11 @@
         <v>10.23</v>
       </c>
       <c r="E74" s="67" t="n">
-        <v>2.38</v>
-      </c>
-      <c r="F74" s="65" t="inlineStr">
-        <is>
-          <t>76.7%</t>
-        </is>
+        <v>2.98</v>
+      </c>
+      <c r="F74" s="81">
+        <f>(D74-E74)/D74</f>
+        <v/>
       </c>
       <c r="G74" s="66" t="inlineStr">
         <is>
@@ -3360,10 +3367,9 @@
       <c r="E93" s="53" t="n">
         <v>58</v>
       </c>
-      <c r="F93" s="57" t="inlineStr">
-        <is>
-          <t>54.7%</t>
-        </is>
+      <c r="F93" s="82">
+        <f>(D93-E93)/D93</f>
+        <v/>
       </c>
       <c r="G93" s="52" t="inlineStr">
         <is>
@@ -3612,10 +3618,9 @@
       <c r="E101" s="47" t="n">
         <v>65</v>
       </c>
-      <c r="F101" s="48" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F101" s="78">
+        <f>(D101-E101)/D101</f>
+        <v/>
       </c>
       <c r="G101" s="46" t="inlineStr">
         <is>
@@ -3643,10 +3648,9 @@
       <c r="E102" s="47" t="n">
         <v>45.74</v>
       </c>
-      <c r="F102" s="48" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F102" s="78">
+        <f>(D102-E102)/D102</f>
+        <v/>
       </c>
       <c r="G102" s="46" t="inlineStr">
         <is>
@@ -4188,6 +4192,7 @@
         </is>
       </c>
     </row>
+    <row r="121"/>
     <row r="122" ht="13.5" customHeight="1" s="37">
       <c r="A122" s="36" t="n">
         <v>100</v>
@@ -4253,12 +4258,11 @@
         <v>408</v>
       </c>
       <c r="E125" s="36" t="n">
-        <v>362.24</v>
-      </c>
-      <c r="F125" s="36" t="inlineStr">
-        <is>
-          <t>11.2%</t>
-        </is>
+        <v>353.75</v>
+      </c>
+      <c r="F125" s="83">
+        <f>(D125-E125)/D125</f>
+        <v/>
       </c>
       <c r="G125" s="36" t="inlineStr">
         <is>
@@ -4279,12 +4283,11 @@
         <v>191</v>
       </c>
       <c r="E126" s="36" t="n">
-        <v>128.45</v>
-      </c>
-      <c r="F126" s="36" t="inlineStr">
-        <is>
-          <t>32.7%</t>
-        </is>
+        <v>165</v>
+      </c>
+      <c r="F126" s="83">
+        <f>(D126-E126)/D126</f>
+        <v/>
       </c>
       <c r="G126" s="36" t="inlineStr">
         <is>
@@ -4305,7 +4308,11 @@
         <v>191</v>
       </c>
       <c r="E127" s="36" t="n">
-        <v>130</v>
+        <v>131.45</v>
+      </c>
+      <c r="F127" s="84">
+        <f>(D127-E127)/D127</f>
+        <v/>
       </c>
       <c r="G127" s="36" t="inlineStr">
         <is>
@@ -4431,7 +4438,11 @@
         <v>255</v>
       </c>
       <c r="E133" s="36" t="n">
-        <v>50</v>
+        <v>18.62</v>
+      </c>
+      <c r="F133" s="84">
+        <f>(D133-E133)/D133</f>
+        <v/>
       </c>
       <c r="G133" s="36" t="inlineStr">
         <is>
@@ -4601,10 +4612,9 @@
       <c r="E141" s="36" t="n">
         <v>123</v>
       </c>
-      <c r="F141" s="36" t="inlineStr">
-        <is>
-          <t>82.4%</t>
-        </is>
+      <c r="F141" s="83">
+        <f>(D141-E141)/D141</f>
+        <v/>
       </c>
       <c r="G141" s="36" t="inlineStr">
         <is>
@@ -4672,12 +4682,11 @@
         <v>234</v>
       </c>
       <c r="E144" s="36" t="n">
-        <v>157.71</v>
-      </c>
-      <c r="F144" s="36" t="inlineStr">
-        <is>
-          <t>32.6%</t>
-        </is>
+        <v>169</v>
+      </c>
+      <c r="F144" s="83">
+        <f>(D144-E144)/D144</f>
+        <v/>
       </c>
       <c r="G144" s="36" t="inlineStr">
         <is>
@@ -5271,10 +5280,9 @@
       <c r="E164" s="36" t="n">
         <v>810</v>
       </c>
-      <c r="F164" s="36" t="inlineStr">
-        <is>
-          <t>70.5%</t>
-        </is>
+      <c r="F164" s="83">
+        <f>(D164-E164)/D164</f>
+        <v/>
       </c>
       <c r="G164" s="36" t="inlineStr">
         <is>
@@ -5302,10 +5310,9 @@
       <c r="E165" s="36" t="n">
         <v>20.1</v>
       </c>
-      <c r="F165" s="36" t="inlineStr">
-        <is>
-          <t>89.3%</t>
-        </is>
+      <c r="F165" s="83">
+        <f>(D165-E165)/D165</f>
+        <v/>
       </c>
       <c r="G165" s="36" t="inlineStr">
         <is>
@@ -5364,10 +5371,9 @@
       <c r="E167" s="36" t="n">
         <v>78</v>
       </c>
-      <c r="F167" s="36" t="inlineStr">
-        <is>
-          <t>37.1%</t>
-        </is>
+      <c r="F167" s="83">
+        <f>(D167-E167)/D167</f>
+        <v/>
       </c>
       <c r="G167" s="36" t="inlineStr">
         <is>
@@ -5395,10 +5401,9 @@
       <c r="E168" s="36" t="n">
         <v>31.15</v>
       </c>
-      <c r="F168" s="36" t="inlineStr">
-        <is>
-          <t>91.9%</t>
-        </is>
+      <c r="F168" s="83">
+        <f>(D168-E168)/D168</f>
+        <v/>
       </c>
       <c r="G168" s="36" t="inlineStr">
         <is>
@@ -5459,10 +5464,9 @@
       <c r="E170" s="36" t="n">
         <v>305.5</v>
       </c>
-      <c r="F170" s="36" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="F170" s="83">
+        <f>(D170-E170)/D170</f>
+        <v/>
       </c>
       <c r="G170" s="36" t="inlineStr">
         <is>
@@ -5519,12 +5523,11 @@
         <v>470</v>
       </c>
       <c r="E172" s="36" t="n">
-        <v>265</v>
-      </c>
-      <c r="F172" s="36" t="inlineStr">
-        <is>
-          <t>43.6%</t>
-        </is>
+        <v>261.25</v>
+      </c>
+      <c r="F172" s="83">
+        <f>(D172-E172)/D172</f>
+        <v/>
       </c>
       <c r="G172" s="36" t="inlineStr">
         <is>
@@ -5585,12 +5588,11 @@
         </is>
       </c>
       <c r="E174" s="36" t="n">
-        <v>208</v>
-      </c>
-      <c r="F174" s="36" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>186.5</v>
+      </c>
+      <c r="F174" s="83">
+        <f>(D174-E174)/D174</f>
+        <v/>
       </c>
       <c r="G174" s="36" t="inlineStr">
         <is>
@@ -6007,19 +6009,19 @@
       </c>
       <c r="B188" s="74" t="inlineStr">
         <is>
-          <t>NS 3000ML IV Bag (KRPL)</t>
+          <t>Hydrogen Peroxide Solution 45</t>
         </is>
       </c>
       <c r="C188" s="74" t="inlineStr">
         <is>
-          <t>IV Fluid</t>
+          <t>Antiseptic/Disinfectant</t>
         </is>
       </c>
       <c r="D188" s="74" t="n">
-        <v>698</v>
+        <v>83</v>
       </c>
       <c r="E188" s="74" t="n">
-        <v>123</v>
+        <v>38.5</v>
       </c>
       <c r="F188" s="76">
         <f>(D188-E188)/D188</f>
@@ -6037,19 +6039,19 @@
       </c>
       <c r="B189" s="74" t="inlineStr">
         <is>
-          <t>Hydrogen Peroxide Solution 45</t>
+          <t>Cloth Drape CD01</t>
         </is>
       </c>
       <c r="C189" s="74" t="inlineStr">
         <is>
-          <t>Antiseptic/Disinfectant</t>
+          <t>OT Consumable — Drape</t>
         </is>
       </c>
       <c r="D189" s="74" t="n">
-        <v>83</v>
+        <v>62</v>
       </c>
       <c r="E189" s="74" t="n">
-        <v>38.5</v>
+        <v>43.33</v>
       </c>
       <c r="F189" s="76">
         <f>(D189-E189)/D189</f>
@@ -6067,19 +6069,19 @@
       </c>
       <c r="B190" s="74" t="inlineStr">
         <is>
-          <t>Spinocan-25 Spinal Needle</t>
+          <t>OT X-Ray Gauze</t>
         </is>
       </c>
       <c r="C190" s="74" t="inlineStr">
         <is>
-          <t>Anaesthesia Consumable</t>
+          <t>OT Consumable — Gauze</t>
         </is>
       </c>
       <c r="D190" s="74" t="n">
-        <v>143.44</v>
+        <v>51.56</v>
       </c>
       <c r="E190" s="74" t="n">
-        <v>80.75</v>
+        <v>24.55</v>
       </c>
       <c r="F190" s="76">
         <f>(D190-E190)/D190</f>
@@ -6097,19 +6099,19 @@
       </c>
       <c r="B191" s="74" t="inlineStr">
         <is>
-          <t>Full Body OT Gown (NAERLZM)</t>
+          <t>Diathermy Pencil (RM)</t>
         </is>
       </c>
       <c r="C191" s="74" t="inlineStr">
         <is>
-          <t>OT Consumable — Protective</t>
+          <t>OT Equipment — Diathermy</t>
         </is>
       </c>
       <c r="D191" s="74" t="n">
-        <v>426</v>
+        <v>917</v>
       </c>
       <c r="E191" s="74" t="n">
-        <v>261.25</v>
+        <v>121.12</v>
       </c>
       <c r="F191" s="76">
         <f>(D191-E191)/D191</f>
@@ -6117,7 +6119,7 @@
       </c>
       <c r="G191" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #493 / 17-Aug-26</t>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6127,19 +6129,19 @@
       </c>
       <c r="B192" s="74" t="inlineStr">
         <is>
-          <t>Cloth Drape CD01</t>
+          <t>Vaccu Suction Set (A)</t>
         </is>
       </c>
       <c r="C192" s="74" t="inlineStr">
         <is>
-          <t>OT Consumable — Drape</t>
+          <t>OT Consumable — Suction</t>
         </is>
       </c>
       <c r="D192" s="74" t="n">
-        <v>62</v>
+        <v>609</v>
       </c>
       <c r="E192" s="74" t="n">
-        <v>43.33</v>
+        <v>64</v>
       </c>
       <c r="F192" s="76">
         <f>(D192-E192)/D192</f>
@@ -6147,7 +6149,7 @@
       </c>
       <c r="G192" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #493 / 17-Aug-26</t>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6157,19 +6159,19 @@
       </c>
       <c r="B193" s="74" t="inlineStr">
         <is>
-          <t>OT X-Ray Gauze</t>
+          <t>Foley's Catheter 3-Way 18Fr</t>
         </is>
       </c>
       <c r="C193" s="74" t="inlineStr">
         <is>
-          <t>OT Consumable — Gauze</t>
+          <t>Urological Consumable</t>
         </is>
       </c>
       <c r="D193" s="74" t="n">
-        <v>51.56</v>
+        <v>460</v>
       </c>
       <c r="E193" s="74" t="n">
-        <v>24.55</v>
+        <v>353.75</v>
       </c>
       <c r="F193" s="76">
         <f>(D193-E193)/D193</f>
@@ -6177,7 +6179,7 @@
       </c>
       <c r="G193" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #493 / 17-Aug-26</t>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6187,19 +6189,19 @@
       </c>
       <c r="B194" s="74" t="inlineStr">
         <is>
-          <t>Ondem 4ML INJ (Ondansetron)</t>
+          <t>Foley's Catheter 3-Way 24Fr</t>
         </is>
       </c>
       <c r="C194" s="74" t="inlineStr">
         <is>
-          <t>Injection — Antiemetic</t>
+          <t>Urological Consumable</t>
         </is>
       </c>
       <c r="D194" s="74" t="n">
-        <v>25.45</v>
+        <v>448</v>
       </c>
       <c r="E194" s="74" t="n">
-        <v>10</v>
+        <v>353.75</v>
       </c>
       <c r="F194" s="76">
         <f>(D194-E194)/D194</f>
@@ -6207,7 +6209,7 @@
       </c>
       <c r="G194" s="74" t="inlineStr">
         <is>
-          <t>M.R. Pharma MR001046 / 18-Aug-26</t>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6217,19 +6219,19 @@
       </c>
       <c r="B195" s="74" t="inlineStr">
         <is>
-          <t>PAN IV 40MG (Pantoprazole IV)</t>
+          <t>Foley's Catheter 2-Way 20Fr</t>
         </is>
       </c>
       <c r="C195" s="74" t="inlineStr">
         <is>
-          <t>Injection — PPI</t>
+          <t>Urological Consumable</t>
         </is>
       </c>
       <c r="D195" s="74" t="n">
-        <v>54.24</v>
+        <v>174</v>
       </c>
       <c r="E195" s="74" t="n">
-        <v>18</v>
+        <v>131.45</v>
       </c>
       <c r="F195" s="76">
         <f>(D195-E195)/D195</f>
@@ -6237,7 +6239,7 @@
       </c>
       <c r="G195" s="74" t="inlineStr">
         <is>
-          <t>M.R. Pharma MR001046 / 18-Aug-26</t>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6247,19 +6249,19 @@
       </c>
       <c r="B196" s="74" t="inlineStr">
         <is>
-          <t>Nllg-Mycin INJ (Gentamicin)</t>
+          <t>Foley's Catheter 2-Way 22Fr</t>
         </is>
       </c>
       <c r="C196" s="74" t="inlineStr">
         <is>
-          <t>Injection — Antibiotic</t>
+          <t>Urological Consumable</t>
         </is>
       </c>
       <c r="D196" s="74" t="n">
-        <v>9.84</v>
+        <v>163.13</v>
       </c>
       <c r="E196" s="74" t="n">
-        <v>5.87</v>
+        <v>131.45</v>
       </c>
       <c r="F196" s="76">
         <f>(D196-E196)/D196</f>
@@ -6267,7 +6269,7 @@
       </c>
       <c r="G196" s="74" t="inlineStr">
         <is>
-          <t>M.R. Pharma MR001046 / 18-Aug-26</t>
+          <t>B.P. Pharma #511 / 19-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6277,19 +6279,19 @@
       </c>
       <c r="B197" s="74" t="inlineStr">
         <is>
-          <t>Diathermy Pencil (RM)</t>
+          <t>Adult Diaper (Large) RAM</t>
         </is>
       </c>
       <c r="C197" s="74" t="inlineStr">
         <is>
-          <t>OT Equipment — Diathermy</t>
+          <t>Ward Consumable</t>
         </is>
       </c>
       <c r="D197" s="74" t="n">
-        <v>917</v>
+        <v>120</v>
       </c>
       <c r="E197" s="74" t="n">
-        <v>121.12</v>
+        <v>25</v>
       </c>
       <c r="F197" s="76">
         <f>(D197-E197)/D197</f>
@@ -6297,7 +6299,7 @@
       </c>
       <c r="G197" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>B.P. Pharma #513 / 20-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6307,19 +6309,19 @@
       </c>
       <c r="B198" s="74" t="inlineStr">
         <is>
-          <t>Vaccu Suction Set (A)</t>
+          <t>Betadine Scrub 500ML</t>
         </is>
       </c>
       <c r="C198" s="74" t="inlineStr">
         <is>
-          <t>OT Consumable — Suction</t>
+          <t>Antiseptic/Disinfectant</t>
         </is>
       </c>
       <c r="D198" s="74" t="n">
-        <v>609</v>
+        <v>1071</v>
       </c>
       <c r="E198" s="74" t="n">
-        <v>64</v>
+        <v>928</v>
       </c>
       <c r="F198" s="76">
         <f>(D198-E198)/D198</f>
@@ -6327,7 +6329,7 @@
       </c>
       <c r="G198" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>B.P. Pharma #526 / 24-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6337,19 +6339,19 @@
       </c>
       <c r="B199" s="74" t="inlineStr">
         <is>
-          <t>Roll Bandage 4" (LC)</t>
+          <t>E Coli Cath L4</t>
         </is>
       </c>
       <c r="C199" s="74" t="inlineStr">
         <is>
-          <t>Dressing &amp; Bandage</t>
+          <t>Urological Consumable</t>
         </is>
       </c>
       <c r="D199" s="74" t="n">
         <v>120</v>
       </c>
       <c r="E199" s="74" t="n">
-        <v>58</v>
+        <v>16.6</v>
       </c>
       <c r="F199" s="76">
         <f>(D199-E199)/D199</f>
@@ -6357,7 +6359,7 @@
       </c>
       <c r="G199" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>B.P. Pharma #531 / 25-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6367,19 +6369,19 @@
       </c>
       <c r="B200" s="74" t="inlineStr">
         <is>
-          <t>Roll Bandage 6" (LC)</t>
+          <t>Face Mask 3PLY (ASPAI)</t>
         </is>
       </c>
       <c r="C200" s="74" t="inlineStr">
         <is>
-          <t>Dressing &amp; Bandage</t>
+          <t>PPE / Protective</t>
         </is>
       </c>
       <c r="D200" s="74" t="n">
-        <v>124</v>
+        <v>1500</v>
       </c>
       <c r="E200" s="74" t="n">
-        <v>78</v>
+        <v>140</v>
       </c>
       <c r="F200" s="76">
         <f>(D200-E200)/D200</f>
@@ -6387,7 +6389,7 @@
       </c>
       <c r="G200" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>B.P. Pharma #545 / 29-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6397,19 +6399,19 @@
       </c>
       <c r="B201" s="74" t="inlineStr">
         <is>
-          <t>Urobag (ROND-10)</t>
+          <t>Moncef 1GM INJ (Cefoperazone)</t>
         </is>
       </c>
       <c r="C201" s="74" t="inlineStr">
         <is>
-          <t>Urological Consumable</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D201" s="74" t="n">
-        <v>361</v>
+        <v>67.05</v>
       </c>
       <c r="E201" s="74" t="n">
-        <v>40.5</v>
+        <v>27.71</v>
       </c>
       <c r="F201" s="76">
         <f>(D201-E201)/D201</f>
@@ -6417,7 +6419,7 @@
       </c>
       <c r="G201" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6427,19 +6429,19 @@
       </c>
       <c r="B202" s="74" t="inlineStr">
         <is>
-          <t>Camera Cover (D904)</t>
+          <t>Vanking 500MG INJ (Vancomycin)</t>
         </is>
       </c>
       <c r="C202" s="74" t="inlineStr">
         <is>
-          <t>OT Consumable — Laparoscopy</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D202" s="74" t="n">
-        <v>237</v>
+        <v>539</v>
       </c>
       <c r="E202" s="74" t="n">
-        <v>169</v>
+        <v>76.40000000000001</v>
       </c>
       <c r="F202" s="76">
         <f>(D202-E202)/D202</f>
@@ -6447,7 +6449,7 @@
       </c>
       <c r="G202" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6457,19 +6459,19 @@
       </c>
       <c r="B203" s="74" t="inlineStr">
         <is>
-          <t>Nasal Cannula (AIRWA)</t>
+          <t>Artacil 50MG INJ</t>
         </is>
       </c>
       <c r="C203" s="74" t="inlineStr">
         <is>
-          <t>Respiratory Consumable</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D203" s="74" t="n">
-        <v>363</v>
+        <v>90.59999999999999</v>
       </c>
       <c r="E203" s="74" t="n">
-        <v>18.62</v>
+        <v>55</v>
       </c>
       <c r="F203" s="76">
         <f>(D203-E203)/D203</f>
@@ -6477,7 +6479,7 @@
       </c>
       <c r="G203" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6487,19 +6489,19 @@
       </c>
       <c r="B204" s="74" t="inlineStr">
         <is>
-          <t>Genellium Pro (Pink 5)</t>
+          <t>Neovec 10MG Vial</t>
         </is>
       </c>
       <c r="C204" s="74" t="inlineStr">
         <is>
-          <t>OT Consumable — Haemostat</t>
+          <t>Injection — Antiemetic</t>
         </is>
       </c>
       <c r="D204" s="74" t="n">
-        <v>2750</v>
+        <v>125.65</v>
       </c>
       <c r="E204" s="74" t="n">
-        <v>810</v>
+        <v>87</v>
       </c>
       <c r="F204" s="76">
         <f>(D204-E204)/D204</f>
@@ -6507,7 +6509,7 @@
       </c>
       <c r="G204" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6517,19 +6519,19 @@
       </c>
       <c r="B205" s="74" t="inlineStr">
         <is>
-          <t>Foley's Catheter 3-Way 22Fr</t>
+          <t>Neovec 4MG INJ</t>
         </is>
       </c>
       <c r="C205" s="74" t="inlineStr">
         <is>
-          <t>Urological Consumable</t>
+          <t>Injection — Antiemetic</t>
         </is>
       </c>
       <c r="D205" s="74" t="n">
-        <v>491</v>
+        <v>78</v>
       </c>
       <c r="E205" s="74" t="n">
-        <v>353.75</v>
+        <v>44</v>
       </c>
       <c r="F205" s="76">
         <f>(D205-E205)/D205</f>
@@ -6537,7 +6539,7 @@
       </c>
       <c r="G205" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6547,19 +6549,19 @@
       </c>
       <c r="B206" s="74" t="inlineStr">
         <is>
-          <t>Foley's Catheter 3-Way 18Fr</t>
+          <t>Teicobiotic-400 INJ (Teicoplanin)</t>
         </is>
       </c>
       <c r="C206" s="74" t="inlineStr">
         <is>
-          <t>Urological Consumable</t>
+          <t>Injection — Antibiotic</t>
         </is>
       </c>
       <c r="D206" s="74" t="n">
-        <v>460</v>
+        <v>3341</v>
       </c>
       <c r="E206" s="74" t="n">
-        <v>353.75</v>
+        <v>488</v>
       </c>
       <c r="F206" s="76">
         <f>(D206-E206)/D206</f>
@@ -6567,7 +6569,7 @@
       </c>
       <c r="G206" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6577,19 +6579,19 @@
       </c>
       <c r="B207" s="74" t="inlineStr">
         <is>
-          <t>Foley's Catheter 3-Way 24Fr</t>
+          <t>Ugaxis-F Tab 1x10</t>
         </is>
       </c>
       <c r="C207" s="74" t="inlineStr">
         <is>
-          <t>Urological Consumable</t>
+          <t>Tablet — Urology</t>
         </is>
       </c>
       <c r="D207" s="74" t="n">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="E207" s="74" t="n">
-        <v>353.75</v>
+        <v>308.57</v>
       </c>
       <c r="F207" s="76">
         <f>(D207-E207)/D207</f>
@@ -6597,7 +6599,7 @@
       </c>
       <c r="G207" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6607,19 +6609,19 @@
       </c>
       <c r="B208" s="74" t="inlineStr">
         <is>
-          <t>Foley's Catheter 2-Way 16Fr</t>
+          <t>Nefsafe Tab 1x10</t>
         </is>
       </c>
       <c r="C208" s="74" t="inlineStr">
         <is>
-          <t>Urological Consumable</t>
+          <t>Tablet — Antibiotic</t>
         </is>
       </c>
       <c r="D208" s="74" t="n">
-        <v>191</v>
+        <v>180</v>
       </c>
       <c r="E208" s="74" t="n">
-        <v>131.45</v>
+        <v>123.43</v>
       </c>
       <c r="F208" s="76">
         <f>(D208-E208)/D208</f>
@@ -6627,7 +6629,7 @@
       </c>
       <c r="G208" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6637,19 +6639,19 @@
       </c>
       <c r="B209" s="74" t="inlineStr">
         <is>
-          <t>Foley's Catheter 2-Way 20Fr</t>
+          <t>KB5 Syrup 200ML</t>
         </is>
       </c>
       <c r="C209" s="74" t="inlineStr">
         <is>
-          <t>Urological Consumable</t>
+          <t>Syrup</t>
         </is>
       </c>
       <c r="D209" s="74" t="n">
-        <v>174</v>
+        <v>242</v>
       </c>
       <c r="E209" s="74" t="n">
-        <v>131.45</v>
+        <v>165.94</v>
       </c>
       <c r="F209" s="76">
         <f>(D209-E209)/D209</f>
@@ -6657,7 +6659,7 @@
       </c>
       <c r="G209" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6667,19 +6669,19 @@
       </c>
       <c r="B210" s="74" t="inlineStr">
         <is>
-          <t>Foley's Catheter 2-Way 22Fr</t>
+          <t>Siluts 8ME Tab 1x10</t>
         </is>
       </c>
       <c r="C210" s="74" t="inlineStr">
         <is>
-          <t>Urological Consumable</t>
+          <t>Tablet</t>
         </is>
       </c>
       <c r="D210" s="74" t="n">
-        <v>163.13</v>
+        <v>315</v>
       </c>
       <c r="E210" s="74" t="n">
-        <v>131.45</v>
+        <v>216</v>
       </c>
       <c r="F210" s="76">
         <f>(D210-E210)/D210</f>
@@ -6687,7 +6689,7 @@
       </c>
       <c r="G210" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #511 / 19-Aug-26</t>
+          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6697,19 +6699,19 @@
       </c>
       <c r="B211" s="74" t="inlineStr">
         <is>
-          <t>RL 500ML Flat Cap</t>
+          <t>SS Tube-16 (Suction Tube)</t>
         </is>
       </c>
       <c r="C211" s="74" t="inlineStr">
         <is>
-          <t>IV Fluid</t>
+          <t>OT Consumable — Suction</t>
         </is>
       </c>
       <c r="D211" s="74" t="n">
-        <v>60.74</v>
+        <v>79.58</v>
       </c>
       <c r="E211" s="74" t="n">
-        <v>23.8</v>
+        <v>18.5</v>
       </c>
       <c r="F211" s="76">
         <f>(D211-E211)/D211</f>
@@ -6717,7 +6719,7 @@
       </c>
       <c r="G211" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #513 / 20-Aug-26</t>
+          <t>B.P. Pharma #548 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6727,19 +6729,19 @@
       </c>
       <c r="B212" s="74" t="inlineStr">
         <is>
-          <t>Weardn Disposable Apron</t>
+          <t>Surgicare-6.0 Suture</t>
         </is>
       </c>
       <c r="C212" s="74" t="inlineStr">
         <is>
-          <t>OT Consumable — Protective</t>
+          <t>Suture</t>
         </is>
       </c>
       <c r="D212" s="74" t="n">
-        <v>672</v>
+        <v>91</v>
       </c>
       <c r="E212" s="74" t="n">
-        <v>186.5</v>
+        <v>21.5</v>
       </c>
       <c r="F212" s="76">
         <f>(D212-E212)/D212</f>
@@ -6747,7 +6749,7 @@
       </c>
       <c r="G212" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #513 / 20-Aug-26</t>
+          <t>B.P. Pharma #548 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6757,19 +6759,19 @@
       </c>
       <c r="B213" s="74" t="inlineStr">
         <is>
-          <t>Adult Diaper (Large) RAM</t>
+          <t>Genellium Pro (Large)</t>
         </is>
       </c>
       <c r="C213" s="74" t="inlineStr">
         <is>
-          <t>Ward Consumable</t>
+          <t>OT Consumable — Haemostat</t>
         </is>
       </c>
       <c r="D213" s="74" t="n">
-        <v>120</v>
+        <v>3200</v>
       </c>
       <c r="E213" s="74" t="n">
-        <v>25</v>
+        <v>2250</v>
       </c>
       <c r="F213" s="76">
         <f>(D213-E213)/D213</f>
@@ -6777,7 +6779,7 @@
       </c>
       <c r="G213" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #513 / 20-Aug-26</t>
+          <t>B.P. Pharma #548 / 31-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6787,19 +6789,19 @@
       </c>
       <c r="B214" s="74" t="inlineStr">
         <is>
-          <t>Betadine Scrub 500ML</t>
+          <t>Adult Diaper 10s (Disposable)</t>
         </is>
       </c>
       <c r="C214" s="74" t="inlineStr">
         <is>
-          <t>Antiseptic/Disinfectant</t>
+          <t>Ward Consumable</t>
         </is>
       </c>
       <c r="D214" s="74" t="n">
-        <v>1071</v>
+        <v>145</v>
       </c>
       <c r="E214" s="74" t="n">
-        <v>928</v>
+        <v>22</v>
       </c>
       <c r="F214" s="76">
         <f>(D214-E214)/D214</f>
@@ -6807,7 +6809,7 @@
       </c>
       <c r="G214" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #526 / 24-Aug-26</t>
+          <t>B.P. Pharma #513 / 20-Aug-26</t>
         </is>
       </c>
     </row>
@@ -6817,19 +6819,19 @@
       </c>
       <c r="B215" s="74" t="inlineStr">
         <is>
-          <t>Dispovan 10ML Syringe (ROMOJE)</t>
+          <t>Surgicare 7.0 Suture</t>
         </is>
       </c>
       <c r="C215" s="74" t="inlineStr">
         <is>
-          <t>Syringe &amp; Needle</t>
+          <t>Suture</t>
         </is>
       </c>
       <c r="D215" s="74" t="n">
-        <v>20.8</v>
+        <v>91</v>
       </c>
       <c r="E215" s="74" t="n">
-        <v>4.55</v>
+        <v>21.5</v>
       </c>
       <c r="F215" s="76">
         <f>(D215-E215)/D215</f>
@@ -6837,1685 +6839,22 @@
       </c>
       <c r="G215" s="74" t="inlineStr">
         <is>
-          <t>B.P. Pharma #531 / 25-Aug-26</t>
+          <t>B.P. Pharma #511 &amp; #513 / Aug-26</t>
         </is>
       </c>
     </row>
     <row r="216">
-      <c r="A216" s="74" t="n">
-        <v>194</v>
-      </c>
-      <c r="B216" s="74" t="inlineStr">
-        <is>
-          <t>E Coli Cath L4</t>
-        </is>
-      </c>
-      <c r="C216" s="74" t="inlineStr">
-        <is>
-          <t>Urological Consumable</t>
-        </is>
-      </c>
-      <c r="D216" s="74" t="n">
-        <v>120</v>
-      </c>
-      <c r="E216" s="74" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="F216" s="76">
-        <f>(D216-E216)/D216</f>
-        <v/>
-      </c>
-      <c r="G216" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #531 / 25-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" s="74" t="n">
-        <v>195</v>
-      </c>
-      <c r="B217" s="74" t="inlineStr">
-        <is>
-          <t>Vein O Line-10 CM</t>
-        </is>
-      </c>
-      <c r="C217" s="74" t="inlineStr">
-        <is>
-          <t>IV Consumable</t>
-        </is>
-      </c>
-      <c r="D217" s="74" t="n">
-        <v>386</v>
-      </c>
-      <c r="E217" s="74" t="n">
-        <v>31.15</v>
-      </c>
-      <c r="F217" s="76">
-        <f>(D217-E217)/D217</f>
-        <v/>
-      </c>
-      <c r="G217" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #531 / 25-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" s="74" t="n">
-        <v>196</v>
-      </c>
-      <c r="B218" s="74" t="inlineStr">
-        <is>
-          <t>I.V. Set (RON)</t>
-        </is>
-      </c>
-      <c r="C218" s="74" t="inlineStr">
-        <is>
-          <t>IV Consumable</t>
-        </is>
-      </c>
-      <c r="D218" s="74" t="n">
-        <v>201</v>
-      </c>
-      <c r="E218" s="74" t="n">
-        <v>14.06</v>
-      </c>
-      <c r="F218" s="76">
-        <f>(D218-E218)/D218</f>
-        <v/>
-      </c>
-      <c r="G218" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #531 / 25-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" s="74" t="n">
-        <v>197</v>
-      </c>
-      <c r="B219" s="74" t="inlineStr">
-        <is>
-          <t>Micro Drip Set (RN)</t>
-        </is>
-      </c>
-      <c r="C219" s="74" t="inlineStr">
-        <is>
-          <t>IV Consumable</t>
-        </is>
-      </c>
-      <c r="D219" s="74" t="n">
-        <v>180</v>
-      </c>
-      <c r="E219" s="74" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="F219" s="76">
-        <f>(D219-E219)/D219</f>
-        <v/>
-      </c>
-      <c r="G219" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #531 / 25-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" s="74" t="n">
-        <v>198</v>
-      </c>
-      <c r="B220" s="74" t="inlineStr">
-        <is>
-          <t>Kaltex Examination Gloves (100s)</t>
-        </is>
-      </c>
-      <c r="C220" s="74" t="inlineStr">
-        <is>
-          <t>OT Consumable — Gloves</t>
-        </is>
-      </c>
-      <c r="D220" s="74" t="n">
-        <v>2344</v>
-      </c>
-      <c r="E220" s="74" t="n">
-        <v>305.5</v>
-      </c>
-      <c r="F220" s="76">
-        <f>(D220-E220)/D220</f>
-        <v/>
-      </c>
-      <c r="G220" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #533 / 26-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" s="74" t="n">
-        <v>199</v>
-      </c>
-      <c r="B221" s="74" t="inlineStr">
-        <is>
-          <t>Face Mask 3PLY (ASPAI)</t>
-        </is>
-      </c>
-      <c r="C221" s="74" t="inlineStr">
-        <is>
-          <t>PPE / Protective</t>
-        </is>
-      </c>
-      <c r="D221" s="74" t="n">
-        <v>1500</v>
-      </c>
-      <c r="E221" s="74" t="n">
-        <v>140</v>
-      </c>
-      <c r="F221" s="76">
-        <f>(D221-E221)/D221</f>
-        <v/>
-      </c>
-      <c r="G221" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #545 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" s="74" t="n">
-        <v>200</v>
-      </c>
-      <c r="B222" s="74" t="inlineStr">
-        <is>
-          <t>Surgical Blade #10 (G) 100s</t>
-        </is>
-      </c>
-      <c r="C222" s="74" t="inlineStr">
-        <is>
-          <t>Surgical Instrument</t>
-        </is>
-      </c>
-      <c r="D222" s="74" t="n">
-        <v>650</v>
-      </c>
-      <c r="E222" s="74" t="n">
-        <v>350</v>
-      </c>
-      <c r="F222" s="76">
-        <f>(D222-E222)/D222</f>
-        <v/>
-      </c>
-      <c r="G222" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #545 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" s="74" t="n">
-        <v>201</v>
-      </c>
-      <c r="B223" s="74" t="inlineStr">
-        <is>
-          <t>Dispovan 5ML Syringe (ROMOJE)</t>
-        </is>
-      </c>
-      <c r="C223" s="74" t="inlineStr">
-        <is>
-          <t>Syringe &amp; Needle</t>
-        </is>
-      </c>
-      <c r="D223" s="74" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="E223" s="74" t="n">
-        <v>2.98</v>
-      </c>
-      <c r="F223" s="76">
-        <f>(D223-E223)/D223</f>
-        <v/>
-      </c>
-      <c r="G223" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #545 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" s="74" t="n">
-        <v>202</v>
-      </c>
-      <c r="B224" s="74" t="inlineStr">
-        <is>
-          <t>All Silicon Foley 14Fr (RM)</t>
-        </is>
-      </c>
-      <c r="C224" s="74" t="inlineStr">
-        <is>
-          <t>Urological Consumable</t>
-        </is>
-      </c>
-      <c r="D224" s="74" t="n">
-        <v>824</v>
-      </c>
-      <c r="E224" s="74" t="n">
-        <v>165</v>
-      </c>
-      <c r="F224" s="76">
-        <f>(D224-E224)/D224</f>
-        <v/>
-      </c>
-      <c r="G224" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #545 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" s="74" t="n">
-        <v>203</v>
-      </c>
-      <c r="B225" s="74" t="inlineStr">
-        <is>
-          <t>Lox 2% Jelly (Lignocaine)</t>
-        </is>
-      </c>
-      <c r="C225" s="74" t="inlineStr">
-        <is>
-          <t>Anaesthesia Consumable</t>
-        </is>
-      </c>
-      <c r="D225" s="74" t="n">
-        <v>34.58</v>
-      </c>
-      <c r="E225" s="74" t="n">
-        <v>27</v>
-      </c>
-      <c r="F225" s="76">
-        <f>(D225-E225)/D225</f>
-        <v/>
-      </c>
-      <c r="G225" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #545 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" s="74" t="n">
-        <v>204</v>
-      </c>
-      <c r="B226" s="74" t="inlineStr">
-        <is>
-          <t>NS 1000ML FFS (CARTE)</t>
-        </is>
-      </c>
-      <c r="C226" s="74" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D226" s="74" t="n">
-        <v>62.65</v>
-      </c>
-      <c r="E226" s="74" t="n">
-        <v>36.53</v>
-      </c>
-      <c r="F226" s="76">
-        <f>(D226-E226)/D226</f>
-        <v/>
-      </c>
-      <c r="G226" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #545 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" s="74" t="n">
-        <v>205</v>
-      </c>
-      <c r="B227" s="74" t="inlineStr">
-        <is>
-          <t>Moncef 1GM INJ (Cefoperazone)</t>
-        </is>
-      </c>
-      <c r="C227" s="74" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D227" s="74" t="n">
-        <v>67.05</v>
-      </c>
-      <c r="E227" s="74" t="n">
-        <v>27.71</v>
-      </c>
-      <c r="F227" s="76">
-        <f>(D227-E227)/D227</f>
-        <v/>
-      </c>
-      <c r="G227" s="74" t="inlineStr">
-        <is>
-          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" s="74" t="n">
-        <v>206</v>
-      </c>
-      <c r="B228" s="74" t="inlineStr">
-        <is>
-          <t>Vanking 500MG INJ (Vancomycin)</t>
-        </is>
-      </c>
-      <c r="C228" s="74" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D228" s="74" t="n">
-        <v>539</v>
-      </c>
-      <c r="E228" s="74" t="n">
-        <v>76.40000000000001</v>
-      </c>
-      <c r="F228" s="76">
-        <f>(D228-E228)/D228</f>
-        <v/>
-      </c>
-      <c r="G228" s="74" t="inlineStr">
-        <is>
-          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" s="74" t="n">
-        <v>207</v>
-      </c>
-      <c r="B229" s="74" t="inlineStr">
-        <is>
-          <t>Artacil 50MG INJ</t>
-        </is>
-      </c>
-      <c r="C229" s="74" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D229" s="74" t="n">
-        <v>90.59999999999999</v>
-      </c>
-      <c r="E229" s="74" t="n">
-        <v>55</v>
-      </c>
-      <c r="F229" s="76">
-        <f>(D229-E229)/D229</f>
-        <v/>
-      </c>
-      <c r="G229" s="74" t="inlineStr">
-        <is>
-          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="230">
-      <c r="A230" s="74" t="n">
-        <v>208</v>
-      </c>
-      <c r="B230" s="74" t="inlineStr">
-        <is>
-          <t>Neovec 10MG Vial</t>
-        </is>
-      </c>
-      <c r="C230" s="74" t="inlineStr">
-        <is>
-          <t>Injection — Antiemetic</t>
-        </is>
-      </c>
-      <c r="D230" s="74" t="n">
-        <v>125.65</v>
-      </c>
-      <c r="E230" s="74" t="n">
-        <v>87</v>
-      </c>
-      <c r="F230" s="76">
-        <f>(D230-E230)/D230</f>
-        <v/>
-      </c>
-      <c r="G230" s="74" t="inlineStr">
-        <is>
-          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="231">
-      <c r="A231" s="74" t="n">
-        <v>209</v>
-      </c>
-      <c r="B231" s="74" t="inlineStr">
-        <is>
-          <t>Neovec 4MG INJ</t>
-        </is>
-      </c>
-      <c r="C231" s="74" t="inlineStr">
-        <is>
-          <t>Injection — Antiemetic</t>
-        </is>
-      </c>
-      <c r="D231" s="74" t="n">
-        <v>78</v>
-      </c>
-      <c r="E231" s="74" t="n">
-        <v>44</v>
-      </c>
-      <c r="F231" s="76">
-        <f>(D231-E231)/D231</f>
-        <v/>
-      </c>
-      <c r="G231" s="74" t="inlineStr">
-        <is>
-          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="232">
-      <c r="A232" s="74" t="n">
-        <v>210</v>
-      </c>
-      <c r="B232" s="74" t="inlineStr">
-        <is>
-          <t>Teicobiotic-400 INJ (Teicoplanin)</t>
-        </is>
-      </c>
-      <c r="C232" s="74" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D232" s="74" t="n">
-        <v>3341</v>
-      </c>
-      <c r="E232" s="74" t="n">
-        <v>488</v>
-      </c>
-      <c r="F232" s="76">
-        <f>(D232-E232)/D232</f>
-        <v/>
-      </c>
-      <c r="G232" s="74" t="inlineStr">
-        <is>
-          <t>M.R. Pharma MR001168 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="233">
-      <c r="A233" s="74" t="n">
-        <v>211</v>
-      </c>
-      <c r="B233" s="74" t="inlineStr">
-        <is>
-          <t>Ugaxis-F Tab 1x10</t>
-        </is>
-      </c>
-      <c r="C233" s="74" t="inlineStr">
-        <is>
-          <t>Tablet — Urology</t>
-        </is>
-      </c>
-      <c r="D233" s="74" t="n">
-        <v>450</v>
-      </c>
-      <c r="E233" s="74" t="n">
-        <v>308.57</v>
-      </c>
-      <c r="F233" s="76">
-        <f>(D233-E233)/D233</f>
-        <v/>
-      </c>
-      <c r="G233" s="74" t="inlineStr">
-        <is>
-          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="234">
-      <c r="A234" s="74" t="n">
-        <v>212</v>
-      </c>
-      <c r="B234" s="74" t="inlineStr">
-        <is>
-          <t>Nefsafe Tab 1x10</t>
-        </is>
-      </c>
-      <c r="C234" s="74" t="inlineStr">
-        <is>
-          <t>Tablet — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D234" s="74" t="n">
-        <v>180</v>
-      </c>
-      <c r="E234" s="74" t="n">
-        <v>123.43</v>
-      </c>
-      <c r="F234" s="76">
-        <f>(D234-E234)/D234</f>
-        <v/>
-      </c>
-      <c r="G234" s="74" t="inlineStr">
-        <is>
-          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="235">
-      <c r="A235" s="74" t="n">
-        <v>213</v>
-      </c>
-      <c r="B235" s="74" t="inlineStr">
-        <is>
-          <t>KB5 Syrup 200ML</t>
-        </is>
-      </c>
-      <c r="C235" s="74" t="inlineStr">
-        <is>
-          <t>Syrup</t>
-        </is>
-      </c>
-      <c r="D235" s="74" t="n">
-        <v>242</v>
-      </c>
-      <c r="E235" s="74" t="n">
-        <v>165.94</v>
-      </c>
-      <c r="F235" s="76">
-        <f>(D235-E235)/D235</f>
-        <v/>
-      </c>
-      <c r="G235" s="74" t="inlineStr">
-        <is>
-          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="236">
-      <c r="A236" s="74" t="n">
-        <v>214</v>
-      </c>
-      <c r="B236" s="74" t="inlineStr">
-        <is>
-          <t>Siluts 8ME Tab 1x10</t>
-        </is>
-      </c>
-      <c r="C236" s="74" t="inlineStr">
-        <is>
-          <t>Tablet</t>
-        </is>
-      </c>
-      <c r="D236" s="74" t="n">
-        <v>315</v>
-      </c>
-      <c r="E236" s="74" t="n">
-        <v>216</v>
-      </c>
-      <c r="F236" s="76">
-        <f>(D236-E236)/D236</f>
-        <v/>
-      </c>
-      <c r="G236" s="74" t="inlineStr">
-        <is>
-          <t>Chirag Enterprises MP-38 / 29-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" s="74" t="n">
-        <v>215</v>
-      </c>
-      <c r="B237" s="74" t="inlineStr">
-        <is>
-          <t>SS Tube-16 (Suction Tube)</t>
-        </is>
-      </c>
-      <c r="C237" s="74" t="inlineStr">
-        <is>
-          <t>OT Consumable — Suction</t>
-        </is>
-      </c>
-      <c r="D237" s="74" t="n">
-        <v>79.58</v>
-      </c>
-      <c r="E237" s="74" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="F237" s="76">
-        <f>(D237-E237)/D237</f>
-        <v/>
-      </c>
-      <c r="G237" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #548 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" s="74" t="n">
-        <v>216</v>
-      </c>
-      <c r="B238" s="74" t="inlineStr">
-        <is>
-          <t>Surgicare-6.0 Suture</t>
-        </is>
-      </c>
-      <c r="C238" s="74" t="inlineStr">
-        <is>
-          <t>Suture</t>
-        </is>
-      </c>
-      <c r="D238" s="74" t="n">
-        <v>91</v>
-      </c>
-      <c r="E238" s="74" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="F238" s="76">
-        <f>(D238-E238)/D238</f>
-        <v/>
-      </c>
-      <c r="G238" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #548 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="239">
-      <c r="A239" s="74" t="n">
-        <v>217</v>
-      </c>
-      <c r="B239" s="74" t="inlineStr">
-        <is>
-          <t>Genellium Pro (Large)</t>
-        </is>
-      </c>
-      <c r="C239" s="74" t="inlineStr">
-        <is>
-          <t>OT Consumable — Haemostat</t>
-        </is>
-      </c>
-      <c r="D239" s="74" t="n">
-        <v>3200</v>
-      </c>
-      <c r="E239" s="74" t="n">
-        <v>2250</v>
-      </c>
-      <c r="F239" s="76">
-        <f>(D239-E239)/D239</f>
-        <v/>
-      </c>
-      <c r="G239" s="74" t="inlineStr">
-        <is>
-          <t>B.P. Pharma #548 / 31-Aug-26</t>
-        </is>
-      </c>
-    </row>
-    <row r="240">
-      <c r="A240" s="72" t="inlineStr">
+      <c r="A216" s="72" t="inlineStr">
         <is>
           <t>🔴 ITEMS MISSING MRP — Collect from vendor and update above</t>
         </is>
       </c>
-      <c r="B240" s="42" t="n"/>
-      <c r="C240" s="42" t="n"/>
-      <c r="D240" s="42" t="n"/>
-      <c r="E240" s="42" t="n"/>
-      <c r="F240" s="42" t="n"/>
-      <c r="G240" s="42" t="n"/>
-    </row>
-    <row r="241">
-      <c r="A241" s="48" t="n">
-        <v>1</v>
-      </c>
-      <c r="B241" s="73" t="inlineStr">
-        <is>
-          <t>NS 100ml — Normal Saline 100ml</t>
-        </is>
-      </c>
-      <c r="C241" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D241" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E241" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F241" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G241" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="242">
-      <c r="A242" s="48" t="n">
-        <v>2</v>
-      </c>
-      <c r="B242" s="73" t="inlineStr">
-        <is>
-          <t>D5 500ml — Dextrose 5%</t>
-        </is>
-      </c>
-      <c r="C242" s="46" t="inlineStr">
-        <is>
-          <t>IV Fluid</t>
-        </is>
-      </c>
-      <c r="D242" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E242" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F242" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G242" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="243">
-      <c r="A243" s="48" t="n">
-        <v>3</v>
-      </c>
-      <c r="B243" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Anawin 0.25% / Sensoricaine 5%/25%</t>
-        </is>
-      </c>
-      <c r="C243" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Anaesthesia</t>
-        </is>
-      </c>
-      <c r="D243" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E243" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F243" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G243" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="244">
-      <c r="A244" s="48" t="n">
-        <v>4</v>
-      </c>
-      <c r="B244" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Gentamicin</t>
-        </is>
-      </c>
-      <c r="C244" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D244" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E244" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F244" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G244" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="245">
-      <c r="A245" s="48" t="n">
-        <v>5</v>
-      </c>
-      <c r="B245" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Tramadol 50mg</t>
-        </is>
-      </c>
-      <c r="C245" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Analgesic</t>
-        </is>
-      </c>
-      <c r="D245" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E245" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F245" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G245" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="246">
-      <c r="A246" s="48" t="n">
-        <v>6</v>
-      </c>
-      <c r="B246" s="73" t="inlineStr">
-        <is>
-          <t>Inj. PCM 100ml (Paracetamol IV)</t>
-        </is>
-      </c>
-      <c r="C246" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Analgesic</t>
-        </is>
-      </c>
-      <c r="D246" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E246" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F246" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G246" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" s="48" t="n">
-        <v>7</v>
-      </c>
-      <c r="B247" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Carboprost (Hemabate)</t>
-        </is>
-      </c>
-      <c r="C247" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Oxytocic</t>
-        </is>
-      </c>
-      <c r="D247" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E247" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F247" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G247" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" s="48" t="n">
-        <v>8</v>
-      </c>
-      <c r="B248" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Adrenaline</t>
-        </is>
-      </c>
-      <c r="C248" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Emergency</t>
-        </is>
-      </c>
-      <c r="D248" s="47" t="n">
-        <v>13.4</v>
-      </c>
-      <c r="E248" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F248" s="47" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G248" s="47" t="inlineStr">
-        <is>
-          <t>Stock OT/Ward: ADRENALIN 1ML</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" s="48" t="n">
-        <v>9</v>
-      </c>
-      <c r="B249" s="73" t="inlineStr">
-        <is>
-          <t>Inj. Cetil (Cefuroxime Axetil)</t>
-        </is>
-      </c>
-      <c r="C249" s="46" t="inlineStr">
-        <is>
-          <t>Injection — Antibiotic</t>
-        </is>
-      </c>
-      <c r="D249" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E249" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F249" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G249" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" s="48" t="n">
-        <v>10</v>
-      </c>
-      <c r="B250" s="73" t="inlineStr">
-        <is>
-          <t>Needles 26G (Injection)</t>
-        </is>
-      </c>
-      <c r="C250" s="46" t="inlineStr">
-        <is>
-          <t>Consumable</t>
-        </is>
-      </c>
-      <c r="D250" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E250" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F250" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G250" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" s="48" t="n">
-        <v>11</v>
-      </c>
-      <c r="B251" s="73" t="inlineStr">
-        <is>
-          <t>Disposable Gloves (Exam)</t>
-        </is>
-      </c>
-      <c r="C251" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D251" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E251" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F251" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G251" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" s="48" t="n">
-        <v>12</v>
-      </c>
-      <c r="B252" s="73" t="inlineStr">
-        <is>
-          <t>Betadine Ointment 40g</t>
-        </is>
-      </c>
-      <c r="C252" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D252" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E252" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F252" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G252" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" s="48" t="n">
-        <v>13</v>
-      </c>
-      <c r="B253" s="73" t="inlineStr">
-        <is>
-          <t>Surgical Blade No. 10</t>
-        </is>
-      </c>
-      <c r="C253" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D253" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E253" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F253" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G253" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" s="48" t="n">
-        <v>14</v>
-      </c>
-      <c r="B254" s="73" t="inlineStr">
-        <is>
-          <t>Surgical Blade No. 20</t>
-        </is>
-      </c>
-      <c r="C254" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D254" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E254" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F254" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G254" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" s="48" t="n">
-        <v>15</v>
-      </c>
-      <c r="B255" s="73" t="inlineStr">
-        <is>
-          <t>Plain Sheet (OT Draping)</t>
-        </is>
-      </c>
-      <c r="C255" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D255" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E255" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F255" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G255" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" s="48" t="n">
-        <v>16</v>
-      </c>
-      <c r="B256" s="73" t="inlineStr">
-        <is>
-          <t>Soft Roll (OT Padding)</t>
-        </is>
-      </c>
-      <c r="C256" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D256" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E256" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F256" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G256" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" s="48" t="n">
-        <v>17</v>
-      </c>
-      <c r="B257" s="73" t="inlineStr">
-        <is>
-          <t>Gypsona POP Bandage 40G</t>
-        </is>
-      </c>
-      <c r="C257" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D257" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E257" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F257" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G257" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" s="48" t="n">
-        <v>18</v>
-      </c>
-      <c r="B258" s="73" t="inlineStr">
-        <is>
-          <t>Cap + Mask (Disposable Set)</t>
-        </is>
-      </c>
-      <c r="C258" s="46" t="inlineStr">
-        <is>
-          <t>Surgical Consumable</t>
-        </is>
-      </c>
-      <c r="D258" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E258" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F258" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G258" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" s="48" t="n">
-        <v>19</v>
-      </c>
-      <c r="B259" s="73" t="inlineStr">
-        <is>
-          <t>Glucostrip (Blood Glucose)</t>
-        </is>
-      </c>
-      <c r="C259" s="46" t="inlineStr">
-        <is>
-          <t>Investigation</t>
-        </is>
-      </c>
-      <c r="D259" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E259" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F259" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G259" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" s="48" t="n">
-        <v>20</v>
-      </c>
-      <c r="B260" s="73" t="inlineStr">
-        <is>
-          <t>Lancet Needle</t>
-        </is>
-      </c>
-      <c r="C260" s="46" t="inlineStr">
-        <is>
-          <t>Investigation</t>
-        </is>
-      </c>
-      <c r="D260" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E260" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F260" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G260" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" s="48" t="n">
-        <v>21</v>
-      </c>
-      <c r="B261" s="73" t="inlineStr">
-        <is>
-          <t>Red Top Tube (Blood Vial)</t>
-        </is>
-      </c>
-      <c r="C261" s="46" t="inlineStr">
-        <is>
-          <t>Investigation</t>
-        </is>
-      </c>
-      <c r="D261" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E261" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F261" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G261" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" s="48" t="n">
-        <v>22</v>
-      </c>
-      <c r="B262" s="73" t="inlineStr">
-        <is>
-          <t>CBC Vial Yellow + Red Top</t>
-        </is>
-      </c>
-      <c r="C262" s="46" t="inlineStr">
-        <is>
-          <t>Investigation</t>
-        </is>
-      </c>
-      <c r="D262" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E262" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F262" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G262" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" s="48" t="n">
-        <v>23</v>
-      </c>
-      <c r="B263" s="73" t="inlineStr">
-        <is>
-          <t>O2 / Oxygen (per use)</t>
-        </is>
-      </c>
-      <c r="C263" s="46" t="inlineStr">
-        <is>
-          <t>Equipment</t>
-        </is>
-      </c>
-      <c r="D263" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E263" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F263" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G263" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" s="48" t="n">
-        <v>24</v>
-      </c>
-      <c r="B264" s="73" t="inlineStr">
-        <is>
-          <t>Pulse Oximeter (per use)</t>
-        </is>
-      </c>
-      <c r="C264" s="46" t="inlineStr">
-        <is>
-          <t>Equipment</t>
-        </is>
-      </c>
-      <c r="D264" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E264" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F264" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G264" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" s="48" t="n">
-        <v>25</v>
-      </c>
-      <c r="B265" s="73" t="inlineStr">
-        <is>
-          <t>Cardiac Monitor (per use)</t>
-        </is>
-      </c>
-      <c r="C265" s="46" t="inlineStr">
-        <is>
-          <t>Equipment</t>
-        </is>
-      </c>
-      <c r="D265" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E265" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F265" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G265" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" s="48" t="n">
-        <v>26</v>
-      </c>
-      <c r="B266" s="73" t="inlineStr">
-        <is>
-          <t>C-arm (per use)</t>
-        </is>
-      </c>
-      <c r="C266" s="46" t="inlineStr">
-        <is>
-          <t>Equipment</t>
-        </is>
-      </c>
-      <c r="D266" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E266" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F266" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G266" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" s="48" t="n">
-        <v>27</v>
-      </c>
-      <c r="B267" s="73" t="inlineStr">
-        <is>
-          <t>Volu-P / TiCUP</t>
-        </is>
-      </c>
-      <c r="C267" s="46" t="inlineStr">
-        <is>
-          <t>Consumable</t>
-        </is>
-      </c>
-      <c r="D267" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="E267" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="F267" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
-      <c r="G267" s="47" t="inlineStr">
-        <is>
-          <t>⚠ FILL IN</t>
-        </is>
-      </c>
+      <c r="B216" s="42" t="n"/>
+      <c r="C216" s="42" t="n"/>
+      <c r="D216" s="42" t="n"/>
+      <c r="E216" s="42" t="n"/>
+      <c r="F216" s="42" t="n"/>
+      <c r="G216" s="42" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="21">

</xml_diff>